<commit_message>
Plan: 9.12 split into 9.12a-d (per-user IP, guest LAN, BORDER, inside DHCP/DNS); 9.2 progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G81"/>
+  <dimension ref="A3:G85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -450,7 +450,6 @@
     <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -2012,18 +2011,22 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>I-235 (models), I-201 (DMKDMP dump), LPSW fast path above 16 MB</t>
+          <t>I-235 (models), I-201 (DMKDMP dump), warm start (I-267, I-268), LPSW fast path above 16 MB, per-user IP (9.12a)</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Next</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>After M4b.3</t>
+          <t>I-201, I-267, I-268 done: dump, SHUTDOWN and warm start work</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2321,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Network pack: BORDER firewall guest</t>
+          <t>Network pack: per-user addresses, CP guest LAN, BORDER firewall, inside DHCP/DNS (9.12a-d)</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2334,29 +2337,57 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
-      <c r="B65" s="10" t="n"/>
-      <c r="C65" s="2" t="n"/>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="5" t="n"/>
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>9.12a</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Addresses</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Per-user IP address at disk IPL from the directory (fixes I-266)</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
       <c r="F65" s="2" t="n"/>
-      <c r="G65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Done with 9.2</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B66" s="10" t="n"/>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>9.12b</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Guest LAN</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>z/Architecture (64-bit)</t>
+          <t>CP virtual NIC per guest on one internal segment (LCS/QETH style, like z/VM Guest LAN)</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2365,205 +2396,193 @@
         </is>
       </c>
       <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Needed for DHCP: CTC links are point-to-point</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.12c</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D67" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="n"/>
+          <t>Firewall</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>BORDER service machine: only outside link; NAT outbound; port forwards to service machines (httpd 9.5)</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Outside link may be bridged (LCS on tap) to get its address from the LAN DHCP</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.12d</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="n"/>
+          <t>DHCP/DNS</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>DHCP and DNS for the inside segment as a service machine (dnsmasq on Debian, or in BORDER)</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F68" s="2" t="n"/>
-      <c r="G68" s="2" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Needs 9.12b</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>10.3</t>
-        </is>
-      </c>
-      <c r="C69" s="14" t="inlineStr">
-        <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="inlineStr">
-        <is>
-          <t>Kit 8</t>
-        </is>
-      </c>
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="10" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
       <c r="E69" s="5" t="n"/>
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="14" t="n"/>
-      <c r="B70" s="13" t="n"/>
-      <c r="C70" s="14" t="n"/>
-      <c r="D70" s="14" t="n"/>
-      <c r="E70" s="5" t="n"/>
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="n"/>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E71" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="n"/>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E72" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
+          <t>Snapshot</t>
         </is>
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>FreeSWITCH</t>
-        </is>
-      </c>
-      <c r="E73" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Kit 8</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="n"/>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D74" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
-        </is>
-      </c>
-      <c r="E74" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A74" s="14" t="n"/>
+      <c r="B74" s="13" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="14" t="n"/>
+      <c r="E74" s="5" t="n"/>
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
     </row>
@@ -2575,17 +2594,17 @@
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
-        </is>
-      </c>
-      <c r="D75" s="14" t="inlineStr">
-        <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
@@ -2604,17 +2623,17 @@
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="D76" s="14" t="inlineStr">
-        <is>
-          <t>CFSERV</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr">
@@ -2633,20 +2652,24 @@
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C77" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="n"/>
+          <t>FreeSWITCH</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
     </row>
@@ -2658,37 +2681,149 @@
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="n"/>
+          <t>Node-RED</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="n"/>
-      <c r="B79" s="11" t="n"/>
-      <c r="C79" s="8" t="n"/>
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>Container</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="n"/>
-      <c r="B80" s="11" t="n"/>
-      <c r="C80" s="8" t="n"/>
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="7" t="n"/>
-      <c r="B81" s="12" t="n"/>
-      <c r="C81" s="7" t="n"/>
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="n"/>
+      <c r="B83" s="11" t="n"/>
+      <c r="C83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n"/>
+      <c r="B84" s="11" t="n"/>
+      <c r="C84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="n"/>
+      <c r="B85" s="12" t="n"/>
+      <c r="C85" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
Plan: 9.12a done, 9.2 progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2026,7 +2026,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>I-201, I-267, I-268 done: dump, SHUTDOWN and warm start work</t>
+          <t>Done: I-201, I-267, I-268, I-269 (dump, SHUTDOWN, warm start, CTC attach). Open: LPSW fast path, I-235, I-265</t>
         </is>
       </c>
     </row>
@@ -2359,13 +2359,17 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Next</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Done with 9.2</t>
+          <t>Address follows the CTC pair (62x/63x or real); vm370plus-net on both Debian disks; verified 10.1.2.2 by itself</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan: 9.13 public tools (Pascal, NJE, UnixNJE, NICOF, game disk, workshop tools), 9.14 TELL everywhere
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G85"/>
+  <dimension ref="A3:G93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2473,29 +2473,57 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="10" t="n"/>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="5" t="n"/>
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>9.13</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Public VM/370 tools for the kit (survey 11 Oct)</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F69" s="2" t="n"/>
-      <c r="G69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Before kit 7 (9.11)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B70" s="10" t="n"/>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>9.13a</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Pascal</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>z/Architecture (64-bit)</t>
+          <t>New Stanford Pascal (Oppolzer, github StanfordPascal/Pascal) replaces CE 2021.03</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -2509,198 +2537,226 @@
     <row r="71">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.13b</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D71" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="n"/>
+          <t>NJE</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>RSCS NJE updates (Coghlan) + TCPNJE: VM/370 NJE to MVS/z/OS/Linux</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F71" s="2" t="n"/>
-      <c r="G71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.13c</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D72" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="n"/>
+          <t>NJE Linux</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>UnixNJE (FUNET-NJE) in the Debian guest: CMS &lt;-&gt; Linux NJE</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F72" s="2" t="n"/>
-      <c r="G72" s="2" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Needs 9.13b</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.13d</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D73" s="14" t="inlineStr">
-        <is>
-          <t>Kit 8</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="n"/>
+          <t>Sockets</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>NICOF + CMSFTPD (devhawala, public domain): sockets API and FTP for CMS</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F73" s="2" t="n"/>
-      <c r="G73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Test before 9.5 (CMS sockets + httpd)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="n"/>
-      <c r="B74" s="13" t="n"/>
-      <c r="C74" s="14" t="n"/>
-      <c r="D74" s="14" t="n"/>
-      <c r="E74" s="5" t="n"/>
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>9.13e</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Game disk: VM/370 games tape (IBM VS BASIC runtime removed), WIOS SNAKE/SLASH, CALL-OS BASIC TREK2, Zork/Dungeon</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>9.13f</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E75" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>VM Workshop 1985/86 tools that run on R6: CARD, FCOPY, CLUST/TERM macros; check DISKPRY, LEDIT, IEBCOPY, JSCAN</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="F75" s="2" t="n"/>
-      <c r="G75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>CPWATCH (85 M0083) is 4c</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>9.14</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>TELL</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E76" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>TELL everywhere: CMS TELL EXEC (CP MSG local, RSCS/NJE remote), Linux tell (vmcp, kernel CONFIG_VMCP) with incoming MSG captured, PC client through BORDER (CHATBOT-style gateway)</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="F76" s="2" t="n"/>
-      <c r="G76" s="2" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B77" s="13" t="inlineStr">
-        <is>
-          <t>11.3</t>
-        </is>
-      </c>
-      <c r="C77" s="14" t="inlineStr">
-        <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
-        </is>
-      </c>
-      <c r="E77" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="10" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="5" t="n"/>
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="C78" s="14" t="inlineStr">
-        <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D78" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
-        </is>
-      </c>
-      <c r="E78" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="n"/>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="F78" s="2" t="n"/>
@@ -2709,80 +2765,72 @@
     <row r="79">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
-        </is>
-      </c>
-      <c r="E79" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="n"/>
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
-        </is>
-      </c>
-      <c r="E80" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="n"/>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Snapshot</t>
         </is>
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Kit 8</t>
         </is>
       </c>
       <c r="E81" s="5" t="n"/>
@@ -2790,44 +2838,252 @@
       <c r="G81" s="2" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B82" s="13" t="inlineStr">
-        <is>
-          <t>11.8</t>
-        </is>
-      </c>
-      <c r="C82" s="14" t="inlineStr">
-        <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D82" s="14" t="inlineStr">
-        <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
+      <c r="A82" s="14" t="n"/>
+      <c r="B82" s="13" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="14" t="n"/>
       <c r="E82" s="5" t="n"/>
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="n"/>
-      <c r="B83" s="11" t="n"/>
-      <c r="C83" s="8" t="n"/>
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="n"/>
-      <c r="B84" s="11" t="n"/>
-      <c r="C84" s="8" t="n"/>
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="7" t="n"/>
-      <c r="B85" s="12" t="n"/>
-      <c r="C85" s="7" t="n"/>
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>VoIP</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>FreeSWITCH</t>
+        </is>
+      </c>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>IoT</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>Node-RED</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>Container</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B88" s="13" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="n"/>
+      <c r="F89" s="2" t="n"/>
+      <c r="G89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="n"/>
+      <c r="B91" s="11" t="n"/>
+      <c r="C91" s="8" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="n"/>
+      <c r="B92" s="11" t="n"/>
+      <c r="C92" s="8" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="n"/>
+      <c r="B93" s="12" t="n"/>
+      <c r="C93" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
I-265 fixed (DMKVSP page-crossing spool move kept the CCW op code in AMODE 31: LINUX READER boots again); TDISK EXEC + HELP (owner request); plan 9.15 Python, 9.16 TDISK; guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G93"/>
+  <dimension ref="A3:G95"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2729,60 +2729,80 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n"/>
-      <c r="B77" s="10" t="n"/>
-      <c r="C77" s="2" t="n"/>
-      <c r="D77" s="2" t="n"/>
-      <c r="E77" s="5" t="n"/>
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>9.15</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Python on CMS: the C89 implementation from mikebeer/python (in creation), built with GCC for CMS; Debian uses standard wheezy python 2.7/3.2 packages</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F77" s="2" t="n"/>
-      <c r="G77" s="2" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B78" s="10" t="n"/>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>9.16</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>TDISK</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>z/Architecture (64-bit)</t>
+          <t>TDISK EXEC: TDISK [cyls] [fm] defines, formats and (with fm) accesses a temporary disk; HELP TDISK</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="n"/>
-      <c r="G78" s="2" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C79" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D79" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="10" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
       <c r="E79" s="5" t="n"/>
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
@@ -2793,22 +2813,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B80" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C80" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D80" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="n"/>
+      <c r="B80" s="10" t="n"/>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
     </row>
@@ -2820,17 +2840,17 @@
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E81" s="5" t="n"/>
@@ -2838,10 +2858,26 @@
       <c r="G81" s="2" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="14" t="n"/>
-      <c r="B82" s="13" t="n"/>
-      <c r="C82" s="14" t="n"/>
-      <c r="D82" s="14" t="n"/>
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
       <c r="E82" s="5" t="n"/>
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
@@ -2849,58 +2885,34 @@
     <row r="83">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E83" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="n"/>
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B84" s="13" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="C84" s="14" t="inlineStr">
-        <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E84" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A84" s="14" t="n"/>
+      <c r="B84" s="13" t="n"/>
+      <c r="C84" s="14" t="n"/>
+      <c r="D84" s="14" t="n"/>
+      <c r="E84" s="5" t="n"/>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
     </row>
@@ -2912,17 +2924,17 @@
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C85" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D85" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
@@ -2941,17 +2953,17 @@
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D86" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E86" s="16" t="inlineStr">
@@ -2970,17 +2982,17 @@
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C87" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
@@ -2999,17 +3011,17 @@
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E88" s="16" t="inlineStr">
@@ -3028,20 +3040,24 @@
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C89" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="n"/>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
     </row>
@@ -3053,37 +3069,91 @@
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="n"/>
-      <c r="B91" s="11" t="n"/>
-      <c r="C91" s="8" t="n"/>
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B91" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="n"/>
-      <c r="B92" s="11" t="n"/>
-      <c r="C92" s="8" t="n"/>
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B92" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="n"/>
+      <c r="F92" s="2" t="n"/>
+      <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="7" t="n"/>
-      <c r="B93" s="12" t="n"/>
-      <c r="C93" s="7" t="n"/>
+      <c r="A93" s="8" t="n"/>
+      <c r="B93" s="11" t="n"/>
+      <c r="C93" s="8" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="n"/>
+      <c r="B94" s="11" t="n"/>
+      <c r="C94" s="8" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="n"/>
+      <c r="B95" s="12" t="n"/>
+      <c r="C95" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.2 done: I-235 model tables kept resident by design; 9.16 TDISK done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Done: I-201, I-267, I-268, I-269 (dump, SHUTDOWN, warm start, CTC attach). Open: LPSW fast path, I-235, I-265</t>
+          <t>I-201, I-265, I-267, I-268, I-269 fixed; LPSW/SVC fast paths; I-235 models kept resident by design (M10 revisits sharer invalidation)</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Plan: 9.10 ASKSERV uses llama.cpp on the PC; 9.17 tiny LLM demo on Debian/390 and CMS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G95"/>
+  <dimension ref="A3:G96"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>AI gateway service machine (ASKSERV)</t>
+          <t>AI gateway service machine (ASKSERV): CMS/Linux/TELL clients; the model runs in llama.cpp on the PC (or a cloud API), reached through BORDER</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2799,36 +2799,44 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n"/>
-      <c r="B79" s="10" t="n"/>
-      <c r="C79" s="2" t="n"/>
-      <c r="D79" s="2" t="n"/>
-      <c r="E79" s="5" t="n"/>
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>9.17</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>Tiny LLM</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>llama2.c-style inference of a tiny model (stories15M) natively on Debian/390 and on CMS (C, high storage, HFP/BFP and byte order converted): a demonstration; real models via 9.10</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F79" s="2" t="n"/>
-      <c r="G79" s="2" t="n"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; llama.cpp itself needs 64-bit, C++17 and GBs</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A80" s="2" t="n"/>
       <c r="B80" s="10" t="n"/>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="5" t="n"/>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
     </row>
@@ -2838,22 +2846,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C81" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D81" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="n"/>
+      <c r="B81" s="10" t="n"/>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
     </row>
@@ -2865,7 +2873,7 @@
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
@@ -2875,7 +2883,7 @@
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E82" s="5" t="n"/>
@@ -2890,17 +2898,17 @@
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E83" s="5" t="n"/>
@@ -2908,40 +2916,36 @@
       <c r="G83" s="2" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="n"/>
-      <c r="B84" s="13" t="n"/>
-      <c r="C84" s="14" t="n"/>
-      <c r="D84" s="14" t="n"/>
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
       <c r="E84" s="5" t="n"/>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B85" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C85" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E85" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A85" s="14" t="n"/>
+      <c r="B85" s="13" t="n"/>
+      <c r="C85" s="14" t="n"/>
+      <c r="D85" s="14" t="n"/>
+      <c r="E85" s="5" t="n"/>
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
     </row>
@@ -2953,17 +2957,17 @@
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E86" s="16" t="inlineStr">
@@ -2982,17 +2986,17 @@
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C87" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D87" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
@@ -3011,17 +3015,17 @@
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E88" s="16" t="inlineStr">
@@ -3040,17 +3044,17 @@
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C89" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
@@ -3069,17 +3073,17 @@
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E90" s="16" t="inlineStr">
@@ -3098,20 +3102,24 @@
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C91" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D91" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="n"/>
     </row>
@@ -3123,17 +3131,17 @@
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E92" s="5" t="n"/>
@@ -3141,9 +3149,29 @@
       <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="n"/>
-      <c r="B93" s="11" t="n"/>
-      <c r="C93" s="8" t="n"/>
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B93" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="n"/>
+      <c r="F93" s="2" t="n"/>
+      <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n"/>
@@ -3151,9 +3179,14 @@
       <c r="C94" s="8" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="7" t="n"/>
-      <c r="B95" s="12" t="n"/>
-      <c r="C95" s="7" t="n"/>
+      <c r="A95" s="8" t="n"/>
+      <c r="B95" s="11" t="n"/>
+      <c r="C95" s="8" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="n"/>
+      <c r="B96" s="12" t="n"/>
+      <c r="C96" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
Plan: M6 split into 6a-6e (6b done), 9.18 MAIL, M12 DOS/VSE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G96"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,8 @@
     <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -1453,7 +1455,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
@@ -1464,177 +1466,165 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="5" t="n"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>FORMAT (BLKSIZE 4096 writes an EDF label, directory and allocation map</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>7.0</t>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>6b</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>ESA/390 guests</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Baseline test guest (STSCH/SSCH/ESA PSW/X'B8')</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
+          <t>EDF disks read: ACCESS, LISTFILE, STATE, TYPE, COPYFILE from (DMSEFS, XA0056DK)</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>7 Oct</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="n"/>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>86699c4; 100,000-record V and 70,000-record F files read</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>7.1</t>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>6c</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>ESA/390 guests</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>SET ESA / machine mode, ESA IPL</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>7 Oct</t>
-        </is>
-      </c>
+          <t>EDF write, erase, rename; files above 65,535 records</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>7.2</t>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>6d</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>ESA/390 guests</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Virtual channel subsystem (DMKVCS)</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>7 Oct</t>
-        </is>
-      </c>
+          <t>Large minidisks (full-volume 3390)</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>7.3</t>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>6e</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>ESA/390 guests</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ESA/390 guest DAT (DMKVAX shadow tables)</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>7 Oct</t>
-        </is>
-      </c>
+          <t>Tools across both formats (DISK DUMP/LOAD, TAPE, MOVEFILE, FULIST)</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
     </row>
     <row r="41" ht="25.5" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>7.4</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>ESA/390 guests</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>What Linux uses besides (secondary space, STAP, SIGP, timers, DIAG 10)</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>7–8 Oct</t>
-        </is>
-      </c>
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
     </row>
     <row r="42">
@@ -1645,7 +1635,7 @@
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1655,7 +1645,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Linux/390 31-bit from the reader, shell on the 3215</t>
+          <t>Baseline test guest (STSCH/SSCH/ESA PSW/X'B8')</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -1665,7 +1655,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>8 Oct</t>
+          <t>7 Oct</t>
         </is>
       </c>
       <c r="G42" s="2" t="n"/>
@@ -1678,7 +1668,7 @@
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1688,7 +1678,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>BusyBox userland, CTC network</t>
+          <t>SET ESA / machine mode, ESA IPL</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -1698,7 +1688,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>8 Oct</t>
+          <t>7 Oct</t>
         </is>
       </c>
       <c r="G43" s="2" t="n"/>
@@ -1711,7 +1701,7 @@
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>7.7</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1721,7 +1711,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Debian 7.11 from a 3390, SSH over CTC</t>
+          <t>Virtual channel subsystem (DMKVCS)</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -1731,7 +1721,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>8–9 Oct</t>
+          <t>7 Oct</t>
         </is>
       </c>
       <c r="G44" s="2" t="n"/>
@@ -1744,7 +1734,7 @@
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>7.8</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1754,7 +1744,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Linux for several users (LINUX EXEC); Linux and CMS side by side</t>
+          <t>ESA/390 guest DAT (DMKVAX shadow tables)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -1764,14 +1754,10 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>9 Oct</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>Two Debians at once: done 11 Oct (M4b.3 step 6)</t>
-        </is>
-      </c>
+          <t>7 Oct</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1781,7 +1767,7 @@
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1791,7 +1777,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Channel programs of any length for ESA/390 guests</t>
+          <t>What Linux uses besides (secondary space, STAP, SIGP, timers, DIAG 10)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -1801,7 +1787,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>10 Oct</t>
+          <t>7–8 Oct</t>
         </is>
       </c>
       <c r="G46" s="2" t="n"/>
@@ -1814,7 +1800,7 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>7.10</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -1824,7 +1810,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>IPL LINUX from its disk (vmzipl)</t>
+          <t>Linux/390 31-bit from the reader, shell on the 3215</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -1834,7 +1820,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>10 Oct</t>
+          <t>8 Oct</t>
         </is>
       </c>
       <c r="G47" s="2" t="n"/>
@@ -1847,7 +1833,7 @@
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>7.11</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1857,7 +1843,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>3390-9 Debian disk (7 GB) as standard</t>
+          <t>BusyBox userland, CTC network</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -1867,39 +1853,63 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>10 Oct</t>
+          <t>8 Oct</t>
         </is>
       </c>
       <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="10" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="2" t="n"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>ESA/390 guests</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Debian 7.11 from a 3390, SSH over CTC</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>8–9 Oct</t>
+        </is>
+      </c>
       <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>cREXX</t>
+          <t>ESA/390 guests</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Current cREXX cross-built for CMS (RXC8, RXAS8, RXBVM8)</t>
+          <t>Linux for several users (LINUX EXEC); Linux and CMS side by side</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -1909,211 +1919,199 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>8 Oct</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="n"/>
+          <t>9 Oct</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Two Debians at once: done 11 Oct (M4b.3 step 6)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>ESA/390 guests</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Channel programs of any length for ESA/390 guests</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>10 Oct</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>7.10</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>ESA/390 guests</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>IPL LINUX from its disk (vmzipl)</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>10 Oct</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n"/>
+    </row>
+    <row r="53" ht="25.5" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>7.11</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>ESA/390 guests</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>3390-9 Debian disk (7 GB) as standard</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>10 Oct</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
           <t>M8</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>cREXX</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Current cREXX cross-built for CMS (RXC8, RXAS8, RXBVM8)</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>8 Oct</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>8.2</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>cREXX</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Current cREXX built natively on CMS</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>9 Oct–</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>RXC/RXAS work; RXBVM82 open</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="10" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="n"/>
-    </row>
-    <row r="53" ht="25.5" customHeight="1">
-      <c r="A53" s="14" t="inlineStr">
-        <is>
-          <t>M9</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>9.1</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Since kit b6</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>SET/QUERY MACHINE, FULIST, GLOBALV, command tables, I-257, I-258</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>10–11 Oct</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="14" t="inlineStr">
-        <is>
-          <t>M9</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>CP leftovers</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>I-235 (models), I-201 (DMKDMP dump), warm start (I-267, I-268), LPSW fast path above 16 MB, per-user IP (9.12a)</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>11 Oct</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>I-201, I-265, I-267, I-268, I-269 fixed; LPSW/SVC fast paths; I-235 models kept resident by design (M10 revisits sharer invalidation)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="14" t="inlineStr">
-        <is>
-          <t>M9</t>
-        </is>
-      </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>9.3</t>
-        </is>
-      </c>
-      <c r="C55" s="14" t="inlineStr">
-        <is>
-          <t>C++</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>C++ on CMS (subset, cross route)</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="2" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>M9</t>
-        </is>
-      </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>9.4</t>
-        </is>
-      </c>
-      <c r="C56" s="14" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>SQL: SQLite on CMS + SQLSERV; MariaDB/PostgreSQL on Debian</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
-    </row>
     <row r="57">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>M9</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>Network</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>CMS sockets + httpd</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="4" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
     </row>
@@ -2125,25 +2123,29 @@
       </c>
       <c r="B58" s="13" t="inlineStr">
         <is>
-          <t>9.6</t>
-        </is>
-      </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>dbase</t>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Since kit b6</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>xBase / Harbour</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="n"/>
+          <t>SET/QUERY MACHINE, FULIST, GLOBALV, command tables, I-257, I-258</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>10–11 Oct</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="n"/>
     </row>
     <row r="59">
@@ -2154,28 +2156,32 @@
       </c>
       <c r="B59" s="13" t="inlineStr">
         <is>
-          <t>9.7</t>
-        </is>
-      </c>
-      <c r="C59" s="14" t="inlineStr">
-        <is>
-          <t>MQ</t>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>CP leftovers</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>MQ and MQTT (CMS and Debian)</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="n"/>
+          <t>I-235 (models), I-201 (DMKDMP dump), warm start (I-267, I-268), LPSW fast path above 16 MB, per-user IP (9.12a)</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>mosquitto on Debian done</t>
+          <t>I-201, I-265, I-267, I-268, I-269 fixed; LPSW/SVC fast paths; I-235 models kept resident by design (M10 revisits sharer invalidation)</t>
         </is>
       </c>
     </row>
@@ -2187,30 +2193,26 @@
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
-          <t>APL</t>
+          <t>C++</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>APL in C on CMS</t>
-        </is>
-      </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>In progress</t>
+          <t>C++ on CMS (subset, cross route)</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>Debian 34/34; CMS run pending</t>
-        </is>
-      </c>
+      <c r="G60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
@@ -2220,17 +2222,17 @@
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
         <is>
-          <t>REXX</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>ooRexx 5 on Debian</t>
+          <t>SQL: SQLite on CMS + SQLSERV; MariaDB/PostgreSQL on Debian</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2249,17 +2251,17 @@
       </c>
       <c r="B62" s="13" t="inlineStr">
         <is>
-          <t>9.10</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>AI gateway service machine (ASKSERV): CMS/Linux/TELL clients; the model runs in llama.cpp on the PC (or a cloud API), reached through BORDER</t>
+          <t>CMS sockets + httpd</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2278,17 +2280,17 @@
       </c>
       <c r="B63" s="13" t="inlineStr">
         <is>
-          <t>9.11</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="C63" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>dbase</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Kit build 7 (distributable snapshot)</t>
+          <t>xBase / Harbour</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2297,11 +2299,7 @@
         </is>
       </c>
       <c r="F63" s="2" t="n"/>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>After the list above</t>
-        </is>
-      </c>
+      <c r="G63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
@@ -2311,17 +2309,17 @@
       </c>
       <c r="B64" s="13" t="inlineStr">
         <is>
-          <t>9.12</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>Firewall</t>
+          <t>MQ</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Network pack: per-user addresses, CP guest LAN, BORDER firewall, inside DHCP/DNS (9.12a-d)</t>
+          <t>MQ and MQTT (CMS and Debian)</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2332,7 +2330,7 @@
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>After M4b.3, before M9</t>
+          <t>mosquitto on Debian done</t>
         </is>
       </c>
     </row>
@@ -2344,32 +2342,28 @@
       </c>
       <c r="B65" s="13" t="inlineStr">
         <is>
-          <t>9.12a</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>APL</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Per-user IP address at disk IPL from the directory (fixes I-266)</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>11 Oct</t>
-        </is>
-      </c>
+          <t>APL in C on CMS</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Address follows the CTC pair (62x/63x or real); vm370plus-net on both Debian disks; verified 10.1.2.2 by itself</t>
+          <t>Debian 34/34; CMS run pending</t>
         </is>
       </c>
     </row>
@@ -2381,17 +2375,17 @@
       </c>
       <c r="B66" s="13" t="inlineStr">
         <is>
-          <t>9.12b</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>Guest LAN</t>
+          <t>REXX</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>CP virtual NIC per guest on one internal segment (LCS/QETH style, like z/VM Guest LAN)</t>
+          <t>ooRexx 5 on Debian</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2400,11 +2394,7 @@
         </is>
       </c>
       <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Needed for DHCP: CTC links are point-to-point</t>
-        </is>
-      </c>
+      <c r="G66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
@@ -2414,17 +2404,17 @@
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>9.12c</t>
+          <t>9.10</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
         <is>
-          <t>Firewall</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>BORDER service machine: only outside link; NAT outbound; port forwards to service machines (httpd 9.5). One network configuration file on MAINT: OUTSIDE DHCP (bridged LCS/tap, address from the LAN) or OUTSIDE STATIC ip/mask gw; inside subnet and addressing; EXPOSE proto port TO user|ip port (default: nothing exposed)</t>
+          <t>AI gateway service machine (ASKSERV): CMS/Linux/TELL clients; the model runs in llama.cpp on the PC (or a cloud API), reached through BORDER</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2433,11 +2423,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>Outside link may be bridged (LCS on tap) to get its address from the LAN DHCP</t>
-        </is>
-      </c>
+      <c r="G67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
@@ -2447,17 +2433,17 @@
       </c>
       <c r="B68" s="13" t="inlineStr">
         <is>
-          <t>9.12d</t>
+          <t>9.11</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
         <is>
-          <t>DHCP/DNS</t>
+          <t>Snapshot</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>DHCP and DNS for the inside segment as a service machine (dnsmasq on Debian, or in BORDER)</t>
+          <t>Kit build 7 (distributable snapshot)</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2468,7 +2454,7 @@
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Needs 9.12b</t>
+          <t>After the list above</t>
         </is>
       </c>
     </row>
@@ -2480,17 +2466,17 @@
       </c>
       <c r="B69" s="13" t="inlineStr">
         <is>
-          <t>9.13</t>
+          <t>9.12</t>
         </is>
       </c>
       <c r="C69" s="14" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Firewall</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Public VM/370 tools for the kit (survey 11 Oct)</t>
+          <t>Network pack: per-user addresses, CP guest LAN, BORDER firewall, inside DHCP/DNS (9.12a-d)</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2501,7 +2487,7 @@
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Before kit 7 (9.11)</t>
+          <t>After M4b.3, before M9</t>
         </is>
       </c>
     </row>
@@ -2513,26 +2499,34 @@
       </c>
       <c r="B70" s="13" t="inlineStr">
         <is>
-          <t>9.13a</t>
+          <t>9.12a</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>Pascal</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>New Stanford Pascal (Oppolzer, github StanfordPascal/Pascal) replaces CE 2021.03</t>
+          <t>Per-user IP address at disk IPL from the directory (fixes I-266)</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="n"/>
-      <c r="G70" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Address follows the CTC pair (62x/63x or real); vm370plus-net on both Debian disks; verified 10.1.2.2 by itself</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="14" t="inlineStr">
@@ -2542,17 +2536,17 @@
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>9.13b</t>
+          <t>9.12b</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>NJE</t>
+          <t>Guest LAN</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>RSCS NJE updates (Coghlan) + TCPNJE: VM/370 NJE to MVS/z/OS/Linux</t>
+          <t>CP virtual NIC per guest on one internal segment (LCS/QETH style, like z/VM Guest LAN)</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -2563,7 +2557,7 @@
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13</t>
+          <t>Needed for DHCP: CTC links are point-to-point</t>
         </is>
       </c>
     </row>
@@ -2575,17 +2569,17 @@
       </c>
       <c r="B72" s="13" t="inlineStr">
         <is>
-          <t>9.13c</t>
+          <t>9.12c</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>NJE Linux</t>
+          <t>Firewall</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>UnixNJE (FUNET-NJE) in the Debian guest: CMS &lt;-&gt; Linux NJE</t>
+          <t>BORDER service machine: only outside link; NAT outbound; port forwards to service machines (httpd 9.5). One network configuration file on MAINT: OUTSIDE DHCP (bridged LCS/tap, address from the LAN) or OUTSIDE STATIC ip/mask gw; inside subnet and addressing; EXPOSE proto port TO user|ip port (default: nothing exposed)</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -2596,7 +2590,7 @@
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Needs 9.13b</t>
+          <t>Outside link may be bridged (LCS on tap) to get its address from the LAN DHCP</t>
         </is>
       </c>
     </row>
@@ -2608,17 +2602,17 @@
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>9.13d</t>
+          <t>9.12d</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
         <is>
-          <t>Sockets</t>
+          <t>DHCP/DNS</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>NICOF + CMSFTPD (devhawala, public domain): sockets API and FTP for CMS</t>
+          <t>DHCP and DNS for the inside segment as a service machine (dnsmasq on Debian, or in BORDER)</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -2629,7 +2623,7 @@
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Test before 9.5 (CMS sockets + httpd)</t>
+          <t>Needs 9.12b</t>
         </is>
       </c>
     </row>
@@ -2641,17 +2635,17 @@
       </c>
       <c r="B74" s="13" t="inlineStr">
         <is>
-          <t>9.13e</t>
+          <t>9.13</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>Games</t>
+          <t>Tools</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Game disk: VM/370 games tape (IBM VS BASIC runtime removed), WIOS SNAKE/SLASH, CALL-OS BASIC TREK2, Zork/Dungeon</t>
+          <t>Public VM/370 tools for the kit (survey 11 Oct)</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -2660,7 +2654,11 @@
         </is>
       </c>
       <c r="F74" s="2" t="n"/>
-      <c r="G74" s="2" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Before kit 7 (9.11)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="14" t="inlineStr">
@@ -2670,17 +2668,17 @@
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>9.13f</t>
+          <t>9.13a</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Pascal</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>VM Workshop 1985/86 tools that run on R6: CARD, FCOPY, CLUST/TERM macros; check DISKPRY, LEDIT, IEBCOPY, JSCAN</t>
+          <t>New Stanford Pascal (Oppolzer, github StanfordPascal/Pascal) replaces CE 2021.03</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -2689,11 +2687,7 @@
         </is>
       </c>
       <c r="F75" s="2" t="n"/>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>CPWATCH (85 M0083) is 4c</t>
-        </is>
-      </c>
+      <c r="G75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="14" t="inlineStr">
@@ -2703,17 +2697,17 @@
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>9.14</t>
+          <t>9.13b</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>TELL</t>
+          <t>NJE</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>TELL everywhere: CMS TELL EXEC (CP MSG local, RSCS/NJE remote), Linux tell (vmcp, kernel CONFIG_VMCP) with incoming MSG captured, PC client through BORDER (CHATBOT-style gateway)</t>
+          <t>RSCS NJE updates (Coghlan) + TCPNJE: VM/370 NJE to MVS/z/OS/Linux</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -2724,7 +2718,7 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct</t>
+          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13</t>
         </is>
       </c>
     </row>
@@ -2736,17 +2730,17 @@
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>9.15</t>
+          <t>9.13c</t>
         </is>
       </c>
       <c r="C77" s="14" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>NJE Linux</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Python on CMS: the C89 implementation from mikebeer/python (in creation), built with GCC for CMS; Debian uses standard wheezy python 2.7/3.2 packages</t>
+          <t>UnixNJE (FUNET-NJE) in the Debian guest: CMS &lt;-&gt; Linux NJE</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -2757,7 +2751,7 @@
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct</t>
+          <t>Needs 9.13b</t>
         </is>
       </c>
     </row>
@@ -2769,32 +2763,28 @@
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>9.16</t>
+          <t>9.13d</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>TDISK</t>
+          <t>Sockets</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>TDISK EXEC: TDISK [cyls] [fm] defines, formats and (with fm) accesses a temporary disk; HELP TDISK</t>
+          <t>NICOF + CMSFTPD (devhawala, public domain): sockets API and FTP for CMS</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>11 Oct</t>
-        </is>
-      </c>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct</t>
+          <t>Test before 9.5 (CMS sockets + httpd)</t>
         </is>
       </c>
     </row>
@@ -2806,17 +2796,17 @@
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>9.17</t>
+          <t>9.13e</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Tiny LLM</t>
+          <t>Games</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>llama2.c-style inference of a tiny model (stories15M) natively on Debian/390 and on CMS (C, high storage, HFP/BFP and byte order converted): a demonstration; real models via 9.10</t>
+          <t>Game disk: VM/370 games tape (IBM VS BASIC runtime removed), WIOS SNAKE/SLASH, CALL-OS BASIC TREK2, Zork/Dungeon</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -2825,36 +2815,60 @@
         </is>
       </c>
       <c r="F79" s="2" t="n"/>
-      <c r="G79" s="2" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; llama.cpp itself needs 64-bit, C++17 and GBs</t>
-        </is>
-      </c>
+      <c r="G79" s="2" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n"/>
-      <c r="B80" s="10" t="n"/>
-      <c r="C80" s="2" t="n"/>
-      <c r="D80" s="2" t="n"/>
-      <c r="E80" s="5" t="n"/>
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>9.13f</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>VM Workshop 1985/86 tools that run on R6: CARD, FCOPY, CLUST/TERM macros; check DISKPRY, LEDIT, IEBCOPY, JSCAN</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F80" s="2" t="n"/>
-      <c r="G80" s="2" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>CPWATCH (85 M0083) is 4c</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B81" s="10" t="n"/>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>9.14</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>TELL</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>z/Architecture (64-bit)</t>
+          <t>TELL everywhere: CMS TELL EXEC (CP MSG local, RSCS/NJE remote), Linux tell (vmcp, kernel CONFIG_VMCP) with incoming MSG captured, PC client through BORDER (CHATBOT-style gateway)</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -2863,145 +2877,177 @@
         </is>
       </c>
       <c r="F81" s="2" t="n"/>
-      <c r="G81" s="2" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.15</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D82" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="n"/>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Python on CMS: the C89 implementation from mikebeer/python (in creation), built with GCC for CMS; Debian uses standard wheezy python 2.7/3.2 packages</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F82" s="2" t="n"/>
-      <c r="G82" s="2" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.16</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D83" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="n"/>
-      <c r="F83" s="2" t="n"/>
-      <c r="G83" s="2" t="n"/>
+          <t>TDISK</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>TDISK EXEC: TDISK [cyls] [fm] defines, formats and (with fm) accesses a temporary disk; HELP TDISK</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.17</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D84" s="14" t="inlineStr">
-        <is>
-          <t>Kit 8</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="n"/>
+          <t>Tiny LLM</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>llama2.c-style inference of a tiny model (stories15M) natively on Debian/390 and on CMS (C, high storage, HFP/BFP and byte order converted): a demonstration; real models via 9.10</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F84" s="2" t="n"/>
-      <c r="G84" s="2" t="n"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; llama.cpp itself needs 64-bit, C++17 and GBs</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="14" t="n"/>
-      <c r="B85" s="13" t="n"/>
-      <c r="C85" s="14" t="n"/>
-      <c r="D85" s="14" t="n"/>
-      <c r="E85" s="5" t="n"/>
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>9.18</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>SENDMAIL / GETMAIL for CMS via a MAILER service machine (SMTP out through BORDER; POP/IMAP or SMTP in, delivered to the reader in class M)</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F85" s="2" t="n"/>
-      <c r="G85" s="2" t="n"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; after 9.12</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B86" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C86" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E86" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="10" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="5" t="n"/>
       <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B87" s="13" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="C87" s="14" t="inlineStr">
-        <is>
-          <t>More Languages</t>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="n"/>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E87" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="F87" s="2" t="n"/>
@@ -3010,116 +3056,84 @@
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>FreeSWITCH</t>
-        </is>
-      </c>
-      <c r="E88" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="n"/>
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C89" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
-        </is>
-      </c>
-      <c r="E89" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="n"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>Snapshot</t>
         </is>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
-        </is>
-      </c>
-      <c r="E90" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Kit 8</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="n"/>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B91" s="13" t="inlineStr">
-        <is>
-          <t>11.6</t>
-        </is>
-      </c>
-      <c r="C91" s="14" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="inlineStr">
-        <is>
-          <t>CFSERV</t>
-        </is>
-      </c>
-      <c r="E91" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A91" s="14" t="n"/>
+      <c r="B91" s="13" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="14" t="n"/>
+      <c r="E91" s="5" t="n"/>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="n"/>
     </row>
@@ -3131,20 +3145,24 @@
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D92" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="n"/>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
     </row>
@@ -3156,37 +3174,352 @@
       </c>
       <c r="B93" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C93" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D93" s="14" t="inlineStr">
-        <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="n"/>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+        </is>
+      </c>
+      <c r="E93" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="n"/>
-      <c r="B94" s="11" t="n"/>
-      <c r="C94" s="8" t="n"/>
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B94" s="13" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>VoIP</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>FreeSWITCH</t>
+        </is>
+      </c>
+      <c r="E94" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="n"/>
+      <c r="G94" s="2" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="n"/>
-      <c r="B95" s="11" t="n"/>
-      <c r="C95" s="8" t="n"/>
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B95" s="13" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>IoT</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>Node-RED</t>
+        </is>
+      </c>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="n"/>
+      <c r="G95" s="2" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="7" t="n"/>
-      <c r="B96" s="12" t="n"/>
-      <c r="C96" s="7" t="n"/>
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B96" s="13" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>Container</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="n"/>
+      <c r="G96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B97" s="13" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E97" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n"/>
+      <c r="G97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="n"/>
+      <c r="F98" s="2" t="n"/>
+      <c r="G98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B99" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C99" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="n"/>
+      <c r="F99" s="2" t="n"/>
+      <c r="G99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="n"/>
+      <c r="B100" s="11" t="n"/>
+      <c r="C100" s="8" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>12a</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>12b</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>12c</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>12e</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>srorso/dos360install</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="n"/>
+      <c r="B106" s="11" t="n"/>
+      <c r="C106" s="8" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="n"/>
+      <c r="B107" s="12" t="n"/>
+      <c r="C107" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
Guide and plan: EDF disks (M6a-M6d done)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -1461,7 +1461,7 @@
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Before M9</t>
+          <t>6a-6d done 11 Oct (EDF under IPL 290); 6e open</t>
         </is>
       </c>
     </row>
@@ -1488,11 +1488,19 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>25de15c; T3350 temp disk and dedicated 3380</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1554,11 +1562,19 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>14bae66; 70,000-record copy byte-identical (edf.py)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1578,16 +1594,24 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Large minidisks (full-volume 3390)</t>
+          <t>Large minidisks: a full-volume 3380 as one EDF disk</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>a101a8f; full 885-cyl 3380 (518 MB); one 112 MB file, 1.4M records, verified</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">

</xml_diff>

<commit_message>
M6e: tools on EDF disks; a saturating item count means 'next'
OS simulation (MOVEFILE) stops its halfword item count at 65,535, so
DMSEFS takes 65,535 after a 65,535 as the next item. Before this,
MOVEFILE of a 100,000-record V file reread record 65,535 forever.

Checked on an EDF temporary disk:
- DISK DUMP.
- MOVEFILE of TDISK EXEC and of the 100,000-record V file.
- COMPARE.
DISK LOAD writes to the A disk by design (as before).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -1455,13 +1455,17 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>6a-6d done 11 Oct (EDF under IPL 290); 6e open</t>
+          <t>EDF under IPL 290 (docs/63); 31-bit nucleus sweep stays background (doc 62 B)</t>
         </is>
       </c>
     </row>
@@ -1636,11 +1640,19 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>DISK DUMP, MOVEFILE (100,000-record V file), COMPARE, COPYFILE on EDF; DISK LOAD writes to A by design; TAPE not run (same RDBUF/WRBUF path)</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="25.5" customHeight="1">
       <c r="A41" s="2" t="n"/>

</xml_diff>

<commit_message>
Kit build 7 delivered and verified on a fresh CE (kt16)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2484,13 +2484,17 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>After the list above</t>
+          <t>b7, 13 parts; verified on a fresh CE (kt16): EDF, TDISK, IPL LINUX</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan: 9.8 APL done (CMS 33/33); 9.19 GnuCOBOL, 9.20 PL/I research
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2393,13 +2393,17 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Debian 34/34; CMS run pending</t>
+          <t>Debian 34/34; CMS 33/33 (primes.apl has lines over 80 columns); e551b9e; needs Hercules 4</t>
         </is>
       </c>
     </row>
@@ -3060,29 +3064,57 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n"/>
-      <c r="B86" s="10" t="n"/>
-      <c r="C86" s="2" t="n"/>
-      <c r="D86" s="2" t="n"/>
-      <c r="E86" s="5" t="n"/>
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>9.19</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>COBOL</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>GnuCOBOL: Debian (open-cobol 1.1 from the wheezy archive, then GnuCOBOL 3.x built natively); CMS through the cross route (cobc -C to C, GCC -m31 with a cross-built libcob and GMP, TEXT/MODULE under IPL 290)</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F86" s="2" t="n"/>
-      <c r="G86" s="2" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; CE has only the old COBOL</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="14" t="inlineStr">
         <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B87" s="10" t="n"/>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>9.20</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>PL/I</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>z/Architecture (64-bit)</t>
+          <t>PL/I beyond CE's PL/I(F): research first -- no maintained open PL/I for s390 (Iron Spring is x86 and closed, pl1gcc unfinished); options: document PL/I(F), a PL/I subset to C translator, old subsets (PL/I-G)</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -3091,29 +3123,17 @@
         </is>
       </c>
       <c r="F87" s="2" t="n"/>
-      <c r="G87" s="2" t="n"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B88" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C88" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D88" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="10" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
       <c r="E88" s="5" t="n"/>
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
@@ -3124,22 +3144,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B89" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C89" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D89" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="n"/>
+      <c r="B89" s="10" t="n"/>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
     </row>
@@ -3151,17 +3171,17 @@
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E90" s="5" t="n"/>
@@ -3169,10 +3189,26 @@
       <c r="G90" s="2" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="n"/>
-      <c r="B91" s="13" t="n"/>
-      <c r="C91" s="14" t="n"/>
-      <c r="D91" s="14" t="n"/>
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B91" s="13" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
       <c r="E91" s="5" t="n"/>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="n"/>
@@ -3180,58 +3216,34 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E92" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B93" s="13" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="C93" s="14" t="inlineStr">
-        <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E93" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A93" s="14" t="n"/>
+      <c r="B93" s="13" t="n"/>
+      <c r="C93" s="14" t="n"/>
+      <c r="D93" s="14" t="n"/>
+      <c r="E93" s="5" t="n"/>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
     </row>
@@ -3243,17 +3255,17 @@
       </c>
       <c r="B94" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C94" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D94" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E94" s="16" t="inlineStr">
@@ -3272,17 +3284,17 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr">
@@ -3301,17 +3313,17 @@
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E96" s="16" t="inlineStr">
@@ -3330,17 +3342,17 @@
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C97" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
@@ -3359,20 +3371,24 @@
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="n"/>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E98" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="n"/>
     </row>
@@ -3384,86 +3400,81 @@
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
-      <c r="E99" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E99" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="n"/>
-      <c r="B100" s="11" t="n"/>
-      <c r="C100" s="8" t="n"/>
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B100" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C100" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D100" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="n"/>
+      <c r="F100" s="2" t="n"/>
+      <c r="G100" s="2" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B101" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B101" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="n"/>
+      <c r="F101" s="2" t="n"/>
+      <c r="G101" s="2" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B102" s="11" t="inlineStr">
-        <is>
-          <t>12b</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A102" s="8" t="n"/>
+      <c r="B102" s="11" t="n"/>
+      <c r="C102" s="8" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
@@ -3473,7 +3484,7 @@
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
@@ -3483,12 +3494,17 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3516,7 @@
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
@@ -3510,7 +3526,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3527,39 +3543,93 @@
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
+          <t>12c</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C105" s="8" t="inlineStr">
+      <c r="C107" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D107" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
+      <c r="G107" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="8" t="n"/>
-      <c r="B106" s="11" t="n"/>
-      <c r="C106" s="8" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="7" t="n"/>
-      <c r="B107" s="12" t="n"/>
-      <c r="C107" s="7" t="n"/>
+    <row r="108">
+      <c r="A108" s="8" t="n"/>
+      <c r="B108" s="11" t="n"/>
+      <c r="C108" s="8" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="n"/>
+      <c r="B109" s="12" t="n"/>
+      <c r="C109" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.19: GnuCOBOL 3.1.2 on Debian/390 (cross-built against wheezy glibc); I-270 recorded
mkcobol-linux.sh builds cobc + static libcob + GMP 6.3 with GCC 13 -m31
against wheezy's glibc 2.13. config.h fix for cross builds: COB_LI_IS_LL
must be undefined on 31-bit (10-19 digit values were 0). Test programs
under VM/370plus (cb1) give output identical to the PC build.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A3:G109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -450,8 +450,6 @@
     <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3081,18 +3079,22 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>GnuCOBOL: Debian (open-cobol 1.1 from the wheezy archive, then GnuCOBOL 3.x built natively); CMS through the cross route (cobc -C to C, GCC -m31 with a cross-built libcob and GMP, TEXT/MODULE under IPL 290)</t>
+          <t>GnuCOBOL 3.1.2. Debian: cross-built cobc + static libcob + GMP 6.3 against wheezy glibc, gcc 4.6 compiles the generated C (done 11 Oct). CMS goal: compile natively -- first cobc/libcob through the cross route (GCC -m31, newlib, cmsrt), then built on CMS by GCC380/GCCLIB31 with a COBOL EXEC (cobc -C, GCC, LOAD, GENMOD)</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct–</t>
+        </is>
+      </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct; CE has only the old COBOL</t>
+          <t>Owner request 11 Oct; CE has only the old COBOL. Debian verified (cb1): test programs identical to the PC; languages/cobol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.20: PL/I research (docs/64-PLI.md); CE PL/I verified under VM/370plus
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3121,13 +3121,17 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="n"/>
+          <t>Research done</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct</t>
+        </is>
+      </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct</t>
+          <t>Owner request 11 Oct. docs/64-PLI.md: CE PL/I works under VM/370plus (pl2, GLOBAL TXTLIB PLILIB); no open PL/I targets s390 or C; next: PLI EXEC polish, then a subset-to-C translator after the 9.19 native-compiler decision</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.21 C/C++ toolchain on CMS (plan row), I-271 EDF module crash; cmsrt: reentrant errno for POSIX calls, =STACK continuation, MAXARGS 128, .got in XIMAGE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G109"/>
+  <dimension ref="A3:G110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3121,51 +3121,63 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>Research done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>11 Oct</t>
+          <t>11 Oct–</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct. docs/64-PLI.md: CE PL/I works under VM/370plus (pl2, GLOBAL TXTLIB PLILIB); no open PL/I targets s390 or C; next: PLI EXEC polish, then a subset-to-C translator after the 9.19 native-compiler decision</t>
+          <t>mikebeer/pli (PL/I to C89): native on CMS with GCC380 (PLIC EXEC), 17 of 19 tests (pp1-pp3); Debian next. docs/64-PLI.md</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n"/>
-      <c r="B88" s="10" t="n"/>
-      <c r="C88" s="2" t="n"/>
-      <c r="D88" s="2" t="n"/>
-      <c r="E88" s="5" t="n"/>
-      <c r="F88" s="2" t="n"/>
-      <c r="G88" s="2" t="n"/>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>9.21</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>C/C++</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Modern C/C++ toolchain on CMS: GCC 13.3 cc1/cc1plus and binutils 2.42 (as, ld, ar) cross-built for the M5f runtime; XL loader for programs above 16 MB; sysroot tar as read-only VFS; CC EXEC; then COBOL (9.19) compiles natively</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>12 Oct–</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Owner decision 12 Oct (GCC380 cannot do long long additions). Done: XL loader (xl1), as on CMS (tc3); cc1 runs on CMS</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A89" s="2" t="n"/>
       <c r="B89" s="10" t="n"/>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+      <c r="E89" s="5" t="n"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
     </row>
@@ -3175,22 +3187,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B90" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C90" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D90" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="n"/>
+      <c r="B90" s="10" t="n"/>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="n"/>
     </row>
@@ -3202,7 +3214,7 @@
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C91" s="14" t="inlineStr">
@@ -3212,7 +3224,7 @@
       </c>
       <c r="D91" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E91" s="5" t="n"/>
@@ -3227,17 +3239,17 @@
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E92" s="5" t="n"/>
@@ -3245,40 +3257,36 @@
       <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="14" t="n"/>
-      <c r="B93" s="13" t="n"/>
-      <c r="C93" s="14" t="n"/>
-      <c r="D93" s="14" t="n"/>
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B93" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
       <c r="E93" s="5" t="n"/>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C94" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E94" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A94" s="14" t="n"/>
+      <c r="B94" s="13" t="n"/>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="14" t="n"/>
+      <c r="E94" s="5" t="n"/>
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
     </row>
@@ -3290,17 +3298,17 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr">
@@ -3319,17 +3327,17 @@
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E96" s="16" t="inlineStr">
@@ -3348,17 +3356,17 @@
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C97" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
@@ -3377,17 +3385,17 @@
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E98" s="16" t="inlineStr">
@@ -3406,17 +3414,17 @@
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
@@ -3435,20 +3443,24 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E100" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="n"/>
     </row>
@@ -3460,17 +3472,17 @@
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E101" s="5" t="n"/>
@@ -3478,41 +3490,34 @@
       <c r="G101" s="2" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="n"/>
-      <c r="B102" s="11" t="n"/>
-      <c r="C102" s="8" t="n"/>
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B102" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="n"/>
+      <c r="F102" s="2" t="n"/>
+      <c r="G102" s="2" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B103" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C103" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A103" s="8" t="n"/>
+      <c r="B103" s="11" t="n"/>
+      <c r="C103" s="8" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
@@ -3522,7 +3527,7 @@
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
@@ -3532,12 +3537,17 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3549,7 +3559,7 @@
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
@@ -3559,7 +3569,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -3576,7 +3586,7 @@
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
@@ -3586,7 +3596,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3603,39 +3613,66 @@
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C107" s="8" t="inlineStr">
+      <c r="C108" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D108" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G108" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="8" t="n"/>
-      <c r="B108" s="11" t="n"/>
-      <c r="C108" s="8" t="n"/>
-    </row>
     <row r="109">
-      <c r="A109" s="7" t="n"/>
-      <c r="B109" s="12" t="n"/>
-      <c r="C109" s="7" t="n"/>
+      <c r="A109" s="8" t="n"/>
+      <c r="B109" s="11" t="n"/>
+      <c r="C109" s="8" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="n"/>
+      <c r="B110" s="12" t="n"/>
+      <c r="C110" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
Milestones: 9.21 and 9.19 done, 9.3 superseded; I-272 (CP hang at LOGOFF); PL/I: CMS file names, '/*' ends stdin; Guide chapter 8 (compilers); READMEs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2242,11 +2242,15 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="n"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Superseded by 9.21: full GCC 13 C++ natively on CMS, not a subset</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
@@ -3084,7 +3088,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3094,7 +3098,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct; CE has only the old COBOL. Debian verified (cb1): test programs identical to the PC. CMS cross route verified (cc3): same output on CMS. Next: cobc and the compile natively on CMS (GCC380). languages/cobol</t>
+          <t>Debian (cb1) and CMS cross route (cc3) identical to the PC; natively on CMS: COBOL EXEC = cobc on CMS + CC EXEC (GCC 13) with libcob/GMP (tc17, 12 Oct). Not included: INDEXED files, SCREEN SECTION. languages/cobol</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3135,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>mikebeer/pli (PL/I to C89): native on CMS with GCC380 (PLIC EXEC), 17 of 19 tests (pp1-pp3); Debian next. docs/64-PLI.md</t>
+          <t>mikebeer/pli (PL/I to C): PLIC EXEC natively on CMS, now via GCC 13 (IEEE float matches the PC); tc21: 12 of 18 identical, rest console spacing, file-name clash (fixed in PLICMS H), T11 needs EOF (cmsrt '/*'); Debian next. CE PL/I(F) works too. docs/64-PLI.md</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3162,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3168,7 +3172,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Owner decision 12 Oct (GCC380 cannot do long long additions). Done: XL loader (xl1), as on CMS (tc3); cc1 runs on CMS</t>
+          <t>Owner decision 12 Oct (GCC380 cannot add long longs). GCC 13.3 cc1/cc1plus (XL loader, above 16 MB), binutils 2.42 as/ld/ar, elf2cms, CC EXEC; SYSROOT TAR + CXXROOT TAR; libstdc++ 13.3 built for newlib/soft float. Native C (tc15/16), C++ incl. iostreams (tc20/21). No C++ exceptions yet. toolchain/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.15 done (Python on CMS, 27/29 = CPython); 9.20: PL/I 19/19 on CMS through GCC 13
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2952,13 +2952,13 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct</t>
+          <t>mikebeer/python (C89, NumPy/pandas/SciPy built in) as PY XIMAGE, PYTHON EXEC; 27 of 29 tests = CPython on CMS (tc23/24; 15_import needs package files, 24_sockets: no sockets yet). 32-bit long fix pushed to mikebeer/python (6e4a7a5). languages/python</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>mikebeer/pli (PL/I to C): PLIC EXEC natively on CMS, now via GCC 13 (IEEE float matches the PC); tc21: 12 of 18 identical, rest console spacing, file-name clash (fixed in PLICMS H), T11 needs EOF (cmsrt '/*'); Debian next. CE PL/I(F) works too. docs/64-PLI.md</t>
+          <t>mikebeer/pli (PL/I to C): PLIC EXEC natively on CMS through GCC 13: 19 of 19 tests = PC (tc22-24). CE PL/I(F) works too. Debian next. docs/64-PLI.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.20 done: PL/I on Debian 19/19; SQLite for CMS (build, SQLITE EXEC, tests); cmsrt: fsync writes, ftruncate, F_GETLK unlocked, DB filetypes binary, POSIX stubs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3125,7 +3125,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>mikebeer/pli (PL/I to C): PLIC EXEC natively on CMS through GCC 13: 19 of 19 tests = PC (tc22-24). CE PL/I(F) works too. Debian next. docs/64-PLI.md</t>
+          <t>mikebeer/pli (PL/I to C89): CMS -- PLIC EXEC through GCC 13, 19/19 tests = PC (tc22-24); Debian -- pli + plic with gcc 4.6, 19/19 (pd1). CE PL/I(F) also works. docs/64-PLI.md, languages/pli</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.4: SQLite 3.46.1 on CMS (SQLITE EXEC); cmsrt: POSIX lseek, stat of open files, nlink, /fn.ft as a CMS file
tc31: the test script gives the PC's output line for line; the database
persists and passes integrity_check when reopened.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2275,11 +2275,15 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F61" s="2" t="n"/>
-      <c r="G61" s="2" t="n"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>SQLite 3.46.1 on CMS done (SQLITE EXEC, tc31: output = PC, database persists); next SQLSERV service machine; MariaDB/PostgreSQL on Debian. languages/sqlite</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="14" t="inlineStr">

</xml_diff>

<commit_message>
9.13a: New Stanford Pascal 2026.10 on CMS (PCINT cross-built, big-endian fix; PCPAS/PCRUN)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2733,11 +2733,15 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F75" s="2" t="n"/>
-      <c r="G75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>New Stanford Pascal 2026.10 on CMS via PCINT (cross-built, 31-bit; big-endian fix pcint-bigendian.patch): PCPAS/PCRUN EXECs, tc33 output = PC. Native 370 code needs a PASCAL2 newer than the published 2024.02. CE 2021.03 unchanged. languages/pascal</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="14" t="inlineStr">

</xml_diff>

<commit_message>
9.6: xBase (mikebeer/xbase 3ca444f) on CMS, 7/7 tests; cmsrt: DBF/DBT/XDX binary; edf.py RAW (exact bytes as V records)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2337,11 +2337,15 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F63" s="2" t="n"/>
-      <c r="G63" s="2" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>mikebeer/xbase (xBase/Clipper/Harbour-style, in cREXX) on CMS (XBASE EXEC, RXBVM8; tc37 7/7 tests = PC; index read fix pushed upstream 3ca444f) and Debian (cREXX bundle). Harbour itself not ported. languages/xbase</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">

</xml_diff>

<commit_message>
milestones: 9.6 xBase C89, 9.19 COBX 19/19, 9.20 PL/I 79eae4d 34/35 on CMS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2343,7 +2343,7 @@
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>mikebeer/xbase (xBase/Clipper/Harbour-style, in cREXX) on CMS (XBASE EXEC, RXBVM8; tc37 7/7 tests = PC; index read fix pushed upstream 3ca444f) and Debian (cREXX bundle). Harbour itself not ported. languages/xbase</t>
+          <t>mikebeer/xbase on CMS and Debian: cREXX version (XBASE RXBIN, tc37 7/7) and the C89 version (XBASEC XIMAGE via XL; tc42 7/7 = PC; 32-bit long fixes pushed upstream 7d2a188); Debian xbase-c. Harbour itself not ported. languages/xbase (mkxbasec.sh)</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Debian (cb1) and CMS cross route (cc3) identical to the PC; natively on CMS: COBOL EXEC = cobc on CMS + CC EXEC (GCC 13) with libcob/GMP (tc17, 12 Oct). Not included: INDEXED files, SCREEN SECTION. languages/cobol</t>
+          <t>GnuCOBOL: Debian (cb1) and CMS natively (COBOL EXEC, tc17). Plus mikebeer/cobol (COBOL-85 + OO, indexed files) as COBX EXEC on CMS: 19/19 tests = PC (tc41-44; record files binary via cobrt-cms.patch); Debian cobol translator. languages/cobol, languages/cobol2c</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>mikebeer/pli (PL/I to C89): CMS -- PLIC EXEC through GCC 13, 19/19 tests = PC (tc22-24); Debian -- pli + plic with gcc 4.6, 19/19 (pd1). CE PL/I(F) also works. docs/64-PLI.md, languages/pli</t>
+          <t>mikebeer/pli 79eae4d (Enterprise PL/I subset to C89): CMS PLIC EXEC through GCC 13, 34/35 tests = PC (tc43-45; t32 AREA counts differ by pointer size); Debian pli + plic. CE PL/I(F) also works. docs/64-PLI.md, languages/pli</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Debian language bundle results: APL 34/34, COBOL 20/20, PL/I 38/39, xBase C 7/7, Smalltalk C 21/22 (pd2/pd3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3110,7 +3110,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>GnuCOBOL: Debian (cb1) and CMS natively (COBOL EXEC, tc17). Plus mikebeer/cobol (COBOL-85 + OO, indexed files) as COBX EXEC on CMS: 19/19 tests = PC (tc41-44; record files binary via cobrt-cms.patch); Debian cobol translator. languages/cobol, languages/cobol2c</t>
+          <t>GnuCOBOL: Debian (cb1) and CMS natively (COBOL EXEC, tc17). Plus mikebeer/cobol (COBOL-85 + OO, indexed files): CMS COBX EXEC 19/19 = PC (tc41-44; record files binary via cobrt-cms.patch); Debian 20/20 (pd2/pd3, languages/common/mkdebtests.sh). languages/cobol, languages/cobol2c</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>mikebeer/pli 79eae4d (Enterprise PL/I subset to C89): CMS PLIC EXEC through GCC 13, 34/35 tests = PC (tc43-45; t32 AREA counts differ by pointer size); Debian pli + plic. CE PL/I(F) also works. docs/64-PLI.md, languages/pli</t>
+          <t>mikebeer/pli 79eae4d (Enterprise PL/I subset to C89): CMS PLIC EXEC through GCC 13, 34/35 = PC (tc43-45); Debian 38/39 incl. multi-file and separately compiled modules (pd2/pd3). Only difference both places: t32 AREA count depends on pointer size. CE PL/I(F) also works. docs/64-PLI.md, languages/pli</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
milestones: 9.22 UNTERSE, 9.23 Info-ZIP/gzip on CMS (owner request), 9.24 kit b8 with LANG disk; LANG and LANGGEN EXECs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G110"/>
+  <dimension ref="A3:G113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3189,85 +3189,113 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n"/>
-      <c r="B89" s="10" t="n"/>
-      <c r="C89" s="2" t="n"/>
-      <c r="D89" s="2" t="n"/>
-      <c r="E89" s="5" t="n"/>
-      <c r="F89" s="2" t="n"/>
-      <c r="G89" s="2" t="n"/>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>9.22</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>UNTERSE</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>TERSE/UNTERSE for CMS and Debian: a C89 TERSE (PACK/SPACK) decompressor after IBM's open-source one, then compression; built with GCC 13 for CMS</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Owner request 12 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B90" s="10" t="n"/>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>9.23</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Info-ZIP zip/unzip and gzip built natively for CMS (GCC 13, cmsrt), beside CE's MINIZIP/MINIUNZ and VMARC</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="F90" s="2" t="n"/>
-      <c r="G90" s="2" t="n"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Owner request 12 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B91" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C91" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="n"/>
-      <c r="F91" s="2" t="n"/>
-      <c r="G91" s="2" t="n"/>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>9.24</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Kit b8: LANG disk (MAINT 19F, VMLANG) with all CMS languages, LANG EXEC, Guide chapter 8, Debian language bundle installed</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>12 Oct–</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Owner decision 12 Oct: a new LANG disk, linked R/O</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B92" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C92" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D92" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="10" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
       <c r="E92" s="5" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
@@ -3278,30 +3306,46 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B93" s="13" t="inlineStr">
-        <is>
-          <t>10.3</t>
-        </is>
-      </c>
-      <c r="C93" s="14" t="inlineStr">
-        <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D93" s="14" t="inlineStr">
-        <is>
-          <t>Kit 8</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="n"/>
+      <c r="B93" s="10" t="n"/>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="n"/>
-      <c r="B94" s="13" t="n"/>
-      <c r="C94" s="14" t="n"/>
-      <c r="D94" s="14" t="n"/>
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B94" s="13" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
+        </is>
+      </c>
       <c r="E94" s="5" t="n"/>
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
@@ -3309,87 +3353,59 @@
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E95" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="n"/>
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E96" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="n"/>
       <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>11.3</t>
-        </is>
-      </c>
-      <c r="C97" s="14" t="inlineStr">
-        <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D97" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
-        </is>
-      </c>
-      <c r="E97" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A97" s="14" t="n"/>
+      <c r="B97" s="13" t="n"/>
+      <c r="C97" s="14" t="n"/>
+      <c r="D97" s="14" t="n"/>
+      <c r="E97" s="5" t="n"/>
       <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="n"/>
     </row>
@@ -3401,17 +3417,17 @@
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D98" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E98" s="16" t="inlineStr">
@@ -3430,17 +3446,17 @@
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
-        </is>
-      </c>
-      <c r="D99" s="14" t="inlineStr">
-        <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
@@ -3459,17 +3475,17 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E100" s="16" t="inlineStr">
@@ -3488,20 +3504,24 @@
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="n"/>
+          <t>Node-RED</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="n"/>
     </row>
@@ -3513,113 +3533,110 @@
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="n"/>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E102" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F102" s="2" t="n"/>
       <c r="G102" s="2" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="n"/>
-      <c r="B103" s="11" t="n"/>
-      <c r="C103" s="8" t="n"/>
+      <c r="A103" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B103" s="13" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E103" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="n"/>
+      <c r="G103" s="2" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B104" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B104" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="n"/>
+      <c r="F104" s="2" t="n"/>
+      <c r="G104" s="2" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B105" s="11" t="inlineStr">
-        <is>
-          <t>12b</t>
-        </is>
-      </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A105" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B105" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="n"/>
+      <c r="F105" s="2" t="n"/>
+      <c r="G105" s="2" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B106" s="11" t="inlineStr">
-        <is>
-          <t>12c</t>
-        </is>
-      </c>
-      <c r="C106" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A106" s="8" t="n"/>
+      <c r="B106" s="11" t="n"/>
+      <c r="C106" s="8" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
@@ -3629,7 +3646,7 @@
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
@@ -3639,12 +3656,17 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3656,39 +3678,120 @@
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
+          <t>12b</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>12c</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C108" s="8" t="inlineStr">
+      <c r="C111" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
+      <c r="G111" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="8" t="n"/>
-      <c r="B109" s="11" t="n"/>
-      <c r="C109" s="8" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="7" t="n"/>
-      <c r="B110" s="12" t="n"/>
-      <c r="C110" s="7" t="n"/>
+    <row r="112">
+      <c r="A112" s="8" t="n"/>
+      <c r="B112" s="11" t="n"/>
+      <c r="C112" s="8" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="n"/>
+      <c r="B113" s="12" t="n"/>
+      <c r="C113" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
Kit build 8: LANG disk (parts 14-15, JOINLANG), README, Guide (LANG section); verified on a fresh CE (kt17-21); milestone 9.24 done, 9.25 spool bridge planned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G113"/>
+  <dimension ref="A3:G114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3214,7 +3214,6 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Owner request 12 Oct</t>
@@ -3247,7 +3246,6 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>Owner request 12 Oct</t>
@@ -3277,7 +3275,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3287,41 +3285,48 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Owner decision 12 Oct: a new LANG disk, linked R/O</t>
+          <t>b8, 15 parts (14-15: LANG disk with JOINLANG); verified on a fresh CE (kt17-21): VMLANG attached by AUTOLOG1, LANG -&gt; L (19F), SQLite 3.46.1, CC HI -&gt; Hi!, Debian login. CMSUSER A cleaned of old language EXECs/MODULEs</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n"/>
-      <c r="B92" s="10" t="n"/>
-      <c r="C92" s="2" t="n"/>
-      <c r="D92" s="2" t="n"/>
-      <c r="E92" s="5" t="n"/>
-      <c r="F92" s="2" t="n"/>
-      <c r="G92" s="2" t="n"/>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>9.25</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Spool bridge</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Linux services on the service-machine interface: vmspool daemon in the Debian guest (vmur reader/punch) turning requests into Asterisk AMI (PHONE EXEC), MQTT, MariaDB calls; replies punched back like SQLSERV</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Owner question 12 Oct (Asterisk); check vmur against our CP first</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A93" s="2" t="n"/>
       <c r="B93" s="10" t="n"/>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
+      <c r="E93" s="5" t="n"/>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
     </row>
@@ -3331,22 +3336,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C94" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D94" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="n"/>
+      <c r="B94" s="10" t="n"/>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
     </row>
@@ -3358,7 +3363,7 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
@@ -3368,7 +3373,7 @@
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E95" s="5" t="n"/>
@@ -3383,17 +3388,17 @@
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E96" s="5" t="n"/>
@@ -3401,40 +3406,36 @@
       <c r="G96" s="2" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="14" t="n"/>
-      <c r="B97" s="13" t="n"/>
-      <c r="C97" s="14" t="n"/>
-      <c r="D97" s="14" t="n"/>
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B97" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
       <c r="E97" s="5" t="n"/>
       <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B98" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C98" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E98" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A98" s="14" t="n"/>
+      <c r="B98" s="13" t="n"/>
+      <c r="C98" s="14" t="n"/>
+      <c r="D98" s="14" t="n"/>
+      <c r="E98" s="5" t="n"/>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="n"/>
     </row>
@@ -3446,17 +3447,17 @@
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
@@ -3475,17 +3476,17 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D100" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E100" s="16" t="inlineStr">
@@ -3504,17 +3505,17 @@
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
@@ -3533,17 +3534,17 @@
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E102" s="16" t="inlineStr">
@@ -3562,17 +3563,17 @@
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
@@ -3591,20 +3592,24 @@
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C104" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="n"/>
     </row>
@@ -3616,17 +3621,17 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E105" s="5" t="n"/>
@@ -3634,41 +3639,34 @@
       <c r="G105" s="2" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="8" t="n"/>
-      <c r="B106" s="11" t="n"/>
-      <c r="C106" s="8" t="n"/>
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B106" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="n"/>
+      <c r="F106" s="2" t="n"/>
+      <c r="G106" s="2" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A107" s="8" t="n"/>
+      <c r="B107" s="11" t="n"/>
+      <c r="C107" s="8" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
@@ -3678,7 +3676,7 @@
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
@@ -3688,12 +3686,17 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3708,7 @@
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
@@ -3715,7 +3718,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3732,7 +3735,7 @@
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
@@ -3742,7 +3745,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3759,39 +3762,66 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C111" s="8" t="inlineStr">
+      <c r="C112" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
+      <c r="G112" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="8" t="n"/>
-      <c r="B112" s="11" t="n"/>
-      <c r="C112" s="8" t="n"/>
-    </row>
     <row r="113">
-      <c r="A113" s="7" t="n"/>
-      <c r="B113" s="12" t="n"/>
-      <c r="C113" s="7" t="n"/>
+      <c r="A113" s="8" t="n"/>
+      <c r="B113" s="11" t="n"/>
+      <c r="C113" s="8" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="n"/>
+      <c r="B114" s="12" t="n"/>
+      <c r="C114" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.23 ZIP/UNZIP/GZIP on CMS (Info-ZIP 3.0/6.0, zlib minigzip) on the LANG disk; cmsrt: real file dates from the FST (I-273), short mkstemp templates (I-274), ZIP/GZ/TGZ/... binary file types; guide; issues I-273..I-275
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3243,12 +3243,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Owner request 12 Oct</t>
+          <t>Info-ZIP zip 3.0 / unzip 6.0 and gzip (zlib 1.3.1 minigzip) for CMS: IZZIP/IZUNZIP/MINIGZ MODULE + ZIP/UNZIP/GZIP EXEC on the LANG disk; round trip on CMS, PC-made .zip unzips (tc64-71); CMS file dates in the archive (cmsrt stat reads the FST via STATE). gzip names fn ft-GZ. No encryption. languages/zip</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.22 UNTERSE: C89 port of tersedecompress (PACK/SPACK, F/V, text/binary) for CMS (UNTRS MODULE, UNTERSE EXEC, on the LANG disk) and Debian; byte-identical to the z/OS originals on CMS (tc72), PC 120/120; edf.py getraw; milestones 9.26 RXPIP; guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G114"/>
+  <dimension ref="A3:G115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3211,12 +3211,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Owner request 12 Oct</t>
+          <t>UNTERSE done: C89 port of the Open Mainframe Project's tersedecompress (Apache 2): PACK and SPACK, host F/V and native, text and binary; PC 120/120 of the testdata (the 4 others are SPACK files with no data); CMS (tc72) byte-identical to the z/OS originals (FB/VB text, binary). UNTRS MODULE + UNTERSE EXEC; Debian unterse. Next: TERSE (compression). languages/terse</t>
         </is>
       </c>
     </row>
@@ -3322,36 +3322,43 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n"/>
-      <c r="B93" s="10" t="n"/>
-      <c r="C93" s="2" t="n"/>
-      <c r="D93" s="2" t="n"/>
-      <c r="E93" s="5" t="n"/>
-      <c r="F93" s="2" t="n"/>
-      <c r="G93" s="2" t="n"/>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>9.26</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>RXPIP</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>mikebeer/rexxpository (RXPIP, pip-style REXX packages) on VM/370plus: 1) rxpip (Regina) in the Debian guest; 2) TAR for CMS; 3) RXPIPSRV service machine + RXPIP EXEC over reader/punch via the 9.25 bridge; 4) CMS install as EXEC files (external functions), CMSNAME map; platform tags brexx-cms-s390, crexx-cms-s390, regina-linux-s390</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Owner question 12 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A94" s="2" t="n"/>
       <c r="B94" s="10" t="n"/>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="n"/>
+      <c r="E94" s="5" t="n"/>
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
     </row>
@@ -3361,22 +3368,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B95" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C95" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="n"/>
+      <c r="B95" s="10" t="n"/>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="n"/>
     </row>
@@ -3388,7 +3395,7 @@
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
@@ -3398,7 +3405,7 @@
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E96" s="5" t="n"/>
@@ -3413,17 +3420,17 @@
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C97" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E97" s="5" t="n"/>
@@ -3431,40 +3438,36 @@
       <c r="G97" s="2" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="14" t="n"/>
-      <c r="B98" s="13" t="n"/>
-      <c r="C98" s="14" t="n"/>
-      <c r="D98" s="14" t="n"/>
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Kit 8</t>
+        </is>
+      </c>
       <c r="E98" s="5" t="n"/>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B99" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C99" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E99" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A99" s="14" t="n"/>
+      <c r="B99" s="13" t="n"/>
+      <c r="C99" s="14" t="n"/>
+      <c r="D99" s="14" t="n"/>
+      <c r="E99" s="5" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
     </row>
@@ -3476,17 +3479,17 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E100" s="16" t="inlineStr">
@@ -3505,17 +3508,17 @@
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D101" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
@@ -3534,17 +3537,17 @@
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E102" s="16" t="inlineStr">
@@ -3563,17 +3566,17 @@
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
@@ -3592,17 +3595,17 @@
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C104" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E104" s="16" t="inlineStr">
@@ -3621,20 +3624,24 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="n"/>
     </row>
@@ -3646,17 +3653,17 @@
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C106" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E106" s="5" t="n"/>
@@ -3664,41 +3671,34 @@
       <c r="G106" s="2" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="8" t="n"/>
-      <c r="B107" s="11" t="n"/>
-      <c r="C107" s="8" t="n"/>
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B107" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C107" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="n"/>
+      <c r="F107" s="2" t="n"/>
+      <c r="G107" s="2" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B108" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A108" s="8" t="n"/>
+      <c r="B108" s="11" t="n"/>
+      <c r="C108" s="8" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
@@ -3718,12 +3718,17 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3740,7 @@
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
@@ -3745,7 +3750,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3762,7 +3767,7 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
@@ -3772,7 +3777,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -3789,39 +3794,66 @@
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C112" s="8" t="inlineStr">
+      <c r="C113" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D113" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E113" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
+      <c r="G113" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="8" t="n"/>
-      <c r="B113" s="11" t="n"/>
-      <c r="C113" s="8" t="n"/>
-    </row>
     <row r="114">
-      <c r="A114" s="7" t="n"/>
-      <c r="B114" s="12" t="n"/>
-      <c r="C114" s="7" t="n"/>
+      <c r="A114" s="8" t="n"/>
+      <c r="B114" s="11" t="n"/>
+      <c r="C114" s="8" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="n"/>
+      <c r="B115" s="12" t="n"/>
+      <c r="C115" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.22 TERSE: SPACK compressor (decoder-model encoder, sizes as IBM SPACK), round trips on PC and CMS (tc74); TRS MODULE + TERSE EXEC on the LANG disk; guide; milestone done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3211,12 +3211,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>UNTERSE done: C89 port of the Open Mainframe Project's tersedecompress (Apache 2): PACK and SPACK, host F/V and native, text and binary; PC 120/120 of the testdata (the 4 others are SPACK files with no data); CMS (tc72) byte-identical to the z/OS originals (FB/VB text, binary). UNTRS MODULE + UNTERSE EXEC; Debian unterse. Next: TERSE (compression). languages/terse</t>
+          <t>UNTERSE: C89 port of the Open Mainframe Project's tersedecompress (Apache 2), PACK/SPACK, F/V, text/binary; testdata 120/120; CMS byte-identical to z/OS originals (tc72). TERSE: new SPACK encoder running the decoder's model (longest known phrase), sizes = IBM SPACK within block padding; PC round trip 26 text + 3 binary, CMS round trip (tc74). TRS/UNTRS MODULE + TERSE/UNTERSE EXEC on the LANG disk; Debian terse/unterse. Open: confirm AMATERSE on z/OS reads our SPACK</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.25 spool bridge: vmspoold in Debian, LXCALL/PHONE/MQTT on CMS (pd15 verified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3312,12 +3312,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Owner question 12 Oct (Asterisk); check vmur against our CP first</t>
+          <t>vmspoold (C) in the Debian guest + LXCALL/PHONE/MQTT EXECs on CMS; services echo, sys, phone (Asterisk), mqtt; verified pd15; needed CP fix I-276</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Milestones 9.27-9.31 (LaTeX, troff, Ghostscript, BookMaster, graphical printing); RXPIP files for the Debian guest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G115"/>
+  <dimension ref="A3:G120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3354,119 +3354,170 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n"/>
-      <c r="B94" s="10" t="n"/>
-      <c r="C94" s="2" t="n"/>
-      <c r="D94" s="2" t="n"/>
-      <c r="E94" s="5" t="n"/>
-      <c r="F94" s="2" t="n"/>
-      <c r="G94" s="2" t="n"/>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>9.27</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>LaTeX</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>TeX/LaTeX in the Debian guest (texlive-base, dvips, pdflatex); LATEX EXEC on CMS over the 9.25 bridge: fn TEX in, fn PDF/PS/DVI back as files</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B95" s="10" t="n"/>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="inlineStr">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>9.28</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>troff</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>groff/troff (man, ms, mm) in the Debian guest; TROFF EXEC on CMS over the bridge; text output to the CMS console or printer, PS/PDF as files</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="F95" s="2" t="n"/>
-      <c r="G95" s="2" t="n"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B96" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C96" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E96" s="5" t="n"/>
-      <c r="F96" s="2" t="n"/>
-      <c r="G96" s="2" t="n"/>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>9.29</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Ghostscript, ps2pdf</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C97" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D97" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="n"/>
-      <c r="F97" s="2" t="n"/>
-      <c r="G97" s="2" t="n"/>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>9.30</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BookMaster</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B98" s="13" t="inlineStr">
-        <is>
-          <t>10.3</t>
-        </is>
-      </c>
-      <c r="C98" s="14" t="inlineStr">
-        <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D98" s="14" t="inlineStr">
-        <is>
-          <t>Kit 8</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="n"/>
-      <c r="F98" s="2" t="n"/>
-      <c r="G98" s="2" t="n"/>
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>9.31</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Graphical printing</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="14" t="n"/>
-      <c r="B99" s="13" t="n"/>
-      <c r="C99" s="14" t="n"/>
-      <c r="D99" s="14" t="n"/>
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="10" t="n"/>
+      <c r="C99" s="2" t="n"/>
+      <c r="D99" s="2" t="n"/>
       <c r="E99" s="5" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
@@ -3474,27 +3525,23 @@
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B100" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C100" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="n"/>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E100" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="F100" s="2" t="n"/>
@@ -3503,116 +3550,84 @@
     <row r="101">
       <c r="A101" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E101" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="n"/>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>FreeSWITCH</t>
-        </is>
-      </c>
-      <c r="E102" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="n"/>
       <c r="F102" s="2" t="n"/>
       <c r="G102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>Snapshot</t>
         </is>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
-        </is>
-      </c>
-      <c r="E103" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Kit 8</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="n"/>
       <c r="F103" s="2" t="n"/>
       <c r="G103" s="2" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B104" s="13" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>Container</t>
-        </is>
-      </c>
-      <c r="D104" s="14" t="inlineStr">
-        <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
-        </is>
-      </c>
-      <c r="E104" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A104" s="14" t="n"/>
+      <c r="B104" s="13" t="n"/>
+      <c r="C104" s="14" t="n"/>
+      <c r="D104" s="14" t="n"/>
+      <c r="E104" s="5" t="n"/>
       <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="n"/>
     </row>
@@ -3624,17 +3639,17 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="D105" s="14" t="inlineStr">
-        <is>
-          <t>CFSERV</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
@@ -3653,20 +3668,24 @@
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C106" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D106" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="n"/>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F106" s="2" t="n"/>
       <c r="G106" s="2" t="n"/>
     </row>
@@ -3678,182 +3697,323 @@
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="n"/>
+          <t>FreeSWITCH</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="8" t="n"/>
-      <c r="B108" s="11" t="n"/>
-      <c r="C108" s="8" t="n"/>
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B108" s="13" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="C108" s="14" t="inlineStr">
+        <is>
+          <t>IoT</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>Node-RED</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="n"/>
+      <c r="G108" s="2" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="8" t="inlineStr">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B109" s="13" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>Container</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="n"/>
+      <c r="G109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E110" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="n"/>
+      <c r="G110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B111" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C111" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="n"/>
+      <c r="F111" s="2" t="n"/>
+      <c r="G111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B112" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C112" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>Kit 9</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="n"/>
+      <c r="F112" s="2" t="n"/>
+      <c r="G112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="n"/>
+      <c r="B113" s="11" t="n"/>
+      <c r="C113" s="8" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="B109" s="11" t="inlineStr">
+      <c r="B114" s="11" t="inlineStr">
         <is>
           <t>12a</t>
         </is>
       </c>
-      <c r="C109" s="8" t="inlineStr">
+      <c r="C114" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D114" t="inlineStr">
         <is>
           <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E114" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr">
+      <c r="G114" t="inlineStr">
         <is>
           <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="8" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="B110" s="11" t="inlineStr">
+      <c r="B115" s="11" t="inlineStr">
         <is>
           <t>12b</t>
         </is>
       </c>
-      <c r="C110" s="8" t="inlineStr">
+      <c r="C115" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E115" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="8" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="B111" s="11" t="inlineStr">
+      <c r="B116" s="11" t="inlineStr">
         <is>
           <t>12c</t>
         </is>
       </c>
-      <c r="C111" s="8" t="inlineStr">
+      <c r="C116" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D116" t="inlineStr">
         <is>
           <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E116" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="8" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="B112" s="11" t="inlineStr">
+      <c r="B117" s="11" t="inlineStr">
         <is>
           <t>12d</t>
         </is>
       </c>
-      <c r="C112" s="8" t="inlineStr">
+      <c r="C117" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D117" t="inlineStr">
         <is>
           <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E117" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="8" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="B113" s="11" t="inlineStr">
+      <c r="B118" s="11" t="inlineStr">
         <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C113" s="8" t="inlineStr">
+      <c r="C118" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D118" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="E118" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr">
+      <c r="G118" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="8" t="n"/>
-      <c r="B114" s="11" t="n"/>
-      <c r="C114" s="8" t="n"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="7" t="n"/>
-      <c r="B115" s="12" t="n"/>
-      <c r="C115" s="7" t="n"/>
+    <row r="119">
+      <c r="A119" s="8" t="n"/>
+      <c r="B119" s="11" t="n"/>
+      <c r="C119" s="8" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="n"/>
+      <c r="B120" s="12" t="n"/>
+      <c r="C120" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.26 RXPIP done: RXPIP RUN DEMO on CMS through the bridge (pd19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3344,12 +3344,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Owner question 12 Oct</t>
+          <t>rxpip server+client in Debian (Regina, rxpipd.py, minicurl), vmspoold service rxpip; CMS RXPIP AVAIL/SEARCH/SHOW/BUILD/RUN/GET verified pd19 (RXPIP RUN DEMO works); TAR for CMS not needed (Linux unpacks); open: PUBLISH from CMS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.28 troff done (TROFF EXEC), 9.31 printing by spool (PSPRINT EXEC + tools/psprint.py), verified pd19
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3408,12 +3408,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Owner request 13 Oct</t>
+          <t>groff (groff-base 1.21 + groff 1.23 ms/me/mm/mom macros) in Debian; TROFF EXEC on CMS: text as fn DOCUMENT, PostScript as fn PS (pd19)</t>
         </is>
       </c>
     </row>
@@ -3504,12 +3504,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Owner request 13 Oct</t>
+          <t>spool path done: PSPRINT EXEC (PRINT LINECOUNT 0) -&gt; 00E -&gt; PC tools/psprint.py extracts PS byte-identical, lp/raw 9100/ps2pdf (pd19); bridge path needs Ghostscript in Debian (9.29)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.29 Ghostscript in the Debian guest, 9.31 graphical printing by spool and by bridge (verified pd19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3440,12 +3440,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Owner request 13 Oct</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3504,12 +3504,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>spool path done: PSPRINT EXEC (PRINT LINECOUNT 0) -&gt; 00E -&gt; PC tools/psprint.py extracts PS byte-identical, lp/raw 9100/ps2pdf (pd19); bridge path needs Ghostscript in Debian (9.29)</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.30 bookie: BookMaster-compatible formatter (BOOKIE EXEC), verified pd19
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3472,12 +3472,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Owner request 13 Oct</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.27 LaTeX: pdfTeX 2023 in the Debian guest, LATEX EXEC on CMS (verified pd19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3376,12 +3376,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Owner request 13 Oct</t>
+          <t>TeX Live 2023 pdfTeX (latex/pdflatex), dvips, makeindex cross-built (wc++ for wheezy C++), 24 MB texmf, formats made on the PC; LATEX EXEC: fn PS back to CMS or PDF; verified pd19 (LATEX HELLO -&gt; PSPRINT -&gt; PDF)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.14 TELL: CMS TELL EXEC (local and AT LINUX), Linux tell + setuid vmmsg, vmspoold tell handler; on 19D and LANG
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2370,13 +2370,13 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>mosquitto on Debian done</t>
+          <t>MQTT on CMS done (MQTT EXEC over the spool bridge, both directions, pd15); mosquitto on Debian. MQ-style queues still open.</t>
         </is>
       </c>
     </row>
@@ -2931,13 +2931,13 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct</t>
+          <t>13 Oct: TELL EXEC (CP MSG local; TELL user AT LINUX via the spool bridge, message as input cards; prompt mode for long text, I-277); Linux tell + setuid vmmsg (CP MSG with the Linux user's name); messages kept in /var/spool/vmspool/msg. On 19D and LANG. RSCS remote and the PC client (BORDER) follow with 9.13b/9.12c.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.32 TELL to and from the internet over MQTT (tellnet, tellgw, logins + ACL, netfwd.py --tls, nettell.py); milestones xlsx: 9.32, kit rows renamed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G120"/>
+  <dimension ref="A3:G121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3514,36 +3514,48 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n"/>
-      <c r="B99" s="10" t="n"/>
-      <c r="C99" s="2" t="n"/>
-      <c r="D99" s="2" t="n"/>
-      <c r="E99" s="5" t="n"/>
-      <c r="F99" s="2" t="n"/>
-      <c r="G99" s="2" t="n"/>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A100" s="2" t="n"/>
       <c r="B100" s="10" t="n"/>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C100" s="2" t="n"/>
+      <c r="D100" s="2" t="n"/>
+      <c r="E100" s="5" t="n"/>
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="n"/>
     </row>
@@ -3553,22 +3565,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B101" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C101" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D101" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="n"/>
+      <c r="B101" s="10" t="n"/>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="n"/>
     </row>
@@ -3580,7 +3592,7 @@
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
@@ -3590,7 +3602,7 @@
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E102" s="5" t="n"/>
@@ -3605,17 +3617,17 @@
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>Kit 8</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E103" s="5" t="n"/>
@@ -3623,40 +3635,36 @@
       <c r="G103" s="2" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="14" t="n"/>
-      <c r="B104" s="13" t="n"/>
-      <c r="C104" s="14" t="n"/>
-      <c r="D104" s="14" t="n"/>
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B104" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E104" s="5" t="n"/>
       <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B105" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C105" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E105" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A105" s="14" t="n"/>
+      <c r="B105" s="13" t="n"/>
+      <c r="C105" s="14" t="n"/>
+      <c r="D105" s="14" t="n"/>
+      <c r="E105" s="5" t="n"/>
       <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="n"/>
     </row>
@@ -3668,17 +3676,17 @@
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C106" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E106" s="16" t="inlineStr">
@@ -3697,17 +3705,17 @@
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D107" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
@@ -3726,17 +3734,17 @@
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C108" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E108" s="16" t="inlineStr">
@@ -3755,17 +3763,17 @@
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C109" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D109" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
@@ -3784,17 +3792,17 @@
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E110" s="16" t="inlineStr">
@@ -3813,20 +3821,24 @@
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E111" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
     </row>
@@ -3838,17 +3850,17 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Kit 9</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E112" s="5" t="n"/>
@@ -3856,41 +3868,34 @@
       <c r="G112" s="2" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="8" t="n"/>
-      <c r="B113" s="11" t="n"/>
-      <c r="C113" s="8" t="n"/>
+      <c r="A113" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C113" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="n"/>
+      <c r="F113" s="2" t="n"/>
+      <c r="G113" s="2" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B114" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A114" s="8" t="n"/>
+      <c r="B114" s="11" t="n"/>
+      <c r="C114" s="8" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
@@ -3900,7 +3905,7 @@
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
@@ -3910,12 +3915,17 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3937,7 @@
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
@@ -3937,7 +3947,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -3954,7 +3964,7 @@
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
@@ -3964,7 +3974,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -3981,39 +3991,66 @@
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C118" s="8" t="inlineStr">
+      <c r="C119" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D119" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
+      <c r="E119" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr">
+      <c r="G119" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="8" t="n"/>
-      <c r="B119" s="11" t="n"/>
-      <c r="C119" s="8" t="n"/>
-    </row>
     <row r="120">
-      <c r="A120" s="7" t="n"/>
-      <c r="B120" s="12" t="n"/>
-      <c r="C120" s="7" t="n"/>
+      <c r="A120" s="8" t="n"/>
+      <c r="B120" s="11" t="n"/>
+      <c r="C120" s="8" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="n"/>
+      <c r="B121" s="12" t="n"/>
+      <c r="C121" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.13d NICOF done: README, Guide section, kit integration; kit README build 11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2836,13 +2836,13 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Test before 9.5 (CMS sockets + httpd)</t>
+          <t>13 Oct (ncf3): NICOF 0.7.0 installed -- NICOFSRC/NICOFPXY/TCPIPPXY (VM50U1 61-70, ECMODE), NCFACC on 19E, AUTOLOG1 starts the proxies, 3270 groups 03CD/03CE, PC side vm370plus/nicof (nicof.jar, nicof.sh). NHFS LIST/GET/PUT, CMSFTPD with Python ftplib: LIST, 837 files, text STOR/RETR, 67 KB binary with FF EF round trip identical (~12 KB/s). Found I-283 (STNSM in BC mode, fixed in CP).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.33 CP/M 2.2: RunCPM in the Debian guest (runcpm, cpm service) and natively on CMS (RUNCPM MODULE, CPM EXEC, CP/M programs on L:); M13 MVS rows; Guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G121"/>
+  <dimension ref="A3:G122"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3551,36 +3551,48 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n"/>
-      <c r="B100" s="10" t="n"/>
-      <c r="C100" s="2" t="n"/>
-      <c r="D100" s="2" t="n"/>
-      <c r="E100" s="5" t="n"/>
-      <c r="F100" s="2" t="n"/>
-      <c r="G100" s="2" t="n"/>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>9.33</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CP/M</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A101" s="2" t="n"/>
       <c r="B101" s="10" t="n"/>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C101" s="2" t="n"/>
+      <c r="D101" s="2" t="n"/>
+      <c r="E101" s="5" t="n"/>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="n"/>
     </row>
@@ -3590,22 +3602,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B102" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C102" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D102" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="n"/>
+      <c r="B102" s="10" t="n"/>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F102" s="2" t="n"/>
       <c r="G102" s="2" t="n"/>
     </row>
@@ -3617,7 +3629,7 @@
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
@@ -3627,7 +3639,7 @@
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E103" s="5" t="n"/>
@@ -3642,17 +3654,17 @@
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C104" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E104" s="5" t="n"/>
@@ -3660,40 +3672,36 @@
       <c r="G104" s="2" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="14" t="n"/>
-      <c r="B105" s="13" t="n"/>
-      <c r="C105" s="14" t="n"/>
-      <c r="D105" s="14" t="n"/>
+      <c r="A105" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B105" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E105" s="5" t="n"/>
       <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B106" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C106" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E106" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A106" s="14" t="n"/>
+      <c r="B106" s="13" t="n"/>
+      <c r="C106" s="14" t="n"/>
+      <c r="D106" s="14" t="n"/>
+      <c r="E106" s="5" t="n"/>
       <c r="F106" s="2" t="n"/>
       <c r="G106" s="2" t="n"/>
     </row>
@@ -3705,17 +3713,17 @@
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
@@ -3734,17 +3742,17 @@
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C108" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D108" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E108" s="16" t="inlineStr">
@@ -3763,17 +3771,17 @@
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C109" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D109" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
@@ -3792,17 +3800,17 @@
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E110" s="16" t="inlineStr">
@@ -3821,17 +3829,17 @@
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
@@ -3850,20 +3858,24 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E112" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
     </row>
@@ -3875,17 +3887,17 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D113" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E113" s="5" t="n"/>
@@ -3893,41 +3905,34 @@
       <c r="G113" s="2" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="n"/>
-      <c r="B114" s="11" t="n"/>
-      <c r="C114" s="8" t="n"/>
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B114" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C114" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="n"/>
+      <c r="F114" s="2" t="n"/>
+      <c r="G114" s="2" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B115" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C115" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A115" s="8" t="n"/>
+      <c r="B115" s="11" t="n"/>
+      <c r="C115" s="8" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
@@ -3937,7 +3942,7 @@
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
@@ -3947,12 +3952,17 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3974,7 @@
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
@@ -3974,7 +3984,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -3991,7 +4001,7 @@
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
@@ -4001,7 +4011,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4018,39 +4028,120 @@
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
           <t>12e</t>
         </is>
       </c>
-      <c r="C119" s="8" t="inlineStr">
+      <c r="C120" s="8" t="inlineStr">
         <is>
           <t>DOS/VSE</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr">
+      <c r="D120" t="inlineStr">
         <is>
           <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
+      <c r="E120" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="G120" t="inlineStr">
         <is>
           <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="8" t="n"/>
-      <c r="B120" s="11" t="n"/>
-      <c r="C120" s="8" t="n"/>
-    </row>
     <row r="121">
-      <c r="A121" s="7" t="n"/>
-      <c r="B121" s="12" t="n"/>
-      <c r="C121" s="7" t="n"/>
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>13b</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>MVS 31-bit</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:G73"/>

</xml_diff>

<commit_message>
9.5: HTTPD web server on CMS works (NICOF client rebuilt with CE GCC, INTRAPI for CE GCCLIB frames); I-285
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2308,11 +2308,15 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F62" s="2" t="n"/>
-      <c r="G62" s="2" t="n"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>13 Oct (http3): HTTPD on CMS (CE GCC + NICOF client rebuilt with CE GCC, INTRAPI for CE frames): GET /, /INDEX.HTML, /HTTPD.C, 404 verified with curl from the PC. Open: IPL 290 (I-285), install on N/LANG, the kit; a socket library for GCC 13 (cmsrt) next.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">

</xml_diff>

<commit_message>
9.7: MQ for CMS -- message queues on RabbitMQ (rabbitmq-c 0.11 ported to GCC 13 + NICOF sockets); MQ EXEC, MQTEST; on the language disk; Guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2374,13 +2374,13 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>MQTT on CMS done (MQTT EXEC over the spool bridge, both directions, pd15); mosquitto on Debian. MQ-style queues still open.</t>
+          <t>MQTT on CMS (MQTT EXEC over the spool bridge, pd15) and mosquitto on Debian; 14 Oct: MQ-style queues on RabbitMQ for CMS (MQ EXEC + MQAMQP: rabbitmq-c 0.11 with GCC 13 on NICOF sockets; PUT/GET/DEPTH/PURGE, GET onto the stack; verified against RabbitMQ 3.12 on the PC, runs mq1/mq2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b14 prep: README (new Debian disk, PGSQL, MQ, rxpip, CP CTC scheduler fixes), LANG README with PGSQL, Guide entry, milestones 9.4 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2275,13 +2275,13 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>SQLite 3.46.1 on CMS (SQLITE EXEC) and the SQLSERV service machine (tc47, 12 Oct). 14 Oct: PostgreSQL 16.15 cross-built for the 31-bit Debian guest (linux390/pgsql/mkpg.sh) and running there (initdb, init script; small settings for 64 MB); PGSQL EXEC on CMS over the spool bridge (each CMS user its own role and database; statements cut at blanks outside quotes for the 80-column cards): CREATE/INSERT/SELECT verified (run pg1). Open: the Debian disk (3390-1) is 97% full -- moving it to the 3390-9; SQLSERV in the kit; MariaDB not planned (C++, too big for 64 MB).</t>
+          <t>SQLite 3.46.1 on CMS (SQLITE EXEC) and the SQLSERV service machine (tc47, 12 Oct). 14 Oct: PostgreSQL 16.15 cross-built for the 31-bit Debian guest (linux390/pgsql/mkpg.sh), started at boot; PGSQL EXEC on CMS over the spool bridge (each CMS user its own role and database): CREATE/INSERT/SELECT verified (pg1); PGSQL on LANG; the Debian disk moved to the 3390-9 (5.8 GB free, bt1: PostgreSQL runs). Kit b14. MariaDB not planned (C++, too big for 64 MB).</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Needed for DHCP: CTC links are point-to-point</t>
+          <t>Needed for DHCP: CTC links are point-to-point. 14 Oct, I-287 (a CTCA star between Linux guests, one way to 9.12b): five CP causes fixed (lock across DMKVCA's wait, cc 1 as pending status, buffers above 16 MB, two scheduler bugs that kept CTC guests in the queue); the Linux-to-Linux link does not connect yet. Choice of approach (CP Guest LAN / CTCA star / LCS+bridge) asked of Mike.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Milestones 9.34/9.35: NetRexx on Debian and on CMS (JamVM + GNU Classpath)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G122"/>
+  <dimension ref="A3:G124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3429,27 +3429,27 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.34</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>NetRexx (Linux)</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>NetRexx in the Debian guest: a Java VM first -- JamVM with the GNU Classpath library (C parts cross-built with wcc, the Java parts built on the PC), NetRexx (RexxLA/netrexx) built on the PC for that VM; nrc/nr: interpret (-exec) and compile</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Mike 14 Oct: NetRexx for both Linux and CMS. Sources from GitHub (RexxLA/netrexx, a GNU Classpath mirror, JamVM); archive.debian.org (OpenJDK 7) is not reachable from the build machine</t>
         </is>
       </c>
     </row>
@@ -3461,27 +3461,27 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.35</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>NetRexx (CMS)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>NetRexx on CMS: the same JamVM + GNU Classpath built with GCC 13 for the EC-mode CMS (IPL 290, above 16 MB, single-threaded), the class library read from the LANG disk; NETREXX EXEC (interpret, then compile)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>After 9.34 (same VM and library); needs no C++</t>
         </is>
       </c>
     </row>
@@ -3493,17 +3493,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3525,17 +3525,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -3543,14 +3543,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3562,90 +3557,109 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
+          <t>9.31</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Graphical printing</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
+      <c r="G102" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="2" t="n"/>
-      <c r="B101" s="10" t="n"/>
-      <c r="C101" s="2" t="n"/>
-      <c r="D101" s="2" t="n"/>
-      <c r="E101" s="5" t="n"/>
-      <c r="F101" s="2" t="n"/>
-      <c r="G101" s="2" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B102" s="10" t="n"/>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="n"/>
-      <c r="G102" s="2" t="n"/>
-    </row>
     <row r="103">
-      <c r="A103" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B103" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C103" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D103" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
+      <c r="A103" s="2" t="n"/>
+      <c r="B103" s="10" t="n"/>
+      <c r="C103" s="2" t="n"/>
+      <c r="D103" s="2" t="n"/>
       <c r="E103" s="5" t="n"/>
       <c r="F103" s="2" t="n"/>
       <c r="G103" s="2" t="n"/>
@@ -3656,22 +3670,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B104" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D104" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="n"/>
+      <c r="B104" s="10" t="n"/>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="n"/>
     </row>
@@ -3683,17 +3697,17 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E105" s="5" t="n"/>
@@ -3701,10 +3715,26 @@
       <c r="G105" s="2" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="14" t="n"/>
-      <c r="B106" s="13" t="n"/>
-      <c r="C106" s="14" t="n"/>
-      <c r="D106" s="14" t="n"/>
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B106" s="13" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
       <c r="E106" s="5" t="n"/>
       <c r="F106" s="2" t="n"/>
       <c r="G106" s="2" t="n"/>
@@ -3712,58 +3742,34 @@
     <row r="107">
       <c r="A107" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E107" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="n"/>
       <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B108" s="13" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="C108" s="14" t="inlineStr">
-        <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E108" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A108" s="14" t="n"/>
+      <c r="B108" s="13" t="n"/>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="14" t="n"/>
+      <c r="E108" s="5" t="n"/>
       <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="n"/>
     </row>
@@ -3775,17 +3781,17 @@
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C109" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D109" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
@@ -3804,17 +3810,17 @@
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D110" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E110" s="16" t="inlineStr">
@@ -3833,17 +3839,17 @@
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
@@ -3862,17 +3868,17 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E112" s="16" t="inlineStr">
@@ -3891,20 +3897,24 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D113" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="n"/>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E113" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
     </row>
@@ -3916,86 +3926,81 @@
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D114" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E114" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="8" t="n"/>
-      <c r="B115" s="11" t="n"/>
-      <c r="C115" s="8" t="n"/>
+      <c r="A115" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B115" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C115" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="n"/>
+      <c r="F115" s="2" t="n"/>
+      <c r="G115" s="2" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B116" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="n"/>
+      <c r="F116" s="2" t="n"/>
+      <c r="G116" s="2" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B117" s="11" t="inlineStr">
-        <is>
-          <t>12b</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A117" s="8" t="n"/>
+      <c r="B117" s="11" t="n"/>
+      <c r="C117" s="8" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
@@ -4005,7 +4010,7 @@
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
@@ -4015,12 +4020,17 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4032,7 +4042,7 @@
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
@@ -4042,7 +4052,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -4059,7 +4069,7 @@
       </c>
       <c r="B120" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
@@ -4069,79 +4079,133 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>12e</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>srorso/dos360install</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
           <t>M13</t>
         </is>
       </c>
-      <c r="B122" s="11" t="inlineStr">
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
         <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C122" s="8" t="inlineStr">
+      <c r="C124" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="D124" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr">
+      <c r="E124" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr">
+      <c r="G124" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
9.35: Java and NetRexx run on CMS (JamVM XIMAGE); mmap page rounding (GC list overrun), getcwd '/', XL loader trims its heap, sbrk shrink; I-289 fixed (XL fstat plist above 16 MB); I-290 opened (PGS001 at logoff); gotchas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3444,12 +3444,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Mike 14 Oct: NetRexx for both Linux and CMS. Sources from GitHub (RexxLA/netrexx, a GNU Classpath mirror, JamVM); archive.debian.org (OpenJDK 7) is not reachable from the build machine</t>
+          <t>JamVM 2.0 + GNU Classpath 0.99 + NetRexx 3.05 run in the Debian guest: nrc -exec hello OK (14 Oct, kt29; 22 min in a 59 MB guest -- paging). Next: install on the shipped Debian disk, java/nrc/nr wrappers, lower -Xmx, ecj for compiling, Guide, kit.</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3476,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>After 9.34 (same VM and library); needs no C++</t>
+          <t>JamVM runs on CMS as JAMVM XIMAGE (XL loader): green-thread pthreads + signal emulation, generated JNI stubs (no libffi), Classpath natives, fdlibm, zlib. Java test program OK on CMS (threads, collections, file I/O, GC; ~2.5 s CPU). NetRexxC starts; open: corrupted bytecode while preparing DateFormatSymbols (memory overlap under investigation). Fixed on the way: I-289 (XL fstat plist above 16 MB), sbrk shrink, XL loader keeps only the image's storage.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b16 built: Java/NetRexx on CMS and Debian, I-290 CP fix, MAINT 256M (directory), README parts 1-18, Guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3444,12 +3444,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (kit b16)</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>JamVM 2.0 + GNU Classpath 0.99 + NetRexx 3.05 run in the Debian guest: nrc -exec hello OK (14 Oct, kt29; 22 min in a 59 MB guest -- paging). Next: install on the shipped Debian disk, java/nrc/nr wrappers, lower -Xmx, ecj for compiling, Guide, kit.</t>
+          <t>Java (JamVM 2.0 + GNU Classpath 0.99), javac (Eclipse ecj 3.5.2), NetRexx 3.05 (nrc compiles with ecj, nr interprets) installed in the Debian guest. Verified 14 Oct on the dev disk at 192 MB: javac+java 287 s, nrc+java 685 s. MAINT may now define 256 MB.</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3476,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (kit b16)</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Java and NetRexx run on CMS (14 Oct): JAVA and NETREXX EXECs, JAMVM XIMAGE via XL; NETREXX HELLO 25 s CPU, JAVA HELLO 3 s. Fixed on the way: mmap page rounding, I-289, I-290 (CP: frames to 128 MB), XL loader trims its heap, opendir('/'), upper-case class names. Left: LANG disk + kit b16, Java compiler (ecj) on CMS.</t>
+          <t>Java and NetRexx on CMS: JAVA, JAVAC (ecj 3.5.2), NETREXX [COMPILE] EXECs; JAMVM XIMAGE (XL). Verified on the fixed CP: JAVAC 27 s CPU, NETREXX interpreted 27 s, COMPILE 45 s, compiled run 3.7 s. Fixed on the way: I-289, I-290 (CP), mmap page rounding, XL heap trim.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b17: CP guest LAN; verified on a fresh CE (kt31)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2609,13 +2609,13 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (kit b17)</t>
         </is>
       </c>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>14 Oct: CP guest LAN (CP DEFINE LCS, module DMKVLN): steps A-D done -- two Linux guests ping each other (lb6), logoff/re-logon/offline-online/DETACH under traffic (lb8), Debian on the LAN with vm370plus-lan, TCP 200 KB intact at ~37 KB/s (lb9). I-292 fixed. Guide section added. Next: kit b17.</t>
+          <t>CP guest LAN: CP DEFINE LCS (3088-60 simulated by CP, module DMKVLN), one segment 10.3.0.0/24, Debian eth0 by vm370plus-lan. Steps A-D tested (lb3-lb11): ping, 1400-byte frames, TCP 200 KB intact (~37 KB/s), logoff/DETACH/offline under traffic. I-292 fixed, I-293 worked around. Kit b17 verified on a fresh CE (kt31).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.12c BORDER: service machine with NAT, firewall and port forwards (kernel #12 + iptables); BORDER EXEC/CONFIG, DIRUP2/3; I-294, I-295
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2642,13 +2642,13 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Outside link may be bridged (LCS on tap) to get its address from the LAN DHCP</t>
+          <t>15 Oct: BORDER service machine (CP AUTOLOG BORDER BORDER): in-storage Linux, kernel #12 (netfilter, iptables 1.4.14), ctc0 10.1.4.2 on CTC pair 0606/0607, eth0 10.3.0.1 on the guest LAN; NAT out, firewall, port forwards from BORDER CONFIG (MAINT 19E). Tested bi2: LAN guest -&gt; PC through NAT, PC -&gt; BORDER:2223 -&gt; guest ssh, unexposed ports dropped. I-294, I-295 found.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b18: BORDER (9.12c); verified on a fresh CE (kt32)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2642,13 +2642,13 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Done (kit b18)</t>
         </is>
       </c>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>15 Oct: BORDER service machine (CP AUTOLOG BORDER BORDER): in-storage Linux, kernel #12 (netfilter, iptables 1.4.14), ctc0 10.1.4.2 on CTC pair 0606/0607, eth0 10.3.0.1 on the guest LAN; NAT out, firewall, port forwards from BORDER CONFIG (MAINT 19E). Tested bi2: LAN guest -&gt; PC through NAT, PC -&gt; BORDER:2223 -&gt; guest ssh, unexposed ports dropped. I-294, I-295 found.</t>
+          <t>BORDER service machine (AUTOLOG BORDER BORDER): in-storage Linux, kernel #12 (netfilter, iptables 1.4.14), ctc0 10.1.4.2 (pair 0606/0607), eth0 10.3.0.1; NAT, firewall, port forwards from BORDER CONFIG (MAINT 19E). Verified on a fresh CE (kt32): LAN guest -&gt; PC through NAT, PC -&gt; 10.1.4.2:2223 -&gt; guest ssh.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.12d: DHCP (udhcpd) and DNS forwarding on BORDER; udhcpc/dhclient on guests; Guide, README build 19; I-296
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2675,13 +2675,13 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Needs 9.12b</t>
+          <t>15 Oct: BORDER runs busybox udhcpd on the LAN (10.3.0.100-199, router and DNS 10.3.0.1) and forwards 10.3.0.1:53 to vmdns= (BORDER CONFIG 'DNS a.b.c.d', default the PC 10.1.4.1). In-storage guests use udhcpc, Debian dhclient when it has no address. Tested dh1 (ramdisk guest 10.3.0.100, nslookup through BORDER) and deb13 (Debian lease from BORDER).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Milestones: 9.12 network pack done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2539,13 +2539,13 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (kit b19)</t>
         </is>
       </c>
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>After M4b.3, before M9</t>
+          <t>Network pack 9.12a-d done: per-user addresses, CP guest LAN, BORDER (NAT, firewall, port forwards), DHCP/DNS.</t>
         </is>
       </c>
     </row>
@@ -2675,13 +2675,13 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Done (kit b19)</t>
         </is>
       </c>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>15 Oct: BORDER runs busybox udhcpd on the LAN (10.3.0.100-199, router and DNS 10.3.0.1) and forwards 10.3.0.1:53 to vmdns= (BORDER CONFIG 'DNS a.b.c.d', default the PC 10.1.4.1). In-storage guests use udhcpc, Debian dhclient when it has no address. Tested dh1 (ramdisk guest 10.3.0.100, nslookup through BORDER) and deb13 (Debian lease from BORDER).</t>
+          <t>BORDER: udhcpd (10.3.0.100-199, router/DNS 10.3.0.1), DNS forwarding to BORDER CONFIG's DNS (default the PC 10.1.4.1); udhcpc in the in-storage Linux, dhclient in Debian. Verified on a fresh CE (kt33).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M8.2: native cREXX build with GCC 13 on CMS (mknat.sh, CRX82 EXEC); milestones 9.36 MCproject, 9.37 Regina, 9.38 MChelpdesk
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G124"/>
+  <dimension ref="A3:G127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3493,27 +3493,32 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.36</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>Project mgmt (MCproject)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>Our own project management system, MCproject (mikebeer/MCproject, under way), on VM/370plus: the server in the Debian guest, reached from the LAN and, through BORDER, from the PC (vmfwd); a CMS front end where it fits (spool bridge or native)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Owner decision 15 Oct: our own system instead of OpenProject (current OpenProject needs Ruby 4.0, Node 24, PostgreSQL 16+, 1 GB RAM, 64-bit: out of reach of the 31-bit Debian 7 guest). The repository is still empty (15 Oct); the VM/370plus port follows its design: language and database to be matched to what runs here (C/C++ GCC 13, Python 2.7/3.2, Regina, PostgreSQL 9.1 or SQLite 3.46 on both sides)</t>
         </is>
       </c>
     </row>
@@ -3525,27 +3530,32 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.37</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>REXX (Regina)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Regina REXX on both sides: (a) Linux: Regina 3.6 in the Debian guest (wheezy package, `regina`/`rexx`); (b) CMS: Regina built natively with GCC 13 and the M5f runtime (cmsrt), REGINA MODULE/XIMAGE on the LANG disk, a REGINA EXEC front end (`REGINA fn [ft]` runs a REXX program from a CMS file), ADDRESS CMS/COMMAND passing commands to CMS (SVC 202), stream I/O on CMS files</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Owner request 15 Oct. (a) Done 10 Oct (installed with THE; used by rxpip, 9.26) -- had no row of its own. (b) Planned: Regina 3.9.x source (LGPL), the toolchain route of 9.21-9.23 (cmscc cross build first, then on CMS); beside the other REXX implementations: CMS REXX/BREXX (CE), cREXX 2022 (M5) and current (M8), NetRexx (9.34/9.35), ooRexx 5 (9.9, Debian)</t>
         </is>
       </c>
     </row>
@@ -3557,27 +3567,32 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.38</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>Helpdesk (MChelpdesk)</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>Our own helpdesk / trouble-ticket system, MChelpdesk (mikebeer/MChelpdesk), on VM/370plus: the server in the Debian guest beside MCproject (9.36), reached from the LAN and, through BORDER, from the PC; tickets from CMS users (a TICKET EXEC over the spool bridge or MSG/reader), mail notification once 9.18 exists</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>Owner request 15 Oct. Follows the MChelpdesk design; shares platform choices with 9.36 (language/database matched to what runs on VM/370plus)</t>
         </is>
       </c>
     </row>
@@ -3589,17 +3604,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3607,14 +3622,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3626,115 +3636,141 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
+          <t>9.30</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BookMaster</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>9.31</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Graphical printing</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D105" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr">
+      <c r="G105" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="2" t="n"/>
-      <c r="B103" s="10" t="n"/>
-      <c r="C103" s="2" t="n"/>
-      <c r="D103" s="2" t="n"/>
-      <c r="E103" s="5" t="n"/>
-      <c r="F103" s="2" t="n"/>
-      <c r="G103" s="2" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B104" s="10" t="n"/>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="n"/>
-      <c r="G104" s="2" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B105" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C105" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D105" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="n"/>
-      <c r="F105" s="2" t="n"/>
-      <c r="G105" s="2" t="n"/>
-    </row>
     <row r="106">
-      <c r="A106" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B106" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C106" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D106" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
+      <c r="A106" s="2" t="n"/>
+      <c r="B106" s="10" t="n"/>
+      <c r="C106" s="2" t="n"/>
+      <c r="D106" s="2" t="n"/>
       <c r="E106" s="5" t="n"/>
       <c r="F106" s="2" t="n"/>
       <c r="G106" s="2" t="n"/>
@@ -3745,30 +3781,46 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B107" s="13" t="inlineStr">
-        <is>
-          <t>10.3</t>
-        </is>
-      </c>
-      <c r="C107" s="14" t="inlineStr">
-        <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="D107" s="14" t="inlineStr">
-        <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="n"/>
+      <c r="B107" s="10" t="n"/>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="14" t="n"/>
-      <c r="B108" s="13" t="n"/>
-      <c r="C108" s="14" t="n"/>
-      <c r="D108" s="14" t="n"/>
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B108" s="13" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="C108" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
+        </is>
+      </c>
       <c r="E108" s="5" t="n"/>
       <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="n"/>
@@ -3776,87 +3828,59 @@
     <row r="109">
       <c r="A109" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C109" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E109" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="n"/>
       <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E110" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="n"/>
       <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B111" s="13" t="inlineStr">
-        <is>
-          <t>11.3</t>
-        </is>
-      </c>
-      <c r="C111" s="14" t="inlineStr">
-        <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D111" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
-        </is>
-      </c>
-      <c r="E111" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A111" s="14" t="n"/>
+      <c r="B111" s="13" t="n"/>
+      <c r="C111" s="14" t="n"/>
+      <c r="D111" s="14" t="n"/>
+      <c r="E111" s="5" t="n"/>
       <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
     </row>
@@ -3868,17 +3892,17 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D112" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E112" s="16" t="inlineStr">
@@ -3897,17 +3921,17 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
-        </is>
-      </c>
-      <c r="D113" s="14" t="inlineStr">
-        <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
@@ -3926,17 +3950,17 @@
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D114" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E114" s="16" t="inlineStr">
@@ -3955,20 +3979,24 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D115" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="n"/>
+          <t>Node-RED</t>
+        </is>
+      </c>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F115" s="2" t="n"/>
       <c r="G115" s="2" t="n"/>
     </row>
@@ -3980,113 +4008,110 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D116" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
-        </is>
-      </c>
-      <c r="E116" s="5" t="n"/>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E116" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="8" t="n"/>
-      <c r="B117" s="11" t="n"/>
-      <c r="C117" s="8" t="n"/>
+      <c r="A117" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D117" s="14" t="inlineStr">
+        <is>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="n"/>
+      <c r="G117" s="2" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B118" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A118" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B118" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C118" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="n"/>
+      <c r="F118" s="2" t="n"/>
+      <c r="G118" s="2" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B119" s="11" t="inlineStr">
-        <is>
-          <t>12b</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A119" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="n"/>
+      <c r="F119" s="2" t="n"/>
+      <c r="G119" s="2" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B120" s="11" t="inlineStr">
-        <is>
-          <t>12c</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A120" s="8" t="n"/>
+      <c r="B120" s="11" t="n"/>
+      <c r="C120" s="8" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
@@ -4096,7 +4121,7 @@
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
@@ -4106,12 +4131,17 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4153,7 @@
       </c>
       <c r="B122" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
@@ -4133,79 +4163,160 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>12d</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>12e</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>srorso/dos360install</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
           <t>M13</t>
         </is>
       </c>
-      <c r="B124" s="11" t="inlineStr">
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
         <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C124" s="8" t="inlineStr">
+      <c r="C127" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="D127" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
+      <c r="E127" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr">
+      <c r="G127" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
M8.2 done: current cREXX built natively on CMS with GCC 13 (RXC82, RXAS82, RXBVM82; hello and library test pass); kit LANG gets them; Guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2126,7 +2126,7 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>RXC/RXAS work; RXBVM82 open</t>
+          <t>15 Oct, route 2 (GCC 13 on CMS, 9.21): all 113 units compiled by cc1 on CMS (CRX82 EXEC, m8/native/mknat.sh), linked by ld there: RXC82, RXAS82, RXBVM82 MODULE. Run n83g: C82HELLO compiled/assembled/run (sum 1..10 = 55), C82LIB with library functions (length/reverse via LIBRARY RXBIN). Fixes on the way: cmsrt file buffers sized from the FST, heap = largest HIGHSTOR piece, XL loads the image before the file buffer, VFS literal ../ paths, cc1 GC params, handler panel 1, scanners from upstream's S370 encoding (rexbscan 3.2 MB -&gt; 169 KB). Open: CMS ar cannot write an archive (temp file), RXC link takes the members the PC map names</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.37 Regina on CMS works (REGINA on LANG); 9.9 ooRexx 5.3 in the Debian guest; Guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2444,11 +2444,15 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>15 Oct: ooRexx 5.3.0 (github ooRexx/ooRexx) cross-built for 31-bit s390 Linux with s390x g++ -m31 against the lx31 glibc 2.39 sysroot, libstdc++/libgcc static, own /opt/oorexx/lib/ld.so.1 + libc (Debian 7's glibc 2.13 is too old); ncurses extension skipped. Installed in the Debian guest over ssh (run rx1), rexx.img made there by rexximage (50 s); rexx -v: 5.3.0, 32-bit; arrays, directories, DateTime, 2**64, NUMERIC DIGITS 30 tested. oorexx/oorexxc in /usr/local/bin (rexx stays Regina)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
@@ -3545,7 +3549,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -3555,7 +3559,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct. (a) Done 10 Oct (installed with THE; used by rxpip, 9.26) -- had no row of its own. (b) Planned: Regina 3.9.x source (LGPL), the toolchain route of 9.21-9.23 (cmscc cross build first, then on CMS); beside the other REXX implementations: CMS REXX/BREXX (CE), cREXX 2022 (M5) and current (M8), NetRexx (9.34/9.35), ooRexx 5 (9.9, Debian). 15 Oct, first cross build: Regina 3.9.5 source (github 0branch/regina mirror), configure with m5f/cmscc works; needs -DNO_EXTERNAL_QUEUES (no sockets) and REGINA_BITS 32, and an OS layer for CMS (os_unx.c assumes fork/exec, uname): ADDRESS CMS/COMMAND by SVC 202 -- open design point: a MODULE command loads at X'20000' over a running MODULE, so Regina runs as an XIMAGE (XL, above 16 MB) and the SVC 202 path must not depend on code in the user area</t>
+          <t>15 Oct. (a) Linux: Regina 3.6 in Debian since 10 Oct. (b) CMS: Regina 3.9.5 cross-built (languages/regina/mkregina.sh: generic OS layer patched for CMS, no external queues, 32-bit), REGINA MODULE on LANG (TEXT + LANGGEN). Run rx3: PARSE VERSION/SOURCE (CMS COMMAND), arithmetic, NUMERIC DIGITS 40, ADDRESS COMMAND STATE/LISTFILE/QUERY DISK rc 0, CP QUERY USERID, LINEOUT/LINEIN on a CMS file. cmsrt got system() (SVC 202, tokenised plist). Limits: commands that are user-area MODULEs would overlay REGINA; 8-character tokens (CMS plist); the X'01' command flag made CMS's CP routine fail (spec. exception), so plain SVC 202</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Milestones: 9.39 REXX dispatch (/*!name), 9.40 local DNS zone
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G127"/>
+  <dimension ref="A3:G129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3608,27 +3608,32 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.39</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>REXX dispatch (/*!)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>CMS EXEC dispatch by first line: /*!name options */ (still a REXX comment) selects the interpreter (BREXX, REGINA, RXC/cREXX, EXEC); plain /* goes to a settable default (SET REXX BREXX|REGINA). Regina as a selectable default once it is resident in high storage (NUCXLOAD), supports ADDRESS CMS/COMMAND/XEDIT, EXECIO and the stack, and calls user-area MODULEs</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Owner request 15 Oct. Hook: DMSEXC first-record check (NUCBREXX). BREXX stays default until Regina passes the BREXX test EXECs</t>
         </is>
       </c>
     </row>
@@ -3640,27 +3645,32 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.40</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Local DNS zone</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Names for VM/370plus guests and services: an authoritative zone on BORDER (dnsmasq or similar) next to the DNS forwarder of 9.12d -- guest names, and the domain and MX record mail (9.18) needs</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Owner request 15 Oct; before or with 9.18</t>
         </is>
       </c>
     </row>
@@ -3672,17 +3682,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -3692,7 +3702,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3704,17 +3714,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3722,14 +3732,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3741,90 +3746,109 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
+          <t>9.31</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Graphical printing</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D107" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
+      <c r="G107" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="2" t="n"/>
-      <c r="B106" s="10" t="n"/>
-      <c r="C106" s="2" t="n"/>
-      <c r="D106" s="2" t="n"/>
-      <c r="E106" s="5" t="n"/>
-      <c r="F106" s="2" t="n"/>
-      <c r="G106" s="2" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B107" s="10" t="n"/>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="n"/>
-      <c r="G107" s="2" t="n"/>
-    </row>
     <row r="108">
-      <c r="A108" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="B108" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C108" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D108" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
+      <c r="A108" s="2" t="n"/>
+      <c r="B108" s="10" t="n"/>
+      <c r="C108" s="2" t="n"/>
+      <c r="D108" s="2" t="n"/>
       <c r="E108" s="5" t="n"/>
       <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="n"/>
@@ -3835,22 +3859,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B109" s="13" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="C109" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D109" s="14" t="inlineStr">
-        <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E109" s="5" t="n"/>
+      <c r="B109" s="10" t="n"/>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="n"/>
     </row>
@@ -3862,17 +3886,17 @@
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E110" s="5" t="n"/>
@@ -3880,10 +3904,26 @@
       <c r="G110" s="2" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="14" t="n"/>
-      <c r="B111" s="13" t="n"/>
-      <c r="C111" s="14" t="n"/>
-      <c r="D111" s="14" t="n"/>
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B111" s="13" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="C111" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
       <c r="E111" s="5" t="n"/>
       <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
@@ -3891,58 +3931,34 @@
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E112" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="n"/>
       <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B113" s="13" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="C113" s="14" t="inlineStr">
-        <is>
-          <t>More Languages</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
-        </is>
-      </c>
-      <c r="E113" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A113" s="14" t="n"/>
+      <c r="B113" s="13" t="n"/>
+      <c r="C113" s="14" t="n"/>
+      <c r="D113" s="14" t="n"/>
+      <c r="E113" s="5" t="n"/>
       <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
     </row>
@@ -3954,17 +3970,17 @@
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D114" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>Multiprocessor-Support</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E114" s="16" t="inlineStr">
@@ -3983,17 +3999,17 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
-        </is>
-      </c>
-      <c r="D115" s="14" t="inlineStr">
-        <is>
-          <t>Node-RED</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
@@ -4012,17 +4028,17 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D116" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E116" s="16" t="inlineStr">
@@ -4041,17 +4057,17 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D117" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
@@ -4070,20 +4086,24 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D118" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E118" s="5" t="n"/>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+        </is>
+      </c>
+      <c r="E118" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F118" s="2" t="n"/>
       <c r="G118" s="2" t="n"/>
     </row>
@@ -4095,86 +4115,81 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
-        </is>
-      </c>
-      <c r="E119" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E119" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F119" s="2" t="n"/>
       <c r="G119" s="2" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="8" t="n"/>
-      <c r="B120" s="11" t="n"/>
-      <c r="C120" s="8" t="n"/>
+      <c r="A120" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B120" s="13" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C120" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D120" s="14" t="inlineStr">
+        <is>
+          <t>Manual Update</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="n"/>
+      <c r="F120" s="2" t="n"/>
+      <c r="G120" s="2" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B121" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A121" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C121" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="n"/>
+      <c r="F121" s="2" t="n"/>
+      <c r="G121" s="2" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B122" s="11" t="inlineStr">
-        <is>
-          <t>12b</t>
-        </is>
-      </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="A122" s="8" t="n"/>
+      <c r="B122" s="11" t="n"/>
+      <c r="C122" s="8" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
@@ -4184,7 +4199,7 @@
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
@@ -4194,12 +4209,17 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4231,7 @@
       </c>
       <c r="B124" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
@@ -4221,7 +4241,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -4238,7 +4258,7 @@
       </c>
       <c r="B125" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
@@ -4248,79 +4268,133 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B126" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>12e</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>DOS/VSE</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>srorso/dos360install</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
           <t>M13</t>
         </is>
       </c>
-      <c r="B127" s="11" t="inlineStr">
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
         <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C127" s="8" t="inlineStr">
+      <c r="C129" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D129" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E129" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
+      <c r="G129" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
Kit b20: native cREXX (M8.2), Regina on CMS, ooRexx, I-297/I-298; 19 parts; verified on a fresh CE (kt34)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2444,7 +2444,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b20)</t>
         </is>
       </c>
       <c r="F66" s="2" t="n"/>
@@ -3549,7 +3549,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b20)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">

</xml_diff>

<commit_message>
Milestones: 9.41 PC spool reader; 9.13b RSCS/TCPNJE route
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G129"/>
+  <dimension ref="A3:G130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2784,7 +2784,7 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13</t>
+          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13 15 Oct: CE has RSCS V1 (DMT* on 39F, no NJE). Route: TCPNJE (Hercules device, spinhawk README.TCPNJE: 2703 BSC inside, NJE over TCP outside) + the RSCS NJE updates; port tcpnje to our Hercules 3.13; kit users need a Hercules with tcpnje. Partners: other Hercules VM, MVS 3.8 NJE38, funetnje in Debian (9.13c).</t>
         </is>
       </c>
     </row>
@@ -3682,27 +3682,32 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.41</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>PC spool reader</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>Spool decks from the PC (Windows and Linux) into VM/370 spool: a Hercules sockdev card reader in vm370ce.conf, started at IPL, and a small Python tool (vmspool deck USERID) that prefixes an ID card and sends the deck; it arrives in the user's reader. Same for printer output back to the PC. Later: vmur in Linux guests (needs DIAG 14/210 in CP)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Owner request 15 Oct (installation decks from the PC)</t>
         </is>
       </c>
     </row>
@@ -3714,17 +3719,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3734,7 +3739,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3746,17 +3751,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -3766,7 +3771,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3778,17 +3783,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3796,14 +3801,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -3815,66 +3815,78 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D108" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G108" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="2" t="n"/>
-      <c r="B108" s="10" t="n"/>
-      <c r="C108" s="2" t="n"/>
-      <c r="D108" s="2" t="n"/>
-      <c r="E108" s="5" t="n"/>
-      <c r="F108" s="2" t="n"/>
-      <c r="G108" s="2" t="n"/>
-    </row>
     <row r="109">
-      <c r="A109" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A109" s="2" t="n"/>
       <c r="B109" s="10" t="n"/>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E109" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C109" s="2" t="n"/>
+      <c r="D109" s="2" t="n"/>
+      <c r="E109" s="5" t="n"/>
       <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="n"/>
     </row>
@@ -3884,22 +3896,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B110" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C110" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D110" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E110" s="5" t="n"/>
+      <c r="B110" s="10" t="n"/>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="n"/>
     </row>
@@ -3911,7 +3923,7 @@
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
@@ -3921,7 +3933,7 @@
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E111" s="5" t="n"/>
@@ -3936,17 +3948,17 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E112" s="5" t="n"/>
@@ -3954,40 +3966,36 @@
       <c r="G112" s="2" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="14" t="n"/>
-      <c r="B113" s="13" t="n"/>
-      <c r="C113" s="14" t="n"/>
-      <c r="D113" s="14" t="n"/>
+      <c r="A113" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C113" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E113" s="5" t="n"/>
       <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B114" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C114" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E114" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A114" s="14" t="n"/>
+      <c r="B114" s="13" t="n"/>
+      <c r="C114" s="14" t="n"/>
+      <c r="D114" s="14" t="n"/>
+      <c r="E114" s="5" t="n"/>
       <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
     </row>
@@ -3999,17 +4007,17 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
@@ -4028,17 +4036,17 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D116" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E116" s="16" t="inlineStr">
@@ -4057,17 +4065,17 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D117" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
@@ -4086,17 +4094,17 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D118" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E118" s="16" t="inlineStr">
@@ -4115,17 +4123,17 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
@@ -4144,20 +4152,24 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E120" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E120" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F120" s="2" t="n"/>
       <c r="G120" s="2" t="n"/>
     </row>
@@ -4169,17 +4181,17 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E121" s="5" t="n"/>
@@ -4187,41 +4199,34 @@
       <c r="G121" s="2" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="8" t="n"/>
-      <c r="B122" s="11" t="n"/>
-      <c r="C122" s="8" t="n"/>
+      <c r="A122" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B122" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C122" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D122" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="n"/>
+      <c r="F122" s="2" t="n"/>
+      <c r="G122" s="2" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B123" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A123" s="8" t="n"/>
+      <c r="B123" s="11" t="n"/>
+      <c r="C123" s="8" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
@@ -4231,7 +4236,7 @@
       </c>
       <c r="B124" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
@@ -4241,12 +4246,17 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4268,7 @@
       </c>
       <c r="B125" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
@@ -4268,7 +4278,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -4285,7 +4295,7 @@
       </c>
       <c r="B126" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
@@ -4295,7 +4305,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -4312,7 +4322,7 @@
       </c>
       <c r="B127" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -4322,39 +4332,34 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B128" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -4364,7 +4369,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4376,25 +4381,57 @@
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C129" s="8" t="inlineStr">
+      <c r="C130" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="D130" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
+      <c r="G130" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
9.39 step 1: /*!name on an EXEC's first line runs it by that command (DMSEXC XA0057DK, cmsrt =EXEC); Regina rebuilt; Guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2784,7 +2784,7 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13 15 Oct: CE has RSCS V1 (DMT* on 39F, no NJE). Route: TCPNJE (Hercules device, spinhawk README.TCPNJE: 2703 BSC inside, NJE over TCP outside) + the RSCS NJE updates; port tcpnje to our Hercules 3.13; kit users need a Hercules with tcpnje. Partners: other Hercules VM, MVS 3.8 NJE38, funetnje in Debian (9.13c).</t>
+          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13 15 Oct: CE has RSCS V1 (DMT* on 39F, no NJE). Route: TCPNJE (Hercules device, spinhawk README.TCPNJE: 2703 BSC inside, NJE over TCP outside) + the RSCS NJE updates; port tcpnje to our Hercules 3.13; kit users need a Hercules with tcpnje. Partners: other Hercules VM, MVS 3.8 NJE38, funetnje in Debian (9.13c). Owner: TCPNJE is the way (15 Oct). Services to run once NJE works: moshix/BITNETServices (RELAY CHAT, TRICKLE, LISTSERV, LOOKUP, ELIZA; needs RSCS class B, MSGNOH).</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Step 1 done (dev)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct. Hook: DMSEXC first-record check (NUCBREXX). BREXX stays default until Regina passes the BREXX test EXECs</t>
+          <t>15 Oct: step 1 -- DMSEXC XA0057DK: first line '/*!name' runs the EXEC as 'name =EXEC fn EXEC args' (SVC 202); cmsrt turns '=EXEC fn ft' into the file fn.ft. Run bang3: BANG EXEC (/*!REGINA) -&gt; Regina, args passed, RC 7 returned; plain '/*' EXEC still BREXX (RC 3); EXEC BANG works too. Next: SET REXX default; Regina resident (NUCXLOAD), shared stack, EXECIO STEM/VAR, CMSFLAG(); PARSE SOURCE as CMS has it</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Milestones: 9.42 Markdown printing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G130"/>
+  <dimension ref="A3:G131"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3719,27 +3719,32 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.42</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>Markdown printing</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>Print Markdown documents (CommonMark + GitHub tables): (a) on CMS, MDPRINT fn MD to the line printer or console -- headings, lists, block quotes, code, tables laid out in 132 columns, no Debian needed; (b) PostScript/PDF: Markdown -&gt; troff ms (+tbl) -&gt; groff, as BOOKIE does, from CMS over the 9.25 bridge (PSPRINT to a printer, PDF back as a file) and as mdprint in the Debian guest</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Owner request 15 Oct. Reuses 9.28 (groff), 9.29 (Ghostscript), 9.30 (bookie route), 9.31 (PSPRINT)</t>
         </is>
       </c>
     </row>
@@ -3751,17 +3756,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -3771,7 +3776,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3783,17 +3788,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3803,7 +3808,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3815,17 +3820,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3833,14 +3838,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -3852,66 +3852,78 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
+      <c r="G109" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="2" t="n"/>
-      <c r="B109" s="10" t="n"/>
-      <c r="C109" s="2" t="n"/>
-      <c r="D109" s="2" t="n"/>
-      <c r="E109" s="5" t="n"/>
-      <c r="F109" s="2" t="n"/>
-      <c r="G109" s="2" t="n"/>
-    </row>
     <row r="110">
-      <c r="A110" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A110" s="2" t="n"/>
       <c r="B110" s="10" t="n"/>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C110" s="2" t="n"/>
+      <c r="D110" s="2" t="n"/>
+      <c r="E110" s="5" t="n"/>
       <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="n"/>
     </row>
@@ -3921,22 +3933,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B111" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C111" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D111" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="n"/>
+      <c r="B111" s="10" t="n"/>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
     </row>
@@ -3948,7 +3960,7 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
@@ -3958,7 +3970,7 @@
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E112" s="5" t="n"/>
@@ -3973,17 +3985,17 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D113" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E113" s="5" t="n"/>
@@ -3991,40 +4003,36 @@
       <c r="G113" s="2" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="14" t="n"/>
-      <c r="B114" s="13" t="n"/>
-      <c r="C114" s="14" t="n"/>
-      <c r="D114" s="14" t="n"/>
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B114" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C114" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E114" s="5" t="n"/>
       <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B115" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C115" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E115" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A115" s="14" t="n"/>
+      <c r="B115" s="13" t="n"/>
+      <c r="C115" s="14" t="n"/>
+      <c r="D115" s="14" t="n"/>
+      <c r="E115" s="5" t="n"/>
       <c r="F115" s="2" t="n"/>
       <c r="G115" s="2" t="n"/>
     </row>
@@ -4036,17 +4044,17 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E116" s="16" t="inlineStr">
@@ -4065,17 +4073,17 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D117" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
@@ -4094,17 +4102,17 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D118" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E118" s="16" t="inlineStr">
@@ -4123,17 +4131,17 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
@@ -4152,17 +4160,17 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E120" s="16" t="inlineStr">
@@ -4181,20 +4189,24 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E121" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F121" s="2" t="n"/>
       <c r="G121" s="2" t="n"/>
     </row>
@@ -4206,17 +4218,17 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E122" s="5" t="n"/>
@@ -4224,41 +4236,34 @@
       <c r="G122" s="2" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="8" t="n"/>
-      <c r="B123" s="11" t="n"/>
-      <c r="C123" s="8" t="n"/>
+      <c r="A123" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C123" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D123" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="n"/>
+      <c r="F123" s="2" t="n"/>
+      <c r="G123" s="2" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B124" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A124" s="8" t="n"/>
+      <c r="B124" s="11" t="n"/>
+      <c r="C124" s="8" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
@@ -4268,7 +4273,7 @@
       </c>
       <c r="B125" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
@@ -4278,12 +4283,17 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4305,7 @@
       </c>
       <c r="B126" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
@@ -4305,7 +4315,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -4322,7 +4332,7 @@
       </c>
       <c r="B127" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -4332,7 +4342,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -4349,7 +4359,7 @@
       </c>
       <c r="B128" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
@@ -4359,39 +4369,34 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -4401,7 +4406,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4413,25 +4418,57 @@
       </c>
       <c r="B130" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C130" s="8" t="inlineStr">
+      <c r="C131" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr">
+      <c r="D131" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr">
+      <c r="E131" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr">
+      <c r="G131" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
9.39 step 2: SETREXX name|BREXX -- the interpreter for plain /* EXECs (NUCON word, read by DMSEXC)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3623,7 +3623,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Step 1 done (dev)</t>
+          <t>Step 2 done (dev)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>15 Oct: step 1 -- DMSEXC XA0057DK: first line '/*!name' runs the EXEC as 'name =EXEC fn EXEC args' (SVC 202); cmsrt turns '=EXEC fn ft' into the file fn.ft. Run bang3: BANG EXEC (/*!REGINA) -&gt; Regina, args passed, RC 7 returned; plain '/*' EXEC still BREXX (RC 3); EXEC BANG works too. Next: SET REXX default; Regina resident (NUCXLOAD), shared stack, EXECIO STEM/VAR, CMSFLAG(); PARSE SOURCE as CMS has it</t>
+          <t>15 Oct: step 1 -- DMSEXC XA0057DK: first line '/*!name' runs the EXEC as 'name =EXEC fn EXEC args' (SVC 202); cmsrt turns '=EXEC fn ft' into fn.ft (run bang3: Regina, args, RC 7; plain /* still BREXX). Step 2 -- SETREXX name|BREXX (cms/SETREXX ASSEMBLE): the default for plain '/*' EXECs, 8 bytes in NUCON (2F reserved @VA05055 after OSMODLDW), read by DMSEXC (run sr1: BREXX -&gt; REGINA -&gt; BREXX). Next (step 3): Regina resident (nested Regina EXECs today load over the running one), shared stack, EXECIO STEM/VAR via EXECCOMM, CMSFLAG(); PARSE SOURCE as CMS has it</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Milestones: 9.43 EXEC 2 (later)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G131"/>
+  <dimension ref="A3:G132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3756,27 +3756,28 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.43</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>EXEC 2</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>Our own EXEC 2 interpreter for CMS (IBM's is VM/SP code, not public), written from the EXEC 2 Reference (bitsavers SC23-0361): &amp;TRACE first line, &amp;variables, &amp;IF/&amp;GOTO/&amp;LOOP, &amp;STACK/&amp;READ, &amp;SUBCOMMAND, built-in functions. Dispatched by DMSEXC like 9.39: a first line starting &amp;TRACE goes to EXEC2, as on VM/SP; EXEC 1 files keep running under EXEC</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
+          <t>Planned (later)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Owner request 15 Oct. Check first what CE's REXXEC2 MODULE (19E) is. Hook: the 9.39 dispatch (XA0057DK)</t>
         </is>
       </c>
     </row>
@@ -3788,17 +3789,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3808,7 +3809,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3820,17 +3821,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3840,7 +3841,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3852,17 +3853,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3870,14 +3871,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -3889,66 +3885,78 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr">
+      <c r="G110" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="2" t="n"/>
-      <c r="B110" s="10" t="n"/>
-      <c r="C110" s="2" t="n"/>
-      <c r="D110" s="2" t="n"/>
-      <c r="E110" s="5" t="n"/>
-      <c r="F110" s="2" t="n"/>
-      <c r="G110" s="2" t="n"/>
-    </row>
     <row r="111">
-      <c r="A111" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A111" s="2" t="n"/>
       <c r="B111" s="10" t="n"/>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C111" s="2" t="n"/>
+      <c r="D111" s="2" t="n"/>
+      <c r="E111" s="5" t="n"/>
       <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
     </row>
@@ -3958,22 +3966,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B112" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C112" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D112" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="n"/>
+      <c r="B112" s="10" t="n"/>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
     </row>
@@ -3985,7 +3993,7 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
@@ -3995,7 +4003,7 @@
       </c>
       <c r="D113" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E113" s="5" t="n"/>
@@ -4010,17 +4018,17 @@
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D114" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E114" s="5" t="n"/>
@@ -4028,40 +4036,36 @@
       <c r="G114" s="2" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="14" t="n"/>
-      <c r="B115" s="13" t="n"/>
-      <c r="C115" s="14" t="n"/>
-      <c r="D115" s="14" t="n"/>
+      <c r="A115" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B115" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C115" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E115" s="5" t="n"/>
       <c r="F115" s="2" t="n"/>
       <c r="G115" s="2" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B116" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C116" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E116" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A116" s="14" t="n"/>
+      <c r="B116" s="13" t="n"/>
+      <c r="C116" s="14" t="n"/>
+      <c r="D116" s="14" t="n"/>
+      <c r="E116" s="5" t="n"/>
       <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="n"/>
     </row>
@@ -4073,17 +4077,17 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
@@ -4102,17 +4106,17 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D118" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E118" s="16" t="inlineStr">
@@ -4131,17 +4135,17 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
@@ -4160,17 +4164,17 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E120" s="16" t="inlineStr">
@@ -4189,17 +4193,17 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
@@ -4218,20 +4222,24 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E122" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E122" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F122" s="2" t="n"/>
       <c r="G122" s="2" t="n"/>
     </row>
@@ -4243,17 +4251,17 @@
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E123" s="5" t="n"/>
@@ -4261,41 +4269,34 @@
       <c r="G123" s="2" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="8" t="n"/>
-      <c r="B124" s="11" t="n"/>
-      <c r="C124" s="8" t="n"/>
+      <c r="A124" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B124" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C124" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="n"/>
+      <c r="F124" s="2" t="n"/>
+      <c r="G124" s="2" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B125" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A125" s="8" t="n"/>
+      <c r="B125" s="11" t="n"/>
+      <c r="C125" s="8" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
@@ -4305,7 +4306,7 @@
       </c>
       <c r="B126" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
@@ -4315,12 +4316,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4332,7 +4338,7 @@
       </c>
       <c r="B127" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -4342,7 +4348,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -4359,7 +4365,7 @@
       </c>
       <c r="B128" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
@@ -4369,7 +4375,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -4386,7 +4392,7 @@
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -4396,39 +4402,34 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B130" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -4438,7 +4439,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4450,25 +4451,57 @@
       </c>
       <c r="B131" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C131" s="8" t="inlineStr">
+      <c r="C132" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr">
+      <c r="D132" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
+      <c r="G132" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
9.39 step 3: XLRES -- XIMAGEs resident above 16 MB as nucleus extensions, a fresh copy per call (Regina EXECs nest); SYSPROFX and LANG load it; Regina also built as XIMAGE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3623,7 +3623,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Step 2 done (dev)</t>
+          <t>Steps 1-3 done (dev)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>15 Oct: step 1 -- DMSEXC XA0057DK: first line '/*!name' runs the EXEC as 'name =EXEC fn EXEC args' (SVC 202); cmsrt turns '=EXEC fn ft' into fn.ft (run bang3: Regina, args, RC 7; plain /* still BREXX). Step 2 -- SETREXX name|BREXX (cms/SETREXX ASSEMBLE): the default for plain '/*' EXECs, 8 bytes in NUCON (2F reserved @VA05055 after OSMODLDW), read by DMSEXC (run sr1: BREXX -&gt; REGINA -&gt; BREXX). Next (step 3): Regina resident (nested Regina EXECs today load over the running one), shared stack, EXECIO STEM/VAR via EXECCOMM, CMSFLAG(); PARSE SOURCE as CMS has it</t>
+          <t>15 Oct: (1) DMSEXC XA0057DK: '/*!name' first line runs the EXEC as 'name =EXEC fn EXEC args'; cmsrt maps =EXEC to fn.ft (bang3). (2) SETREXX name|BREXX: default for plain '/*' EXECs, NUCON word read by DMSEXC (sr1). (3) XLRES (cms/XLRES ASSEMBLE, nucleus extension loaded by SYSPROFX under IPL 290): XLRES LOAD name keeps an XIMAGE above 16 MB and registers name; each call runs a fresh relocated copy with its own low block, so Regina EXECs nest (NEST -&gt; BANG, rc 7 back, rc 5); LANG loads REGINA XIMAGE (xi1). Next: CMS stack/EXECIO STEM-VAR via EXECCOMM, CMSFLAG(), PARSE SOURCE as CMS has it</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3774,6 @@
           <t>Planned (later)</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Owner request 15 Oct. Check first what CE's REXXEC2 MODULE (19E) is. Hook: the 9.39 dispatch (XA0057DK)</t>

</xml_diff>

<commit_message>
9.39 step 4: Regina on the CMS stack and EXECCOMM (EXECIO STEM/VAR, GLOBALV GET/PUT); cmsrt: cms_subcom, extended plist on CMS commands, cms_program_init hook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3623,7 +3623,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Steps 1-3 done (dev)</t>
+          <t>Steps 1-4 done (dev)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>15 Oct: (1) DMSEXC XA0057DK: '/*!name' first line runs the EXEC as 'name =EXEC fn EXEC args'; cmsrt maps =EXEC to fn.ft (bang3). (2) SETREXX name|BREXX: default for plain '/*' EXECs, NUCON word read by DMSEXC (sr1). (3) XLRES (cms/XLRES ASSEMBLE, nucleus extension loaded by SYSPROFX under IPL 290): XLRES LOAD name keeps an XIMAGE above 16 MB and registers name; each call runs a fresh relocated copy with its own low block, so Regina EXECs nest (NEST -&gt; BANG, rc 7 back, rc 5); LANG loads REGINA XIMAGE (xi1). Next: CMS stack/EXECIO STEM-VAR via EXECCOMM, CMSFLAG(), PARSE SOURCE as CMS has it</t>
+          <t>15 Oct: (1) DMSEXC XA0057DK: '/*!name' first line -&gt; 'name =EXEC fn EXEC args' (bang3). (2) SETREXX name|BREXX: default for plain '/*' EXECs (sr1). (3) XLRES: XIMAGEs resident above 16 MB as nucleus extensions, a fresh copy per call -- Regina EXECs nest (xi1). (4) Regina's CMS integration: PUSH/QUEUE/QUEUED() on the CMS console stack (ATTN, NUMFINRD; st1); EXECCOMM as a SUBCOM of each running Regina (cmsrt cms_subcom: AMODE 24 stub in the low block), so EXECIO STEM/VAR and GLOBALV GET/PUT reach Regina variables (eio7); cmsrt passes the extended plist (R0) on CMS commands, as EXECIO needs. Next: CMSFLAG(), PARSE SOURCE as CMS has it, kit b21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b21: REXX dispatch (/*!name, SETREXX), Regina resident (XLRES) with CMS stack and EXECCOMM; verified on a fresh CE (kt35)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3549,7 +3549,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Done (kit b20)</t>
+          <t>Done (kit b20; resident and CMS-integrated b21)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Steps 1-4 done (dev)</t>
+          <t>Done (kit b21)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">

</xml_diff>

<commit_message>
9.41: vmspool -- decks from the PC into a user's reader through Hercules socket card readers (10C text, 20C binary), started by AUTOLOG1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3697,7 +3697,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct (installation decks from the PC)</t>
+          <t>16 Oct: Hercules socket card readers 010C (127.0.0.1:3505, ascii) and 020C (:3506, ebcdic) in vm370ce.conf, started by AUTOLOG1 at IPL; tools/vmspool.py FILE USERID [FN FT] [--binary] prefixes 'ID USERID NAME FN FT' and sends the deck (Python 3, Windows/Linux). Verified sp1 (text, 8466-card binary REGINA XIMAGE, second text deck) and sp3 (readers started by AUTOLOG1, deck in CMSUSER's reader). Printer output back to the PC (sockdev 1403) and vmur in Linux guests: later</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.42: MDPRINT and UNSTREAM installed on 19E (test md-install), milestones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3707,7 +3707,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>16 Oct: Hercules socket card readers 010C (127.0.0.1:3505, ascii) and 020C (:3506, ebcdic) in vm370ce.conf, started by AUTOLOG1 at IPL; tools/vmspool.py FILE USERID [FN FT] [--binary] prefixes 'ID USERID NAME FN FT' and sends the deck (Python 3, Windows/Linux). Verified sp1 (text, 8466-card binary REGINA XIMAGE, second text deck) and sp3 (readers started by AUTOLOG1, deck in CMSUSER's reader). Printer output back to the PC (sockdev 1403) and vmur in Linux guests: later</t>
+          <t>vmspool.py: text 010C/3505, binary and stream 020C/3506, AUTOLOG1 starts both; UNSTREAM EXEC for lines over 80. Tests sp-vmspool, sp-vmspool-autostart.</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct. Reuses 9.28 (groff), 9.29 (Ghostscript), 9.30 (bookie route), 9.31 (PSPRINT)</t>
+          <t>MDPRINT EXEC on 19E: TYPE/DISK/PRINT on CMS (headings, nested lists, code, quotes, tables), (PS via the spool bridge 'markdown' handler (md2ms + groff -ms -t). Debian: md2ms, mdprint. UNSTREAM for long-line files from vmspool. Test md-install (mdi2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b22: vmspool (9.41) and Markdown printing (9.42); kittest.sh; Debian handler on lnx190
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3697,7 +3697,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b22)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>vmspool.py: text 010C/3505, binary and stream 020C/3506, AUTOLOG1 starts both; UNSTREAM EXEC for lines over 80. Tests sp-vmspool, sp-vmspool-autostart.</t>
+          <t>vmspool.py: text 010C/3505, binary and stream 020C/3506, AUTOLOG1 starts both; UNSTREAM EXEC for lines over 80. Verified on a fresh CE + b22 (kt36): PCHELLO EXEC and SAMPLE MD (stream) sent from the PC arrived in CMSUSER's reader.</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b22)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>MDPRINT EXEC on 19E: TYPE/DISK/PRINT on CMS (headings, nested lists, code, quotes, tables). (PS: vmspool handler 'markdown' in Debian (md2ms with its own ms subset, groff -t; Debian has no ms macros). Debian: md2ms, mdprint. UNSTREAM for long-line files from vmspool. Tests md-install (mdi2), md-debian (mdd3).</t>
+          <t>MDPRINT EXEC (19E): TYPE/DISK/PRINT on CMS; (PS via the vmspool 'markdown' handler in Debian (md2ms with its own ms subset, groff -t). Debian: md2ms, mdprint. Tests md-install, md-debian (mdd4, on lnx190); fresh CE + b22 (kt36): UNSTREAM + MDPRINT TYPE/DISK.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.40: local DNS zone on BORDER (vmdns, kernel #13), BORDER CONFIG DOMAIN/HOST/MX, dnsq/fakedns tools
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3660,7 +3660,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct; before or with 9.18</t>
+          <t>vmdns on BORDER (kernel #13 initramfs): local zone from BORDER CONFIG (DOMAIN, HOST, MX) answered on 10.3.0.1 (A, PTR, MX, NS, SOA, NXDOMAIN), others relayed to DNS (the PC); DHCP gives the search domain. Test dns-border (dns2). Open: search line for Debian's static LAN address.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.18: mail -- vmmaild (SMTP in), mail service + SENDMAIL/GETMAIL, vmspoold outbox, LXCALL orders its answer; LAN names in Debian /etc/hosts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3075,13 +3075,13 @@
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct; after 9.12</t>
+          <t>Debian (MAINT) is the mail host: vmmaild (SMTP in, port 25) puts userid@DOMAIN mail into the user's reader as 'sender MAIL' via vmspoold's new outbox; service 'mail' + SENDMAIL EXEC send from CMS (CMS users at once, others by SMARTHOST or MX); GETMAIL reads MAIL files into MAILnnnn MAIL A; LXCALL orders its answer first. vm370plus-lan writes the LAN names to /etc/hosts + search. Tests mail-debian (mail1), mdd5.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b23: local DNS zone (9.40) and mail (9.18); kt37
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3075,13 +3075,13 @@
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b23)</t>
         </is>
       </c>
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Debian (MAINT) is the mail host: vmmaild (SMTP in, port 25) puts userid@DOMAIN mail into the user's reader as 'sender MAIL' via vmspoold's new outbox; service 'mail' + SENDMAIL EXEC send from CMS (CMS users at once, others by SMARTHOST or MX); GETMAIL reads MAIL files into MAILnnnn MAIL A; LXCALL orders its answer first. vm370plus-lan writes the LAN names to /etc/hosts + search. Tests mail-debian (mail1), mdd5.</t>
+          <t>Debian (MAINT) is the mail host: vmmaild (SMTP in) -&gt; reader files 'sender MAIL' via vmspoold's outbox; service 'mail' + SENDMAIL EXEC (CMS users at once, others by SMARTHOST or MX); GETMAIL -&gt; MAILnnnn MAIL A. Tests mail-debian (mail1: PC-&gt;CMS, CMS-&gt;CMS, CMS-&gt;smarthost); fresh CE + b23 (kt37: SENDMAIL to cmsuser and maint, GETMAIL).</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b23)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>vmdns on BORDER (kernel #13 initramfs): local zone from BORDER CONFIG (DOMAIN, HOST, MX) answered on 10.3.0.1 (A, PTR, MX, NS, SOA, NXDOMAIN), others relayed to DNS (the PC); DHCP gives the search domain. Test dns-border (dns2). Open: search line for Debian's static LAN address.</t>
+          <t>vmdns on BORDER (kernel #13): local zone from BORDER CONFIG (DOMAIN, HOST, MX) on 10.3.0.1 (A, PTR, MX, NS, SOA, NXDOMAIN), others relayed to DNS (the PC); DHCP gives the search domain; Debian writes the LAN names to /etc/hosts. Tests dns-border (dns2); kit b23 (kt37: LINUX13 on BORDER 191, BORDER CONFIG).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.10: AI gateway -- ASK EXEC, service ask (OpenAI-compatible or Anthropic API), ask on Linux, fakellm test server
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2477,11 +2477,15 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>AI gateway over the spool bridge: ASK EXEC (19E) -&gt; service 'ask' in the Debian guest -&gt; the model of /etc/vmspool.d/ask.conf (OpenAI protocol: llama.cpp llama-server / Ollama / LM Studio on the PC, or Anthropic's API), per-user history (ASK NEW), (FILE adds a file; 'ask' on Linux. Tests ask-debian (ask1, fake model tools/fakellm.py), ask-cms-file.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">

</xml_diff>

<commit_message>
9.44: printer on the PC -- socket printer 010E (class P, started by AUTOLOG1), vmprint.py, PCPRINT EXEC
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G132"/>
+  <dimension ref="A3:G133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3792,27 +3792,32 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.44</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>Printer on the PC</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>CP printer output to the PC as files: a socket printer 010E (1403 sockdev) that AUTOLOG1 starts for class P; vmprint.py on the PC writes each print file as .txt or .ps (.pdf, lp); PCPRINT EXEC on CMS</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Done (dev; kit next)</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>16 Oct</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Found while doing 9.41/9.42 (the reader side). AUTOLOG1: START 10E CLASS P NOSEP; if vmprint was not connected, CP stops 10E (INT REQ) and the operator STARTs it again. Tests pr-socket-printer, pr-socket-printer-late, pr-pcprint (pr4: a listing and a PostScript job from PCPRINT).</t>
         </is>
       </c>
     </row>
@@ -3824,17 +3829,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3844,7 +3849,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3856,17 +3861,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3876,7 +3881,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3888,17 +3893,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3906,14 +3911,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -3925,66 +3925,78 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
+      <c r="G111" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="2" t="n"/>
-      <c r="B111" s="10" t="n"/>
-      <c r="C111" s="2" t="n"/>
-      <c r="D111" s="2" t="n"/>
-      <c r="E111" s="5" t="n"/>
-      <c r="F111" s="2" t="n"/>
-      <c r="G111" s="2" t="n"/>
-    </row>
     <row r="112">
-      <c r="A112" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A112" s="2" t="n"/>
       <c r="B112" s="10" t="n"/>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C112" s="2" t="n"/>
+      <c r="D112" s="2" t="n"/>
+      <c r="E112" s="5" t="n"/>
       <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
     </row>
@@ -3994,22 +4006,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B113" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C113" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D113" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="n"/>
+      <c r="B113" s="10" t="n"/>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
     </row>
@@ -4021,7 +4033,7 @@
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
@@ -4031,7 +4043,7 @@
       </c>
       <c r="D114" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E114" s="5" t="n"/>
@@ -4046,17 +4058,17 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D115" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E115" s="5" t="n"/>
@@ -4064,40 +4076,36 @@
       <c r="G115" s="2" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="14" t="n"/>
-      <c r="B116" s="13" t="n"/>
-      <c r="C116" s="14" t="n"/>
-      <c r="D116" s="14" t="n"/>
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E116" s="5" t="n"/>
       <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B117" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C117" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E117" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A117" s="14" t="n"/>
+      <c r="B117" s="13" t="n"/>
+      <c r="C117" s="14" t="n"/>
+      <c r="D117" s="14" t="n"/>
+      <c r="E117" s="5" t="n"/>
       <c r="F117" s="2" t="n"/>
       <c r="G117" s="2" t="n"/>
     </row>
@@ -4109,17 +4117,17 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E118" s="16" t="inlineStr">
@@ -4138,17 +4146,17 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D119" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
@@ -4167,17 +4175,17 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E120" s="16" t="inlineStr">
@@ -4196,17 +4204,17 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
@@ -4225,17 +4233,17 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E122" s="16" t="inlineStr">
@@ -4254,20 +4262,24 @@
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E123" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E123" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F123" s="2" t="n"/>
       <c r="G123" s="2" t="n"/>
     </row>
@@ -4279,17 +4291,17 @@
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D124" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E124" s="5" t="n"/>
@@ -4297,41 +4309,34 @@
       <c r="G124" s="2" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="8" t="n"/>
-      <c r="B125" s="11" t="n"/>
-      <c r="C125" s="8" t="n"/>
+      <c r="A125" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B125" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C125" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D125" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="n"/>
+      <c r="F125" s="2" t="n"/>
+      <c r="G125" s="2" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A126" s="8" t="n"/>
+      <c r="B126" s="11" t="n"/>
+      <c r="C126" s="8" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
@@ -4341,7 +4346,7 @@
       </c>
       <c r="B127" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -4351,12 +4356,17 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4378,7 @@
       </c>
       <c r="B128" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
@@ -4378,7 +4388,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -4395,7 +4405,7 @@
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -4405,7 +4415,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -4422,7 +4432,7 @@
       </c>
       <c r="B130" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
@@ -4432,39 +4442,34 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B131" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -4474,7 +4479,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4486,25 +4491,57 @@
       </c>
       <c r="B132" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C132" s="8" t="inlineStr">
+      <c r="C133" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr">
+      <c r="D133" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
+      <c r="E133" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr">
+      <c r="G133" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
9.17: llama2.c on CMS and Debian/390 (big-endian port, LLAMA EXEC, language disk), bit-exact with the PC
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3046,13 +3046,13 @@
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Owner request 11 Oct; llama.cpp itself needs 64-bit, C++17 and GBs</t>
+          <t>llama2.c run.c ported for big-endian 31-bit (languages/llama2c/mk390.py): Debian (llama2c, llama; 3 tok/s on a dim-32 model) and CMS (LLAMA2C MODULE + LLAMA EXEC on the language disk, soft float, 0.9 tok/s); bit-exact with the PC on random-weight models (mkrandom.py). The stories15M model is not shipped (no Hugging Face access from the build machine). Tests llm-cms-random (llm2), llm-debian (llmd), llm-install (llmi).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b24: AI gateway (9.10), printer on the PC (9.44), llama2.c (9.17); kt38
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2477,13 +2477,13 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b24)</t>
         </is>
       </c>
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>AI gateway over the spool bridge: ASK EXEC (19E) -&gt; service 'ask' in the Debian guest -&gt; the model of /etc/vmspool.d/ask.conf (OpenAI protocol: llama.cpp llama-server / Ollama / LM Studio on the PC, or Anthropic's API), per-user history (ASK NEW), (FILE adds a file; 'ask' on Linux. Tests ask-debian (ask1, fake model tools/fakellm.py), ask-cms-file.</t>
+          <t>AI gateway: ASK EXEC (19E) -&gt; service 'ask' (Debian) -&gt; /etc/vmspool.d/ask.conf: OpenAI protocol (llama.cpp llama-server / Ollama / LM Studio on the PC, cloud) or Anthropic's API; per-user history, ASK NEW, (FILE; 'ask' on Linux. Tests ask-debian (ask1, tools/fakellm.py), ask-cms-file; shipped in b24.</t>
         </is>
       </c>
     </row>
@@ -3046,13 +3046,13 @@
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b24)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>llama2.c run.c ported for big-endian 31-bit (languages/llama2c/mk390.py): Debian (llama2c, llama; 3 tok/s on a dim-32 model) and CMS (LLAMA2C MODULE + LLAMA EXEC on the language disk, soft float, 0.9 tok/s); bit-exact with the PC on random-weight models (mkrandom.py). The stories15M model is not shipped (no Hugging Face access from the build machine). Tests llm-cms-random (llm2), llm-debian (llmd), llm-install (llmi).</t>
+          <t>llama2.c run.c for big-endian 31-bit (languages/llama2c): Debian llama2c/llama, CMS LLAMA2C MODULE + LLAMA EXEC on the language disk (soft float); bit-exact with the PC on random-weight models. stories15M not shipped (no Hugging Face access). Tests llm-*, fresh CE + b24 (kt38: LLAMA from L, same 24 tokens as the PC).</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b24)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Found while doing 9.41/9.42 (the reader side). AUTOLOG1: START 10E CLASS P NOSEP; if vmprint was not connected, CP stops 10E (INT REQ) and the operator STARTs it again. Tests pr-socket-printer, pr-socket-printer-late, pr-pcprint (pr4: a listing and a PostScript job from PCPRINT).</t>
+          <t>Socket printer 010E (1403 sockdev, port 1403), started by AUTOLOG1 for class P NOSEP; tools/vmprint.py writes print files as .txt/.ps (--pdf, --lp); PCPRINT EXEC. Tests pr-*, fresh CE + b24 (kt38: PCPRINT listing arrived through vmprint).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.43: EXEC 2 -- EXEC2 EXEC interpreter, DMSEXC dispatch of &TRACE files (290 nucleus); MAINT PROFILE EXEC restored
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3775,12 +3775,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Planned (later)</t>
+          <t>Done (dev; kit next)</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct. Check first what CE's REXXEC2 MODULE (19E) is. Hook: the 9.39 dispatch (XA0057DK)</t>
+          <t>EXEC2 EXEC (19E, REXX, our own from the EXEC 2 language): statements, assignments with arithmetic and functions, right-to-left substitution, &amp;LOOP/&amp;GOTO/&amp;IF/&amp;CALL/&amp;RETURN, &amp;STACK/&amp;READ/&amp;BEGSTACK/&amp;BEGTYPE, &amp;ERROR, &amp;TRACE. DMSEXC XA0057DK: a first line &amp;TRACE runs 'EXEC EXEC2 =EXEC fn EXEC args' (290 nucleus rebuilt). CE's REXXEC2 MODULE is BREXX's function-package loader, not EXEC 2. Tests exec2-dispatch (e2d3): the same results as on the PC (Regina), EXEC 1 and REXX unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.17: LLAMA GET verified end to end (llg2), wait counted in WAKEUPs; Debian disk cleaned (no model, outq empty)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3046,13 +3046,13 @@
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Done (kit b24)</t>
+          <t>Done (kit b24; model by download, kit b25)</t>
         </is>
       </c>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>llama2.c run.c for big-endian 31-bit (languages/llama2c): Debian llama2c/llama, CMS LLAMA2C MODULE + LLAMA EXEC on the language disk (soft float); bit-exact with the PC on random-weight models. stories15M not shipped (no Hugging Face access). Tests llm-*, fresh CE + b24 (kt38: LLAMA from L, same 24 tokens as the PC).</t>
+          <t>llama2.c run.c for big-endian 31-bit (languages/llama2c): Debian llama2c/llama, CMS LLAMA2C MODULE + LLAMA EXEC on the language disk (soft float); bit-exact with the PC. stories15M (58 MB) not shipped: llama --get (Debian, /etc/llama.conf: vm370plus.com) and LLAMA GET fm (CMS: service llamaget, binary punch by vmspoold's outbox, READCARD onto an EDF disk; ~1 h). CMS story 'Once upon a time, there was a' (0.066 tok/s), Debian 192M 0.11 tok/s. Tests llm-*, llm-get-small (llg2: the whole chain).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b25: EXEC 2, MAINT PROFILE EXEC, llama model by download; verified on a fresh CE (kt39); Guide refreshed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3775,12 +3775,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Done (dev; kit next)</t>
+          <t>Done (kit b25)</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>EXEC2 EXEC (19E, REXX, our own from the EXEC 2 language): statements, assignments with arithmetic and functions, right-to-left substitution, &amp;LOOP/&amp;GOTO/&amp;IF/&amp;CALL/&amp;RETURN, &amp;STACK/&amp;READ/&amp;BEGSTACK/&amp;BEGTYPE, &amp;ERROR, &amp;TRACE. DMSEXC XA0057DK: a first line &amp;TRACE runs 'EXEC EXEC2 =EXEC fn EXEC args' (290 nucleus rebuilt). CE's REXXEC2 MODULE is BREXX's function-package loader, not EXEC 2. Tests exec2-dispatch (e2d3): the same results as on the PC (Regina), EXEC 1 and REXX unchanged.</t>
+          <t>EXEC 2 on CMS: EXEC2 EXEC (19E), our own interpreter (REXX, 72 columns); DMSEXC (290 nucleus) sends an EXEC whose first line starts with &amp;TRACE to it; EXEC2 fn args under any CMS. Tests exec2-dispatch, kt39 (fresh CE, b25).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.45 setup wizard added to the milestones; 9.13b: NJE via Debian (NJE-II), mknje.sh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G133"/>
+  <dimension ref="A3:G134"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2782,13 +2782,13 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress (NJE via Debian)</t>
         </is>
       </c>
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>TCPNJE is in SDL Hyperion; we run Hercules 3.13 15 Oct: CE has RSCS V1 (DMT* on 39F, no NJE). Route: TCPNJE (Hercules device, spinhawk README.TCPNJE: 2703 BSC inside, NJE over TCP outside) + the RSCS NJE updates; port tcpnje to our Hercules 3.13; kit users need a Hercules with tcpnje. Partners: other Hercules VM, MVS 3.8 NJE38, funetnje in Debian (9.13c). Owner: TCPNJE is the way (15 Oct). Services to run once NJE works: moshix/BITNETServices (RELAY CHAT, TRICKLE, LISTSERV, LOOKUP, ELIZA; needs RSCS class B, MSGNOH).</t>
+          <t>16 Oct: the RSCS NJE updates are out of reach; instead NJE-II (FUNET-NJE, github.com/moshix/NJE-II) in the Debian guest makes VM/370plus an NJE node over TCPNJE (port 175): CMS TELL/SENDFILE through the spool bridge, files and messages in through vmspoold's outbox and CP MSG. linux390/nje/mknje.sh fetches and builds it (s390, PC); the source stays out of the repo (HUJI licence).</t>
         </is>
       </c>
     </row>
@@ -3829,27 +3829,27 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.45</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>Setup wizard</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>A setup wizard for VM/370plus on the PC (Windows, Linux, macOS): checks Hercules and Python, unpacks CE and the kit parts, joins the Debian and language disks, asks for the settings (MAINSIZE, node and domain names, ports for 3270/printer/readers, the LAN, mail smarthost, AI model and URL, NJE peers) and writes vm370ce.conf, BORDER CONFIG and the Debian /etc files; then a first IPL with a check that everything came up</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Asked for 16 Oct (user)</t>
         </is>
       </c>
     </row>
@@ -3861,17 +3861,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3893,17 +3893,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3925,17 +3925,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3943,14 +3943,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -3962,66 +3957,78 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
+      <c r="G112" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="2" t="n"/>
-      <c r="B112" s="10" t="n"/>
-      <c r="C112" s="2" t="n"/>
-      <c r="D112" s="2" t="n"/>
-      <c r="E112" s="5" t="n"/>
-      <c r="F112" s="2" t="n"/>
-      <c r="G112" s="2" t="n"/>
-    </row>
     <row r="113">
-      <c r="A113" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A113" s="2" t="n"/>
       <c r="B113" s="10" t="n"/>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C113" s="2" t="n"/>
+      <c r="D113" s="2" t="n"/>
+      <c r="E113" s="5" t="n"/>
       <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
     </row>
@@ -4031,22 +4038,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B114" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C114" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D114" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="n"/>
+      <c r="B114" s="10" t="n"/>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
     </row>
@@ -4058,7 +4065,7 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
@@ -4068,7 +4075,7 @@
       </c>
       <c r="D115" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E115" s="5" t="n"/>
@@ -4083,17 +4090,17 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D116" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E116" s="5" t="n"/>
@@ -4101,40 +4108,36 @@
       <c r="G116" s="2" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="14" t="n"/>
-      <c r="B117" s="13" t="n"/>
-      <c r="C117" s="14" t="n"/>
-      <c r="D117" s="14" t="n"/>
+      <c r="A117" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D117" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E117" s="5" t="n"/>
       <c r="F117" s="2" t="n"/>
       <c r="G117" s="2" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B118" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C118" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E118" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A118" s="14" t="n"/>
+      <c r="B118" s="13" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="14" t="n"/>
+      <c r="E118" s="5" t="n"/>
       <c r="F118" s="2" t="n"/>
       <c r="G118" s="2" t="n"/>
     </row>
@@ -4146,17 +4149,17 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
@@ -4175,17 +4178,17 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D120" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E120" s="16" t="inlineStr">
@@ -4204,17 +4207,17 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
@@ -4233,17 +4236,17 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E122" s="16" t="inlineStr">
@@ -4262,17 +4265,17 @@
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E123" s="16" t="inlineStr">
@@ -4291,20 +4294,24 @@
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D124" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E124" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E124" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F124" s="2" t="n"/>
       <c r="G124" s="2" t="n"/>
     </row>
@@ -4316,17 +4323,17 @@
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C125" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D125" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E125" s="5" t="n"/>
@@ -4334,41 +4341,34 @@
       <c r="G125" s="2" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="8" t="n"/>
-      <c r="B126" s="11" t="n"/>
-      <c r="C126" s="8" t="n"/>
+      <c r="A126" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B126" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C126" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D126" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="n"/>
+      <c r="F126" s="2" t="n"/>
+      <c r="G126" s="2" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B127" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A127" s="8" t="n"/>
+      <c r="B127" s="11" t="n"/>
+      <c r="C127" s="8" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="B128" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
@@ -4388,12 +4388,17 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4410,7 @@
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -4415,7 +4420,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -4432,7 +4437,7 @@
       </c>
       <c r="B130" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
@@ -4442,7 +4447,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -4459,7 +4464,7 @@
       </c>
       <c r="B131" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
@@ -4469,39 +4474,34 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B132" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4523,25 +4523,57 @@
       </c>
       <c r="B133" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B134" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C133" s="8" t="inlineStr">
+      <c r="C134" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr">
+      <c r="D134" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
+      <c r="E134" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr">
+      <c r="G134" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
9.46 OS/2 server code via ROSE (later) added to the milestones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G134"/>
+  <dimension ref="A3:G135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3861,27 +3861,27 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.46</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>OS/2 server code (later)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>OS/2 programs in the Linux guest through ROSE (github.com/mikebeer/rose), the OS/2 API in portable C: (1) recompile OS/2 source (C, C++, REXX) against a native build of ROSE's API layer, as Winelib does -- ROSE's Phase 7 64-bit API track, with s390 as another target; big-endian fixes for code that reads Intel-order binary data; (2) unchanged OS/2 binaries under a user-mode x86 emulator (QEMU i386 user mode emulates the LDT ROSE's 16-bit code needs) -- slow; (3) a full emulated PC with ArcaOS -- slowest, not open source. Our guest is 31-bit s390 (Debian 7), not s390x: route 1 needs ROSE's API layer to build 31-bit too</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Asked for 16 Oct (user): later. Route 1 first (recompile against ROSE's API layer).</t>
         </is>
       </c>
     </row>
@@ -3893,17 +3893,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3925,17 +3925,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3957,17 +3957,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -3975,14 +3975,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -3994,66 +3989,78 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D113" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
+      <c r="G113" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="2" t="n"/>
-      <c r="B113" s="10" t="n"/>
-      <c r="C113" s="2" t="n"/>
-      <c r="D113" s="2" t="n"/>
-      <c r="E113" s="5" t="n"/>
-      <c r="F113" s="2" t="n"/>
-      <c r="G113" s="2" t="n"/>
-    </row>
     <row r="114">
-      <c r="A114" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A114" s="2" t="n"/>
       <c r="B114" s="10" t="n"/>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C114" s="2" t="n"/>
+      <c r="D114" s="2" t="n"/>
+      <c r="E114" s="5" t="n"/>
       <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
     </row>
@@ -4063,22 +4070,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B115" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C115" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D115" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="n"/>
+      <c r="B115" s="10" t="n"/>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F115" s="2" t="n"/>
       <c r="G115" s="2" t="n"/>
     </row>
@@ -4090,7 +4097,7 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
@@ -4100,7 +4107,7 @@
       </c>
       <c r="D116" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E116" s="5" t="n"/>
@@ -4115,17 +4122,17 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D117" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E117" s="5" t="n"/>
@@ -4133,40 +4140,36 @@
       <c r="G117" s="2" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="14" t="n"/>
-      <c r="B118" s="13" t="n"/>
-      <c r="C118" s="14" t="n"/>
-      <c r="D118" s="14" t="n"/>
+      <c r="A118" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B118" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C118" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E118" s="5" t="n"/>
       <c r="F118" s="2" t="n"/>
       <c r="G118" s="2" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B119" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C119" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E119" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A119" s="14" t="n"/>
+      <c r="B119" s="13" t="n"/>
+      <c r="C119" s="14" t="n"/>
+      <c r="D119" s="14" t="n"/>
+      <c r="E119" s="5" t="n"/>
       <c r="F119" s="2" t="n"/>
       <c r="G119" s="2" t="n"/>
     </row>
@@ -4178,17 +4181,17 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E120" s="16" t="inlineStr">
@@ -4207,17 +4210,17 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D121" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
@@ -4236,17 +4239,17 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E122" s="16" t="inlineStr">
@@ -4265,17 +4268,17 @@
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E123" s="16" t="inlineStr">
@@ -4294,17 +4297,17 @@
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D124" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E124" s="16" t="inlineStr">
@@ -4323,20 +4326,24 @@
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C125" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D125" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E125" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E125" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F125" s="2" t="n"/>
       <c r="G125" s="2" t="n"/>
     </row>
@@ -4348,17 +4355,17 @@
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C126" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D126" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E126" s="5" t="n"/>
@@ -4366,41 +4373,34 @@
       <c r="G126" s="2" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="n"/>
-      <c r="B127" s="11" t="n"/>
-      <c r="C127" s="8" t="n"/>
+      <c r="A127" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B127" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C127" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D127" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="n"/>
+      <c r="F127" s="2" t="n"/>
+      <c r="G127" s="2" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B128" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A128" s="8" t="n"/>
+      <c r="B128" s="11" t="n"/>
+      <c r="C128" s="8" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -4420,12 +4420,17 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4442,7 @@
       </c>
       <c r="B130" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
@@ -4447,7 +4452,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -4464,7 +4469,7 @@
       </c>
       <c r="B131" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
@@ -4474,7 +4479,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -4491,7 +4496,7 @@
       </c>
       <c r="B132" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
@@ -4501,39 +4506,34 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B133" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4555,25 +4555,57 @@
       </c>
       <c r="B134" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C134" s="8" t="inlineStr">
+      <c r="C135" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr">
+      <c r="D135" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr">
+      <c r="G135" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
Kit b26 verified on a fresh CE (kt40, kt41 with KITNET=1): NJE both ways, RSCS gateway, no STK001 after Debian halt; kittest: absolute helper paths, KITNET; STATE, milestones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2782,13 +2782,13 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>In progress (NJE via Debian)</t>
+          <t>Done (kit b26)</t>
         </is>
       </c>
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>16 Oct: the RSCS NJE updates are out of reach; instead NJE-II (FUNET-NJE, github.com/moshix/NJE-II) in the Debian guest makes VM/370plus an NJE node over TCPNJE (port 175): CMS TELL/SENDFILE through the spool bridge, files and messages in through vmspoold's outbox and CP MSG. linux390/nje/mknje.sh fetches and builds it (s390, PC); the source stays out of the repo (HUJI licence).</t>
+          <t>NJE via Debian: NJE-II (github.com/moshix/NJE-II) in the Debian guest, node VM370CE, TCPNJE port 175, first peer PCNJE (10.1.1.1). CMS SENDFILE/RECEIVE (CE's NETDATA) and TELL user AT node; RSCS = gateway (NJEGATE EXEC), RSCS V1 kept as RSCSV1. Tests nje-link (njt1), nje-gateway (njt7), kt40 (fresh CE + b26). Source not in the repo (HUJI licence): linux390/nje/mknje.sh.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.45 setup wizard: vm370plus-setup.py (install, conf, guest settings via the vmspool service setup); README and Guide; mkkit ships it; tests wizard-apply (wiz2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3844,12 +3844,12 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (kit b27)</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Asked for 16 Oct (user)</t>
+          <t>vm370plus-setup.py (kit/, beside the parts and in vm370plus/tools): finds CE's zip and the newest complete kit, checks Hercules, unpacks, joins the disks (SHA-256), asks MAINSIZE, 3270 port, CTC link, mail, AI, NJE; writes vm370ce.conf and vm370plus-settings.json; --apply sends the guest settings to the Debian service setup (mail.conf, ask.conf, njeconf). Tests: install from CE + b26 parts; wizard-apply (wiz2: smarthost, 107-char API key, two NJE peers).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.45: the wizard offers to install Hercules (hercules-helper build of SDL Hyperion, Homebrew, distribution package) and a tn3270 emulator; 9.13e: Zork (Dungeon) for CMS on the language disk (languages/zork/mkzork.sh, LANGGEN)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3844,12 +3844,12 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Done (kit b27)</t>
+          <t>Done (kit b27; prerequisites b28)</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>vm370plus-setup.py (kit/, beside the parts and in vm370plus/tools): finds CE's zip and the newest complete kit, checks Hercules, unpacks, joins the disks (SHA-256), asks MAINSIZE, 3270 port, CTC link, mail, AI, NJE; writes vm370ce.conf and vm370plus-settings.json; --apply sends the guest settings to the Debian service setup (mail.conf, ask.conf, njeconf). Tests: install from CE + b26 parts; wizard-apply (wiz2: smarthost, 107-char API key, two NJE peers).</t>
+          <t>vm370plus-setup.py: finds CE's zip and the newest complete kit, checks Python, Hercules and a tn3270 emulator and offers to install them (asking first): Linux -- build the newest SDL Hyperion with hercules-helper (wrljet), or Homebrew, or the distribution's package; macOS -- Homebrew; Windows -- pointer to SDL Hyperion's releases (WC3270 comes with CE). Unpacks, joins the disks (SHA-256), asks MAINSIZE, 3270 port, CTC, mail, AI, NJE; writes vm370ce.conf and vm370plus-settings.json; --apply sends the guest settings to the Debian service setup. Tests: install from CE + b26/b27; wizard-apply (wiz2); prerequisite prompts (Linux, Hercules hidden).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.13e: ZORK on CMS verified (zk1: play, SAVE); LANG README, Guide section
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2881,11 +2881,15 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress (Zork done)</t>
         </is>
       </c>
       <c r="F79" s="2" t="n"/>
-      <c r="G79" s="2" t="n"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>17 Oct: Dungeon (Zork), public-domain C version (github.com/devshane/zork), cross-built for CMS (languages/zork/mkzork.sh, M5f cmscc), ZORK MODULE + DTEXTC DAT on the language disk; test zork-cms (zk1: play, SAVE, QUIT). Still to do: the VM/370 games tape, WIOS SNAKE/SLASH, TREK2.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Kit b28: ZORK, wizard prerequisites; verified kt43; 9.13c done; STATE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2815,13 +2815,13 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done (kit b26)</t>
         </is>
       </c>
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Needs 9.13b</t>
+          <t>Came with 9.13b: NJE-II in the Debian guest is node VM370CE; Linux users reach CMS users with /usr/local/nje/bin/tell user@VM370CE and sendfile user@VM370CE (local delivery: njemsg -&gt; CP MSG, njefile -&gt; reader, NETDATA class N for RECEIVE); CMS reaches Linux through the same node.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Early-user fixes verified (ur2: MAINT DEDICATE 250 + LINUX attach + Debian boot; ur3: LANG hint under IPL CMS, LANG EXEC on 19D); 9.47 MariaDB started: toolchain file, wc++ fixes (no-as-needed, -lrt/-lpthread, drop -lgcc_s, clock waits in the shim)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G135"/>
+  <dimension ref="A3:G136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3616,32 +3616,32 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>9.39</t>
+          <t>9.47</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>REXX dispatch (/*!)</t>
+          <t>MariaDB</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CMS EXEC dispatch by first line: /*!name options */ (still a REXX comment) selects the interpreter (BREXX, REGINA, RXC/cREXX, EXEC); plain /* goes to a settable default (SET REXX BREXX|REGINA). Regina as a selectable default once it is resident in high storage (NUCXLOAD), supports ADDRESS CMS/COMMAND/XEDIT, EXECIO and the stack, and calls user-area MODULEs</t>
+          <t>MariaDB 10.11 cross-built for the 31-bit Debian guest (wc++, GCC 13 -m31, wheezy glibc), the database of MCproject (9.36) and MChelpdesk (9.38): both are Regina REXX servers on MariaDB 10.6+ through the mariadb client, so they run unchanged</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Done (kit b21)</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>15 Oct–</t>
+          <t>17 Oct–</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>15 Oct: (1) DMSEXC XA0057DK: '/*!name' first line -&gt; 'name =EXEC fn EXEC args' (bang3). (2) SETREXX name|BREXX: default for plain '/*' EXECs (sr1). (3) XLRES: XIMAGEs resident above 16 MB as nucleus extensions, a fresh copy per call -- Regina EXECs nest (xi1). (4) Regina's CMS integration: PUSH/QUEUE/QUEUED() on the CMS console stack (ATTN, NUMFINRD; st1); EXECCOMM as a SUBCOM of each running Regina (cmsrt cms_subcom: AMODE 24 stub in the low block), so EXECIO STEM/VAR and GLOBALV GET/PUT reach Regina variables (eio7); cmsrt passes the extended plist (R0) on CMS commands, as EXECIO needs. Next: CMSFLAG(), PARSE SOURCE as CMS has it, kit b21</t>
+          <t>Owner decision 17 Oct (option 1 of 3; the others: MySQL 5.5 from wheezy with schema changes, or a port to PostgreSQL 16). Server-only build, InnoDB/Aria, no performance_schema, bundled WolfSSL/zlib/PCRE2, ncurses cross-built for the client</t>
         </is>
       </c>
     </row>
@@ -3653,22 +3653,22 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>9.40</t>
+          <t>9.39</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Local DNS zone</t>
+          <t>REXX dispatch (/*!)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Names for VM/370plus guests and services: an authoritative zone on BORDER (dnsmasq or similar) next to the DNS forwarder of 9.12d -- guest names, and the domain and MX record mail (9.18) needs</t>
+          <t>CMS EXEC dispatch by first line: /*!name options */ (still a REXX comment) selects the interpreter (BREXX, REGINA, RXC/cREXX, EXEC); plain /* goes to a settable default (SET REXX BREXX|REGINA). Regina as a selectable default once it is resident in high storage (NUCXLOAD), supports ADDRESS CMS/COMMAND/XEDIT, EXECIO and the stack, and calls user-area MODULEs</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Done (kit b23)</t>
+          <t>Done (kit b21)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>vmdns on BORDER (kernel #13): local zone from BORDER CONFIG (DOMAIN, HOST, MX) on 10.3.0.1 (A, PTR, MX, NS, SOA, NXDOMAIN), others relayed to DNS (the PC); DHCP gives the search domain; Debian writes the LAN names to /etc/hosts. Tests dns-border (dns2); kit b23 (kt37: LINUX13 on BORDER 191, BORDER CONFIG).</t>
+          <t>15 Oct: (1) DMSEXC XA0057DK: '/*!name' first line -&gt; 'name =EXEC fn EXEC args' (bang3). (2) SETREXX name|BREXX: default for plain '/*' EXECs (sr1). (3) XLRES: XIMAGEs resident above 16 MB as nucleus extensions, a fresh copy per call -- Regina EXECs nest (xi1). (4) Regina's CMS integration: PUSH/QUEUE/QUEUED() on the CMS console stack (ATTN, NUMFINRD; st1); EXECCOMM as a SUBCOM of each running Regina (cmsrt cms_subcom: AMODE 24 stub in the low block), so EXECIO STEM/VAR and GLOBALV GET/PUT reach Regina variables (eio7); cmsrt passes the extended plist (R0) on CMS commands, as EXECIO needs. Next: CMSFLAG(), PARSE SOURCE as CMS has it, kit b21</t>
         </is>
       </c>
     </row>
@@ -3690,22 +3690,22 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>9.41</t>
+          <t>9.40</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>PC spool reader</t>
+          <t>Local DNS zone</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Spool decks from the PC (Windows and Linux) into VM/370 spool: a Hercules sockdev card reader in vm370ce.conf, started at IPL, and a small Python tool (vmspool deck USERID) that prefixes an ID card and sends the deck; it arrives in the user's reader. Same for printer output back to the PC. Later: vmur in Linux guests (needs DIAG 14/210 in CP)</t>
+          <t>Names for VM/370plus guests and services: an authoritative zone on BORDER (dnsmasq or similar) next to the DNS forwarder of 9.12d -- guest names, and the domain and MX record mail (9.18) needs</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Done (kit b22)</t>
+          <t>Done (kit b23)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>vmspool.py: text 010C/3505, binary and stream 020C/3506, AUTOLOG1 starts both; UNSTREAM EXEC for lines over 80. Verified on a fresh CE + b22 (kt36): PCHELLO EXEC and SAMPLE MD (stream) sent from the PC arrived in CMSUSER's reader.</t>
+          <t>vmdns on BORDER (kernel #13): local zone from BORDER CONFIG (DOMAIN, HOST, MX) on 10.3.0.1 (A, PTR, MX, NS, SOA, NXDOMAIN), others relayed to DNS (the PC); DHCP gives the search domain; Debian writes the LAN names to /etc/hosts. Tests dns-border (dns2); kit b23 (kt37: LINUX13 on BORDER 191, BORDER CONFIG).</t>
         </is>
       </c>
     </row>
@@ -3727,17 +3727,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>9.42</t>
+          <t>9.41</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Markdown printing</t>
+          <t>PC spool reader</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Print Markdown documents (CommonMark + GitHub tables): (a) on CMS, MDPRINT fn MD to the line printer or console -- headings, lists, block quotes, code, tables laid out in 132 columns, no Debian needed; (b) PostScript/PDF: Markdown -&gt; troff ms (+tbl) -&gt; groff, as BOOKIE does, from CMS over the 9.25 bridge (PSPRINT to a printer, PDF back as a file) and as mdprint in the Debian guest</t>
+          <t>Spool decks from the PC (Windows and Linux) into VM/370 spool: a Hercules sockdev card reader in vm370ce.conf, started at IPL, and a small Python tool (vmspool deck USERID) that prefixes an ID card and sends the deck; it arrives in the user's reader. Same for printer output back to the PC. Later: vmur in Linux guests (needs DIAG 14/210 in CP)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>MDPRINT EXEC (19E): TYPE/DISK/PRINT on CMS; (PS via the vmspool 'markdown' handler in Debian (md2ms with its own ms subset, groff -t). Debian: md2ms, mdprint. Tests md-install, md-debian (mdd4, on lnx190); fresh CE + b22 (kt36): UNSTREAM + MDPRINT TYPE/DISK.</t>
+          <t>vmspool.py: text 010C/3505, binary and stream 020C/3506, AUTOLOG1 starts both; UNSTREAM EXEC for lines over 80. Verified on a fresh CE + b22 (kt36): PCHELLO EXEC and SAMPLE MD (stream) sent from the PC arrived in CMSUSER's reader.</t>
         </is>
       </c>
     </row>
@@ -3764,27 +3764,32 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>9.43</t>
+          <t>9.42</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>EXEC 2</t>
+          <t>Markdown printing</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Our own EXEC 2 interpreter for CMS (IBM's is VM/SP code, not public), written from the EXEC 2 Reference (bitsavers SC23-0361): &amp;TRACE first line, &amp;variables, &amp;IF/&amp;GOTO/&amp;LOOP, &amp;STACK/&amp;READ, &amp;SUBCOMMAND, built-in functions. Dispatched by DMSEXC like 9.39: a first line starting &amp;TRACE goes to EXEC2, as on VM/SP; EXEC 1 files keep running under EXEC</t>
+          <t>Print Markdown documents (CommonMark + GitHub tables): (a) on CMS, MDPRINT fn MD to the line printer or console -- headings, lists, block quotes, code, tables laid out in 132 columns, no Debian needed; (b) PostScript/PDF: Markdown -&gt; troff ms (+tbl) -&gt; groff, as BOOKIE does, from CMS over the 9.25 bridge (PSPRINT to a printer, PDF back as a file) and as mdprint in the Debian guest</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Done (kit b25)</t>
+          <t>Done (kit b22)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>15 Oct–</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>EXEC 2 on CMS: EXEC2 EXEC (19E), our own interpreter (REXX, 72 columns); DMSEXC (290 nucleus) sends an EXEC whose first line starts with &amp;TRACE to it; EXEC2 fn args under any CMS. Tests exec2-dispatch, kt39 (fresh CE, b25).</t>
+          <t>MDPRINT EXEC (19E): TYPE/DISK/PRINT on CMS; (PS via the vmspool 'markdown' handler in Debian (md2ms with its own ms subset, groff -t). Debian: md2ms, mdprint. Tests md-install, md-debian (mdd4, on lnx190); fresh CE + b22 (kt36): UNSTREAM + MDPRINT TYPE/DISK.</t>
         </is>
       </c>
     </row>
@@ -3796,32 +3801,27 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9.44</t>
+          <t>9.43</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Printer on the PC</t>
+          <t>EXEC 2</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>CP printer output to the PC as files: a socket printer 010E (1403 sockdev) that AUTOLOG1 starts for class P; vmprint.py on the PC writes each print file as .txt or .ps (.pdf, lp); PCPRINT EXEC on CMS</t>
+          <t>Our own EXEC 2 interpreter for CMS (IBM's is VM/SP code, not public), written from the EXEC 2 Reference (bitsavers SC23-0361): &amp;TRACE first line, &amp;variables, &amp;IF/&amp;GOTO/&amp;LOOP, &amp;STACK/&amp;READ, &amp;SUBCOMMAND, built-in functions. Dispatched by DMSEXC like 9.39: a first line starting &amp;TRACE goes to EXEC2, as on VM/SP; EXEC 1 files keep running under EXEC</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Done (kit b24)</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>16 Oct</t>
+          <t>Done (kit b25)</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Socket printer 010E (1403 sockdev, port 1403), started by AUTOLOG1 for class P NOSEP; tools/vmprint.py writes print files as .txt/.ps (--pdf, --lp); PCPRINT EXEC. Tests pr-*, fresh CE + b24 (kt38: PCPRINT listing arrived through vmprint).</t>
+          <t>EXEC 2 on CMS: EXEC2 EXEC (19E), our own interpreter (REXX, 72 columns); DMSEXC (290 nucleus) sends an EXEC whose first line starts with &amp;TRACE to it; EXEC2 fn args under any CMS. Tests exec2-dispatch, kt39 (fresh CE, b25).</t>
         </is>
       </c>
     </row>
@@ -3833,27 +3833,32 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9.45</t>
+          <t>9.44</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Setup wizard</t>
+          <t>Printer on the PC</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>A setup wizard for VM/370plus on the PC (Windows, Linux, macOS): checks Hercules and Python, unpacks CE and the kit parts, joins the Debian and language disks, asks for the settings (MAINSIZE, node and domain names, ports for 3270/printer/readers, the LAN, mail smarthost, AI model and URL, NJE peers) and writes vm370ce.conf, BORDER CONFIG and the Debian /etc files; then a first IPL with a check that everything came up</t>
+          <t>CP printer output to the PC as files: a socket printer 010E (1403 sockdev) that AUTOLOG1 starts for class P; vmprint.py on the PC writes each print file as .txt or .ps (.pdf, lp); PCPRINT EXEC on CMS</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Done (kit b27; prerequisites b28)</t>
+          <t>Done (kit b24)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>16 Oct</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>vm370plus-setup.py: finds CE's zip and the newest complete kit, checks Python, Hercules and a tn3270 emulator and offers to install them (asking first): Linux -- build the newest SDL Hyperion with hercules-helper (wrljet), or Homebrew, or the distribution's package; macOS -- Homebrew; Windows -- pointer to SDL Hyperion's releases (WC3270 comes with CE). Unpacks, joins the disks (SHA-256), asks MAINSIZE, 3270 port, CTC, mail, AI, NJE; writes vm370ce.conf and vm370plus-settings.json; --apply sends the guest settings to the Debian service setup. Tests: install from CE + b26/b27; wizard-apply (wiz2); prerequisite prompts (Linux, Hercules hidden).</t>
+          <t>Socket printer 010E (1403 sockdev, port 1403), started by AUTOLOG1 for class P NOSEP; tools/vmprint.py writes print files as .txt/.ps (--pdf, --lp); PCPRINT EXEC. Tests pr-*, fresh CE + b24 (kt38: PCPRINT listing arrived through vmprint).</t>
         </is>
       </c>
     </row>
@@ -3865,27 +3870,27 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>9.46</t>
+          <t>9.45</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>OS/2 server code (later)</t>
+          <t>Setup wizard</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>OS/2 programs in the Linux guest through ROSE (github.com/mikebeer/rose), the OS/2 API in portable C: (1) recompile OS/2 source (C, C++, REXX) against a native build of ROSE's API layer, as Winelib does -- ROSE's Phase 7 64-bit API track, with s390 as another target; big-endian fixes for code that reads Intel-order binary data; (2) unchanged OS/2 binaries under a user-mode x86 emulator (QEMU i386 user mode emulates the LDT ROSE's 16-bit code needs) -- slow; (3) a full emulated PC with ArcaOS -- slowest, not open source. Our guest is 31-bit s390 (Debian 7), not s390x: route 1 needs ROSE's API layer to build 31-bit too</t>
+          <t>A setup wizard for VM/370plus on the PC (Windows, Linux, macOS): checks Hercules and Python, unpacks CE and the kit parts, joins the Debian and language disks, asks for the settings (MAINSIZE, node and domain names, ports for 3270/printer/readers, the LAN, mail smarthost, AI model and URL, NJE peers) and writes vm370ce.conf, BORDER CONFIG and the Debian /etc files; then a first IPL with a check that everything came up</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Later</t>
+          <t>Done (kit b27; prerequisites b28)</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Asked for 16 Oct (user): later. Route 1 first (recompile against ROSE's API layer).</t>
+          <t>vm370plus-setup.py: finds CE's zip and the newest complete kit, checks Python, Hercules and a tn3270 emulator and offers to install them (asking first): Linux -- build the newest SDL Hyperion with hercules-helper (wrljet), or Homebrew, or the distribution's package; macOS -- Homebrew; Windows -- pointer to SDL Hyperion's releases (WC3270 comes with CE). Unpacks, joins the disks (SHA-256), asks MAINSIZE, 3270 port, CTC, mail, AI, NJE; writes vm370ce.conf and vm370plus-settings.json; --apply sends the guest settings to the Debian service setup. Tests: install from CE + b26/b27; wizard-apply (wiz2); prerequisite prompts (Linux, Hercules hidden).</t>
         </is>
       </c>
     </row>
@@ -3897,27 +3902,27 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>9.29</t>
+          <t>9.46</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Ghostscript, ps2pdf</t>
+          <t>OS/2 server code (later)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
+          <t>OS/2 programs in the Linux guest through ROSE (github.com/mikebeer/rose), the OS/2 API in portable C: (1) recompile OS/2 source (C, C++, REXX) against a native build of ROSE's API layer, as Winelib does -- ROSE's Phase 7 64-bit API track, with s390 as another target; big-endian fixes for code that reads Intel-order binary data; (2) unchanged OS/2 binaries under a user-mode x86 emulator (QEMU i386 user mode emulates the LDT ROSE's 16-bit code needs) -- slow; (3) a full emulated PC with ArcaOS -- slowest, not open source. Our guest is 31-bit s390 (Debian 7), not s390x: route 1 needs ROSE's API layer to build 31-bit too</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
+          <t>Asked for 16 Oct (user): later. Route 1 first (recompile against ROSE's API layer).</t>
         </is>
       </c>
     </row>
@@ -3929,17 +3934,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>9.30</t>
+          <t>9.29</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>BookMaster</t>
+          <t>Ghostscript, ps2pdf</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
+          <t>Ghostscript in the Debian guest: PS-&gt;PDF (ps2pdf), PDF-&gt;PS (pdf2ps), PS/PDF-&gt;PCL/raster for printers; PS2PDF EXEC on CMS</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3949,7 +3954,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
+          <t>Ghostscript 10.02.1 cross-built (languages/ghostscript/mkgs.sh), gs + ps2pdf/pdf2ps/ps2ps in /usr/local/bin of the Debian guest; PS-&gt;PDF verified pd19</t>
         </is>
       </c>
     </row>
@@ -3961,17 +3966,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>9.31</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Graphical printing</t>
+          <t>BookMaster</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
+          <t>A BookMaster-compatible formatter (BookMaster is IBM-licensed; we build our own): :userdoc./:h1./:p./:ol./:dl. GML tags to SCRIPT-style line output, PS and PDF (via 9.29); BOOKIE EXEC on CMS</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -3981,7 +3986,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
+          <t>bookie: our BookMaster-compatible formatter (languages/bookie/bookie.py -&gt; troff ms+tbl -&gt; groff), BOOKIE EXEC on CMS: text and PostScript, PSPRINT to printer/PDF (pd19). Not done: index, running heads, revision codes</t>
         </is>
       </c>
     </row>
@@ -3993,17 +3998,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>TELL internet</t>
+          <t>Graphical printing</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+          <t>PS/PDF from CMS or Linux to a real printer: (a) bridge: PSPRINT EXEC -&gt; Debian -&gt; Ghostscript -&gt; CUPS/LPD/IPP/port 9100 printer on the PC LAN (needs routing/NAT on the PC for the guest's CTC network); (b) spool: PostScript text on a virtual printer, Hercules 1403 to a file or socket on the PC, a PC script hands it to the printer (PS only, lines up to 132; PDF goes through (a) or ps first)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4011,14 +4016,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>13 Oct</t>
-        </is>
-      </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+          <t>both paths verified pd19: spool (PSPRINT -&gt; 00E -&gt; PC psprint.py, PS byte-identical, ps2pdf) and bridge (PSPRINT (BRIDGE -&gt; Debian gs -&gt; pdf/ps/pcl -&gt; printer port 9100 or lp queue, print.conf); a real printer on the user's LAN still to try</t>
         </is>
       </c>
     </row>
@@ -4030,66 +4030,78 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
+          <t>9.32</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>TELL internet</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>TELL to and from users on the internet: CMS TELL user AT NET publishes to MQTT topic vm/tell/out/&lt;user&gt;; outside users (any MQTT client, password, ACL) publish to vm/tell/from/&lt;user&gt;/to/&lt;vmuser&gt;, a gateway in the Debian guest turns it into CP MSG '(net:user) text'; a forwarder on the PC exposes the broker (router port forward is the owner's)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>13 Oct</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>13 Oct (pd24): TELL user AT NET -&gt; MQTT vm/tell/out/user; outside users publish vm/tell/from/&lt;login&gt;/to/&lt;userid&gt;, tellgw sends CP MSG '(net:login)'; logins (tellnet-user) + ACL on the guest's outside listener, local listener unchanged; tools/netfwd.py (--tls, port 8883) on the PC, tools/nettell.py client. Verified both ways, not-logged-on answer, wrong password and forged sender rejected, TLS. The router's port forward is the owner's. Interim until BORDER (9.12c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
           <t>9.33</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t>CP/M</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D114" t="inlineStr">
         <is>
           <t>CP/M 2.2 on VM/370plus through a Z80 emulator: (a) RunCPM (MIT) in the Debian guest, interactive and as a spool-bridge service (CPM EXEC); (b) natively on CMS (GCC 13 / cmsrt): CP/M disk as CMS files, console on the CMS terminal. CP/M 2.2 binaries freely redistributable (Caldera/Lineo 2001)</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
         <is>
           <t>13 Oct</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr">
+      <c r="G114" t="inlineStr">
         <is>
           <t>13 Oct: (a) Debian: RunCPM 6.9 (31-bit), runcpm for Linux users, vmspoold service cpm, CPM ... (LINUX on CMS: PUT/GET/RUN verified (ASM/LOAD/HELLO). (b) CMS natively: RUNCPM MODULE on LANG (abstraction_cms.h: drive X: = CMS disk X, binary files, pending empty files, line console), CP/M 2.2 programs on L:, CPM IMPORT/EXPORT text conversion; CPM L:ASM HELLO; L:LOAD HELLO; HELLO prints its line (cpmlang). Patch languages/cpm/runcpm-vm370plus.patch, mkcpm.sh.</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="2" t="n"/>
-      <c r="B114" s="10" t="n"/>
-      <c r="C114" s="2" t="n"/>
-      <c r="D114" s="2" t="n"/>
-      <c r="E114" s="5" t="n"/>
-      <c r="F114" s="2" t="n"/>
-      <c r="G114" s="2" t="n"/>
-    </row>
     <row r="115">
-      <c r="A115" s="14" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
+      <c r="A115" s="2" t="n"/>
       <c r="B115" s="10" t="n"/>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>64-bit</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>z/Architecture (64-bit)</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+      <c r="C115" s="2" t="n"/>
+      <c r="D115" s="2" t="n"/>
+      <c r="E115" s="5" t="n"/>
       <c r="F115" s="2" t="n"/>
       <c r="G115" s="2" t="n"/>
     </row>
@@ -4099,22 +4111,22 @@
           <t>M10</t>
         </is>
       </c>
-      <c r="B116" s="13" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="C116" s="14" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D116" s="14" t="inlineStr">
-        <is>
-          <t>Migration documentation 31 -&gt; 64 bit</t>
-        </is>
-      </c>
-      <c r="E116" s="5" t="n"/>
+      <c r="B116" s="10" t="n"/>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>64-bit</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>z/Architecture (64-bit)</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="n"/>
     </row>
@@ -4126,7 +4138,7 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
@@ -4136,7 +4148,7 @@
       </c>
       <c r="D117" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
+          <t>Migration documentation 31 -&gt; 64 bit</t>
         </is>
       </c>
       <c r="E117" s="5" t="n"/>
@@ -4151,17 +4163,17 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D118" s="14" t="inlineStr">
         <is>
-          <t>Kit after 64-bit (z/Architecture)</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E118" s="5" t="n"/>
@@ -4169,40 +4181,36 @@
       <c r="G118" s="2" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="14" t="n"/>
-      <c r="B119" s="13" t="n"/>
-      <c r="C119" s="14" t="n"/>
-      <c r="D119" s="14" t="n"/>
+      <c r="A119" s="14" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>Kit after 64-bit (z/Architecture)</t>
+        </is>
+      </c>
       <c r="E119" s="5" t="n"/>
       <c r="F119" s="2" t="n"/>
       <c r="G119" s="2" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="14" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="B120" s="13" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="C120" s="14" t="inlineStr">
-        <is>
-          <t>Multiprocessor-Support</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>MP (CP on several CPUs, virtual MP)</t>
-        </is>
-      </c>
-      <c r="E120" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+      <c r="A120" s="14" t="n"/>
+      <c r="B120" s="13" t="n"/>
+      <c r="C120" s="14" t="n"/>
+      <c r="D120" s="14" t="n"/>
+      <c r="E120" s="5" t="n"/>
       <c r="F120" s="2" t="n"/>
       <c r="G120" s="2" t="n"/>
     </row>
@@ -4214,17 +4222,17 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>More Languages</t>
+          <t>Multiprocessor-Support</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
+          <t>MP (CP on several CPUs, virtual MP)</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
@@ -4243,17 +4251,17 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>VoIP</t>
-        </is>
-      </c>
-      <c r="D122" s="14" t="inlineStr">
-        <is>
-          <t>FreeSWITCH</t>
+          <t>More Languages</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>GNU APL, full C++, Java on CMS, NetRexx 4</t>
         </is>
       </c>
       <c r="E122" s="16" t="inlineStr">
@@ -4272,17 +4280,17 @@
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>IoT</t>
+          <t>VoIP</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>Node-RED</t>
+          <t>FreeSWITCH</t>
         </is>
       </c>
       <c r="E123" s="16" t="inlineStr">
@@ -4301,17 +4309,17 @@
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>IoT</t>
         </is>
       </c>
       <c r="D124" s="14" t="inlineStr">
         <is>
-          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
+          <t>Node-RED</t>
         </is>
       </c>
       <c r="E124" s="16" t="inlineStr">
@@ -4330,17 +4338,17 @@
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="C125" s="14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D125" s="14" t="inlineStr">
         <is>
-          <t>CFSERV</t>
+          <t>Docker, QEMU/ReactOS,  Bochs/DOS</t>
         </is>
       </c>
       <c r="E125" s="16" t="inlineStr">
@@ -4359,20 +4367,24 @@
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C126" s="14" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="D126" s="14" t="inlineStr">
         <is>
-          <t>Manual Update</t>
-        </is>
-      </c>
-      <c r="E126" s="5" t="n"/>
+          <t>CFSERV</t>
+        </is>
+      </c>
+      <c r="E126" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="F126" s="2" t="n"/>
       <c r="G126" s="2" t="n"/>
     </row>
@@ -4384,17 +4396,17 @@
       </c>
       <c r="B127" s="13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="C127" s="14" t="inlineStr">
         <is>
-          <t>Snapshot</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D127" s="14" t="inlineStr">
         <is>
-          <t>Kit after M11</t>
+          <t>Manual Update</t>
         </is>
       </c>
       <c r="E127" s="5" t="n"/>
@@ -4402,41 +4414,34 @@
       <c r="G127" s="2" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="8" t="n"/>
-      <c r="B128" s="11" t="n"/>
-      <c r="C128" s="8" t="n"/>
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B128" s="13" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C128" s="14" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="D128" s="14" t="inlineStr">
+        <is>
+          <t>Kit after M11</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="n"/>
+      <c r="F128" s="2" t="n"/>
+      <c r="G128" s="2" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="8" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="B129" s="11" t="inlineStr">
-        <is>
-          <t>12a</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>DOS/VSE</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>Owner request 11 Oct; S/370-mode guest</t>
-        </is>
-      </c>
+      <c r="A129" s="8" t="n"/>
+      <c r="B129" s="11" t="n"/>
+      <c r="C129" s="8" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
@@ -4446,7 +4451,7 @@
       </c>
       <c r="B130" s="11" t="inlineStr">
         <is>
-          <t>12b</t>
+          <t>12a</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
@@ -4456,12 +4461,17 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
+          <t>DOS/VS Release 34 installed in a virtual machine (system packs, directory entry, IPL)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Owner request 11 Oct; S/370-mode guest</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4483,7 @@
       </c>
       <c r="B131" s="11" t="inlineStr">
         <is>
-          <t>12c</t>
+          <t>12b</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
@@ -4483,7 +4493,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
+          <t>DOS/VS under our CP as a regression of the S/370 guest paths (SIO/TIO, CCW translation, V=V)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -4500,7 +4510,7 @@
       </c>
       <c r="B132" s="11" t="inlineStr">
         <is>
-          <t>12d</t>
+          <t>12c</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
@@ -4510,7 +4520,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
+          <t>POWER spooling through VM reader/punch; jobs submitted from CMS</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -4527,7 +4537,7 @@
       </c>
       <c r="B133" s="11" t="inlineStr">
         <is>
-          <t>12e</t>
+          <t>12d</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
@@ -4537,39 +4547,34 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
+          <t>CMS/DOS simulation cross-checked against real DOS/VS</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
           <t>Planned</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B134" s="11" t="inlineStr">
         <is>
-          <t>13a</t>
+          <t>12e</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t>MVS guest</t>
+          <t>DOS/VSE</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+          <t>Research: inventory DOS/360 R26 and DOS/VS R34 tapes for source; feasibility of a 31/64-bit DOS</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -4579,7 +4584,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+          <t>srorso/dos360install</t>
         </is>
       </c>
     </row>
@@ -4591,25 +4596,57 @@
       </c>
       <c r="B135" s="11" t="inlineStr">
         <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>MVS guest</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>TK5 (MVS 3.8j) as a S/370 guest under VM/370plus: DASD, consoles, JES2 through the VM spool; a regression of the S/370 guest paths like M12</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Owner question 13 Oct; near-term, like DOS/VS (M12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="8" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B136" s="11" t="inlineStr">
+        <is>
           <t>13b</t>
         </is>
       </c>
-      <c r="C135" s="8" t="inlineStr">
+      <c r="C136" s="8" t="inlineStr">
         <is>
           <t>MVS 31-bit</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr">
+      <c r="D136" t="inlineStr">
         <is>
           <t>Research: feasibility of a 31-bit MVS from the public-domain MVS 3.8j source (the MVS/XA step: 31-bit addressing, channel subsystem I/O, storage management, SVCs, access methods) -- scope estimate before any work</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr">
+      <c r="E136" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr">
+      <c r="G136" t="inlineStr">
         <is>
           <t>Owner question 13 Oct; very late in the list (after M10-M12)</t>
         </is>

</xml_diff>

<commit_message>
I-301: same on pristine CE (cetest.sh), not a regression; DIAG 58 probe programs and drivers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -2881,13 +2881,13 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>In progress (Zork done)</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>17 Oct: Dungeon (Zork), public-domain C version (github.com/devshane/zork), cross-built for CMS (languages/zork/mkzork.sh, M5f cmscc), ZORK MODULE + DTEXTC DAT on the language disk; test zork-cms (zk1: play, SAVE, QUIT). Still to do: the VM/370 games tape, WIOS SNAKE/SLASH, TREK2.</t>
+          <t>Zork done (b28). M0058 SNAKE/SLASH: blank screen under DIAG 58 full screen, same on pristine CE (I-301), deferred. DISKPRY (M0080) on the language disk.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.36: MCproject runs in the Debian guest (mcp-install, vminetd on 8080, health from the PC); mcapps README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3520,7 +3520,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Owner decision 15 Oct: our own system instead of OpenProject (current OpenProject needs Ruby 4.0, Node 24, PostgreSQL 16+, 1 GB RAM, 64-bit: out of reach of the 31-bit Debian 7 guest). The repository is still empty (15 Oct); the VM/370plus port follows its design: language and database to be matched to what runs here (C/C++ GCC 13, Python 2.7/3.2, Regina, PostgreSQL 9.1 or SQLite 3.46 on both sides)</t>
+          <t>Owner decision 15 Oct: our own system instead of OpenProject. 17 Oct: runs unchanged in the Debian guest on MariaDB 10.11 (9.47), Regina 3.9.5 (linux390/regina39), wheezy perl/curl: mcp-install, operator created, served on port 8080 by vminetd (mcp.rexx --inetd); health from the PC in 17 s (mc1). Open: login takes ~10 min (SHA-512 crypt 400,000 rounds, wheezy libcrypt has no yescrypt) -- owner asked about a rounds setting.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.36/9.38: MCproject (8080) and MChelpdesk (8081) run in the Debian guest; vmcgid; init scripts; README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3530,7 +3530,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Owner decision 15 Oct: our own system instead of OpenProject. 17 Oct: runs unchanged in the Debian guest on MariaDB 10.11 (9.47), Regina 3.9.5 (linux390/regina39), wheezy perl/curl: mcp-install, operator created, served on port 8080 by vminetd (mcp.rexx --inetd); health from the PC in 17 s (mc1). Open: login takes ~10 min (SHA-512 crypt 400,000 rounds, wheezy libcrypt has no yescrypt) -- owner asked about a rounds setting.</t>
+          <t>17 Oct: runs unchanged in the Debian guest on MariaDB 10.11 (9.47), Regina 3.9.5 (linux390/regina39), wheezy perl/curl: mcp-install, operator, port 8080 by vminetd (mcp.rexx --inetd). pw_crypt_rounds added upstream (ab8973b; 55 tests OK): operator login from the PC in 74 s (mc1). Next: kit, CMS front end.</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Owner request 15 Oct. Follows the MChelpdesk design; shares platform choices with 9.36 (language/database matched to what runs on VM/370plus)</t>
+          <t>17 Oct: runs in the Debian guest (deploy/install.sh, MariaDB 10.11, Regina 3.9.5), port 8081 by vmcgid (CGI); pw_hash_iterations added upstream (d3ab569; 150 tests OK): login from the PC in 60 s (mc1). Next: kit, TICKET EXEC for CMS users, mail.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kit b31 verified on a fresh CE (kt46): apps at boot, MARIADB and TICKET from CMSUSER; 9.36 and 9.38 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -3520,7 +3520,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (kit b31)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (kit b31)</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>17 Oct: runs in the Debian guest (deploy/install.sh, MariaDB 10.11, Regina 3.9.5), port 8081 by vmcgid (CGI); pw_hash_iterations added upstream (d3ab569; 150 tests OK): login from the PC in 60 s (mc1); kit b30 (kt45). TICKET EXEC (19E) -&gt; vmspool ticket -&gt; mailin, tenant vm370plus: CMSUSER created VM3-000001 (tk1). Next: tenant in the kit, worker/cron, mail notifications.</t>
+          <t>17 Oct: runs in the Debian guest (deploy/install.sh, MariaDB 10.11, Regina 3.9.5), port 8081 by vmcgid (CGI); pw_hash_iterations added upstream (d3ab569; 150 tests OK). TICKET EXEC (19E) -&gt; vmspool ticket -&gt; mailin, tenant vm370plus; follow-ups by [VM3-nnnnnn] (tk1, tk2); workers by cron. Kit b31 verified on a fresh CE (kt46: VM3-000003 from CMSUSER).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
4c: CPWATCH runs again -- I-302 CP fix (DIAG 38 finds the symbol table through ESA/390 STEs and the new PAGSWP offset; DIAG 4 31-bit), CPWATCH rebuilt with 31-bit fixes; nucleus rewritten
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBNU8KnKzXkgscse8vw6so
</commit_message>
<xml_diff>
--- a/docs/VM370PLUS-Milestones.xlsx
+++ b/docs/VM370PLUS-Milestones.xlsx
@@ -1163,13 +1163,13 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>After CP leftovers</t>
+          <t>17 Oct: CPWATCH 3.3 runs again (I-251): rebuilt against VM/370plus's macros (cpwatch/r6), two 31-bit fixes in CPWATCH, and the CP fix I-302 (DIAG 38 symbol table, DIAG 4 31-bit). Idle CPU, menu and SYSTEM STATUS via DIAL CPWATCH (cw12, cw13).</t>
         </is>
       </c>
     </row>

</xml_diff>